<commit_message>
modified:   excel_data/Innovation_Fund_Projects_data - 130426.xlsx 	modified:   public/data/meta.json 	modified:   public/data/projects.json
</commit_message>
<xml_diff>
--- a/excel_data/Innovation_Fund_Projects_data - 130426.xlsx
+++ b/excel_data/Innovation_Fund_Projects_data - 130426.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zeplatform-my.sharepoint.com/personal/salman_muhammad_zeplatform_eu/Documents/Technical/IF mapping tool/if-map/excel_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1729" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{556170CE-5DED-44BF-8C31-DBD2A5203152}"/>
+  <xr:revisionPtr revIDLastSave="1739" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFEA8AE1-D4F1-4A6E-B791-DE0730027B57}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
     <sheet name="IF Projects" sheetId="2" r:id="rId2"/>
-    <sheet name="Legend" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId3"/>
+    <sheet name="Legend" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'IF Projects'!$A$1:$AE$61</definedName>
@@ -693,7 +694,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1303" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1321" uniqueCount="595">
   <si>
     <t>EU Innovation Fund — CCS/CCU Project Portfolio Summary</t>
   </si>
@@ -2744,12 +2745,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2793,6 +2788,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF4CCCC"/>
         <bgColor rgb="FFF4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -2985,10 +2986,7 @@
     <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="16" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3022,13 +3020,13 @@
     <xf numFmtId="166" fontId="3" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3040,25 +3038,25 @@
     <xf numFmtId="167" fontId="3" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="22" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3073,14 +3071,41 @@
     <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3090,7 +3115,6 @@
     <xf numFmtId="0" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3103,29 +3127,6 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3445,40 +3446,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="90" t="s">
+      <c r="A1" s="77" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
-      <c r="F1" s="75"/>
-      <c r="G1" s="75"/>
-      <c r="H1" s="75"/>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="92" t="s">
+      <c r="A2" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="75"/>
-      <c r="C2" s="75"/>
-      <c r="D2" s="75"/>
-      <c r="E2" s="75"/>
-      <c r="F2" s="75"/>
-      <c r="G2" s="75"/>
-      <c r="H2" s="75"/>
+      <c r="B2" s="73"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
     </row>
     <row r="4" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="79" t="s">
+      <c r="A4" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="75"/>
-      <c r="F4" s="75"/>
-      <c r="G4" s="75"/>
-      <c r="H4" s="75"/>
+      <c r="B4" s="73"/>
+      <c r="C4" s="73"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="73"/>
+      <c r="H4" s="73"/>
     </row>
     <row r="5" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3495,12 +3496,12 @@
       <c r="B6" s="3">
         <v>62</v>
       </c>
-      <c r="C6" s="75"/>
-      <c r="D6" s="75"/>
-      <c r="E6" s="75"/>
-      <c r="F6" s="75"/>
-      <c r="G6" s="75"/>
-      <c r="H6" s="75"/>
+      <c r="C6" s="73"/>
+      <c r="D6" s="73"/>
+      <c r="E6" s="73"/>
+      <c r="F6" s="73"/>
+      <c r="G6" s="73"/>
+      <c r="H6" s="73"/>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
@@ -3509,12 +3510,12 @@
       <c r="B7" s="5">
         <v>16</v>
       </c>
-      <c r="C7" s="75"/>
-      <c r="D7" s="75"/>
-      <c r="E7" s="75"/>
-      <c r="F7" s="75"/>
-      <c r="G7" s="75"/>
-      <c r="H7" s="75"/>
+      <c r="C7" s="73"/>
+      <c r="D7" s="73"/>
+      <c r="E7" s="73"/>
+      <c r="F7" s="73"/>
+      <c r="G7" s="73"/>
+      <c r="H7" s="73"/>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -3523,12 +3524,12 @@
       <c r="B8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="75"/>
-      <c r="D8" s="75"/>
-      <c r="E8" s="75"/>
-      <c r="F8" s="75"/>
-      <c r="G8" s="75"/>
-      <c r="H8" s="75"/>
+      <c r="C8" s="73"/>
+      <c r="D8" s="73"/>
+      <c r="E8" s="73"/>
+      <c r="F8" s="73"/>
+      <c r="G8" s="73"/>
+      <c r="H8" s="73"/>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
@@ -3537,12 +3538,12 @@
       <c r="B9" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="75"/>
-      <c r="D9" s="75"/>
-      <c r="E9" s="75"/>
-      <c r="F9" s="75"/>
-      <c r="G9" s="75"/>
-      <c r="H9" s="75"/>
+      <c r="C9" s="73"/>
+      <c r="D9" s="73"/>
+      <c r="E9" s="73"/>
+      <c r="F9" s="73"/>
+      <c r="G9" s="73"/>
+      <c r="H9" s="73"/>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -3551,12 +3552,12 @@
       <c r="B10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="75"/>
-      <c r="D10" s="75"/>
-      <c r="E10" s="75"/>
-      <c r="F10" s="75"/>
-      <c r="G10" s="75"/>
-      <c r="H10" s="75"/>
+      <c r="C10" s="73"/>
+      <c r="D10" s="73"/>
+      <c r="E10" s="73"/>
+      <c r="F10" s="73"/>
+      <c r="G10" s="73"/>
+      <c r="H10" s="73"/>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
@@ -3565,12 +3566,12 @@
       <c r="B11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="75"/>
-      <c r="D11" s="75"/>
-      <c r="E11" s="75"/>
-      <c r="F11" s="75"/>
-      <c r="G11" s="75"/>
-      <c r="H11" s="75"/>
+      <c r="C11" s="73"/>
+      <c r="D11" s="73"/>
+      <c r="E11" s="73"/>
+      <c r="F11" s="73"/>
+      <c r="G11" s="73"/>
+      <c r="H11" s="73"/>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
@@ -3579,24 +3580,24 @@
       <c r="B12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="75"/>
-      <c r="D12" s="75"/>
-      <c r="E12" s="75"/>
-      <c r="F12" s="75"/>
-      <c r="G12" s="75"/>
-      <c r="H12" s="75"/>
+      <c r="C12" s="73"/>
+      <c r="D12" s="73"/>
+      <c r="E12" s="73"/>
+      <c r="F12" s="73"/>
+      <c r="G12" s="73"/>
+      <c r="H12" s="73"/>
     </row>
     <row r="15" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="79" t="s">
+      <c r="A15" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="75"/>
-      <c r="C15" s="75"/>
-      <c r="D15" s="75"/>
-      <c r="E15" s="75"/>
-      <c r="F15" s="75"/>
-      <c r="G15" s="75"/>
-      <c r="H15" s="75"/>
+      <c r="B15" s="73"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="73"/>
+      <c r="E15" s="73"/>
+      <c r="F15" s="73"/>
+      <c r="G15" s="73"/>
+      <c r="H15" s="73"/>
     </row>
     <row r="16" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -3605,14 +3606,14 @@
       <c r="B16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="91" t="s">
+      <c r="C16" s="79" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="88"/>
-      <c r="E16" s="88"/>
-      <c r="F16" s="88"/>
-      <c r="G16" s="88"/>
-      <c r="H16" s="73"/>
+      <c r="D16" s="75"/>
+      <c r="E16" s="75"/>
+      <c r="F16" s="75"/>
+      <c r="G16" s="75"/>
+      <c r="H16" s="76"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
@@ -3621,14 +3622,14 @@
       <c r="B17" s="9">
         <v>21</v>
       </c>
-      <c r="C17" s="87" t="s">
+      <c r="C17" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="88"/>
-      <c r="E17" s="88"/>
-      <c r="F17" s="88"/>
-      <c r="G17" s="88"/>
-      <c r="H17" s="73"/>
+      <c r="D17" s="75"/>
+      <c r="E17" s="75"/>
+      <c r="F17" s="75"/>
+      <c r="G17" s="75"/>
+      <c r="H17" s="76"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
@@ -3637,14 +3638,14 @@
       <c r="B18" s="11">
         <v>20</v>
       </c>
-      <c r="C18" s="89" t="s">
+      <c r="C18" s="78" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="88"/>
-      <c r="E18" s="88"/>
-      <c r="F18" s="88"/>
-      <c r="G18" s="88"/>
-      <c r="H18" s="73"/>
+      <c r="D18" s="75"/>
+      <c r="E18" s="75"/>
+      <c r="F18" s="75"/>
+      <c r="G18" s="75"/>
+      <c r="H18" s="76"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -3653,14 +3654,14 @@
       <c r="B19" s="13">
         <v>10</v>
       </c>
-      <c r="C19" s="87" t="s">
+      <c r="C19" s="74" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="88"/>
-      <c r="E19" s="88"/>
-      <c r="F19" s="88"/>
-      <c r="G19" s="88"/>
-      <c r="H19" s="73"/>
+      <c r="D19" s="75"/>
+      <c r="E19" s="75"/>
+      <c r="F19" s="75"/>
+      <c r="G19" s="75"/>
+      <c r="H19" s="76"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
@@ -3669,14 +3670,14 @@
       <c r="B20" s="15">
         <v>4</v>
       </c>
-      <c r="C20" s="89" t="s">
+      <c r="C20" s="78" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="88"/>
-      <c r="E20" s="88"/>
-      <c r="F20" s="88"/>
-      <c r="G20" s="88"/>
-      <c r="H20" s="73"/>
+      <c r="D20" s="75"/>
+      <c r="E20" s="75"/>
+      <c r="F20" s="75"/>
+      <c r="G20" s="75"/>
+      <c r="H20" s="76"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
@@ -3685,14 +3686,14 @@
       <c r="B21" s="17">
         <v>3</v>
       </c>
-      <c r="C21" s="87" t="s">
+      <c r="C21" s="74" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="88"/>
-      <c r="E21" s="88"/>
-      <c r="F21" s="88"/>
-      <c r="G21" s="88"/>
-      <c r="H21" s="73"/>
+      <c r="D21" s="75"/>
+      <c r="E21" s="75"/>
+      <c r="F21" s="75"/>
+      <c r="G21" s="75"/>
+      <c r="H21" s="76"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="16" t="s">
@@ -3701,14 +3702,14 @@
       <c r="B22" s="17">
         <v>1</v>
       </c>
-      <c r="C22" s="89" t="s">
+      <c r="C22" s="78" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="88"/>
-      <c r="E22" s="88"/>
-      <c r="F22" s="88"/>
-      <c r="G22" s="88"/>
-      <c r="H22" s="73"/>
+      <c r="D22" s="75"/>
+      <c r="E22" s="75"/>
+      <c r="F22" s="75"/>
+      <c r="G22" s="75"/>
+      <c r="H22" s="76"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="16" t="s">
@@ -3717,14 +3718,14 @@
       <c r="B23" s="17">
         <v>1</v>
       </c>
-      <c r="C23" s="87" t="s">
+      <c r="C23" s="74" t="s">
         <v>34</v>
       </c>
-      <c r="D23" s="88"/>
-      <c r="E23" s="88"/>
-      <c r="F23" s="88"/>
-      <c r="G23" s="88"/>
-      <c r="H23" s="73"/>
+      <c r="D23" s="75"/>
+      <c r="E23" s="75"/>
+      <c r="F23" s="75"/>
+      <c r="G23" s="75"/>
+      <c r="H23" s="76"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="s">
@@ -3733,14 +3734,14 @@
       <c r="B24" s="19">
         <v>1</v>
       </c>
-      <c r="C24" s="89" t="s">
+      <c r="C24" s="78" t="s">
         <v>36</v>
       </c>
-      <c r="D24" s="88"/>
-      <c r="E24" s="88"/>
-      <c r="F24" s="88"/>
-      <c r="G24" s="88"/>
-      <c r="H24" s="73"/>
+      <c r="D24" s="75"/>
+      <c r="E24" s="75"/>
+      <c r="F24" s="75"/>
+      <c r="G24" s="75"/>
+      <c r="H24" s="76"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="20" t="s">
@@ -3749,26 +3750,26 @@
       <c r="B25" s="21">
         <v>1</v>
       </c>
-      <c r="C25" s="87" t="s">
+      <c r="C25" s="74" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="88"/>
-      <c r="E25" s="88"/>
-      <c r="F25" s="88"/>
-      <c r="G25" s="88"/>
-      <c r="H25" s="73"/>
+      <c r="D25" s="75"/>
+      <c r="E25" s="75"/>
+      <c r="F25" s="75"/>
+      <c r="G25" s="75"/>
+      <c r="H25" s="76"/>
     </row>
     <row r="28" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="79" t="s">
+      <c r="A28" s="72" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="75"/>
-      <c r="C28" s="75"/>
-      <c r="D28" s="75"/>
-      <c r="E28" s="75"/>
-      <c r="F28" s="75"/>
-      <c r="G28" s="75"/>
-      <c r="H28" s="75"/>
+      <c r="B28" s="73"/>
+      <c r="C28" s="73"/>
+      <c r="D28" s="73"/>
+      <c r="E28" s="73"/>
+      <c r="F28" s="73"/>
+      <c r="G28" s="73"/>
+      <c r="H28" s="73"/>
     </row>
     <row r="29" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -3912,6 +3913,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="C19:H19"/>
     <mergeCell ref="A1:H1"/>
@@ -3928,12 +3935,6 @@
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="C6:H6"/>
     <mergeCell ref="C24:H24"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C23:H23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3971,7 +3972,7 @@
     <col min="32" max="16384" width="30" style="29"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" s="46" customFormat="1" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" s="45" customFormat="1" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="28" t="s">
         <v>60</v>
       </c>
@@ -3993,7 +3994,7 @@
       <c r="G1" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="H1" s="45" t="s">
+      <c r="H1" s="44" t="s">
         <v>66</v>
       </c>
       <c r="I1" s="28" t="s">
@@ -4070,7 +4071,7 @@
       <c r="A2" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="55" t="s">
         <v>137</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -4148,7 +4149,7 @@
       <c r="AA2" s="30" t="s">
         <v>140</v>
       </c>
-      <c r="AB2" s="47" t="s">
+      <c r="AB2" s="46" t="s">
         <v>352</v>
       </c>
       <c r="AC2" s="30" t="s">
@@ -4157,7 +4158,7 @@
       <c r="AD2" s="30" t="s">
         <v>340</v>
       </c>
-      <c r="AE2" s="61" t="s">
+      <c r="AE2" s="60" t="s">
         <v>570</v>
       </c>
     </row>
@@ -4165,7 +4166,7 @@
       <c r="A3" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="B3" s="56" t="s">
+      <c r="B3" s="55" t="s">
         <v>394</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -4243,7 +4244,7 @@
       <c r="AA3" s="30" t="s">
         <v>92</v>
       </c>
-      <c r="AB3" s="47" t="s">
+      <c r="AB3" s="46" t="s">
         <v>250</v>
       </c>
       <c r="AC3" s="30" t="s">
@@ -4252,7 +4253,7 @@
       <c r="AD3" s="30" t="s">
         <v>397</v>
       </c>
-      <c r="AE3" s="62" t="s">
+      <c r="AE3" s="61" t="s">
         <v>571</v>
       </c>
     </row>
@@ -4260,7 +4261,7 @@
       <c r="A4" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="54" t="s">
         <v>290</v>
       </c>
       <c r="C4" s="4" t="s">
@@ -4338,7 +4339,7 @@
       <c r="AA4" s="34" t="s">
         <v>292</v>
       </c>
-      <c r="AB4" s="47" t="s">
+      <c r="AB4" s="46" t="s">
         <v>351</v>
       </c>
       <c r="AC4" s="34" t="s">
@@ -4347,7 +4348,7 @@
       <c r="AD4" s="34" t="s">
         <v>344</v>
       </c>
-      <c r="AE4" s="63" t="s">
+      <c r="AE4" s="62" t="s">
         <v>27</v>
       </c>
     </row>
@@ -4355,7 +4356,7 @@
       <c r="A5" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="B5" s="56" t="s">
+      <c r="B5" s="55" t="s">
         <v>354</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -4433,7 +4434,7 @@
       <c r="AA5" s="30" t="s">
         <v>178</v>
       </c>
-      <c r="AB5" s="47" t="s">
+      <c r="AB5" s="46" t="s">
         <v>356</v>
       </c>
       <c r="AC5" s="30" t="s">
@@ -4442,7 +4443,7 @@
       <c r="AD5" s="30" t="s">
         <v>358</v>
       </c>
-      <c r="AE5" s="64" t="s">
+      <c r="AE5" s="63" t="s">
         <v>572</v>
       </c>
     </row>
@@ -4450,7 +4451,7 @@
       <c r="A6" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="B6" s="56" t="s">
+      <c r="B6" s="55" t="s">
         <v>281</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -4528,7 +4529,7 @@
       <c r="AA6" s="30" t="s">
         <v>283</v>
       </c>
-      <c r="AB6" s="47" t="s">
+      <c r="AB6" s="46" t="s">
         <v>362</v>
       </c>
       <c r="AC6" s="30" t="s">
@@ -4537,7 +4538,7 @@
       <c r="AD6" s="30" t="s">
         <v>578</v>
       </c>
-      <c r="AE6" s="65" t="s">
+      <c r="AE6" s="64" t="s">
         <v>573</v>
       </c>
     </row>
@@ -4545,7 +4546,7 @@
       <c r="A7" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B7" s="56" t="s">
+      <c r="B7" s="55" t="s">
         <v>130</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -4623,7 +4624,7 @@
       <c r="AA7" s="30" t="s">
         <v>133</v>
       </c>
-      <c r="AB7" s="47" t="s">
+      <c r="AB7" s="46" t="s">
         <v>364</v>
       </c>
       <c r="AC7" s="30" t="s">
@@ -4632,7 +4633,7 @@
       <c r="AD7" s="30" t="s">
         <v>365</v>
       </c>
-      <c r="AE7" s="64" t="s">
+      <c r="AE7" s="63" t="s">
         <v>572</v>
       </c>
     </row>
@@ -4640,7 +4641,7 @@
       <c r="A8" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="B8" s="56" t="s">
+      <c r="B8" s="55" t="s">
         <v>120</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -4718,7 +4719,7 @@
       <c r="AA8" s="30" t="s">
         <v>124</v>
       </c>
-      <c r="AB8" s="47" t="s">
+      <c r="AB8" s="46" t="s">
         <v>367</v>
       </c>
       <c r="AC8" s="30" t="s">
@@ -4727,7 +4728,7 @@
       <c r="AD8" s="30" t="s">
         <v>368</v>
       </c>
-      <c r="AE8" s="64" t="s">
+      <c r="AE8" s="63" t="s">
         <v>572</v>
       </c>
     </row>
@@ -4735,7 +4736,7 @@
       <c r="A9" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="B9" s="55" t="s">
+      <c r="B9" s="54" t="s">
         <v>224</v>
       </c>
       <c r="C9" s="4" t="s">
@@ -4765,13 +4766,13 @@
       <c r="K9" s="41" t="s">
         <v>92</v>
       </c>
-      <c r="L9" s="50">
+      <c r="L9" s="49">
         <v>25.819174</v>
       </c>
       <c r="M9" s="41" t="s">
         <v>92</v>
       </c>
-      <c r="N9" s="50" t="s">
+      <c r="N9" s="49" t="s">
         <v>92</v>
       </c>
       <c r="O9" s="41" t="s">
@@ -4813,7 +4814,7 @@
       <c r="AA9" s="34" t="s">
         <v>226</v>
       </c>
-      <c r="AB9" s="47" t="s">
+      <c r="AB9" s="46" t="s">
         <v>370</v>
       </c>
       <c r="AC9" s="34" t="s">
@@ -4822,7 +4823,7 @@
       <c r="AD9" s="34" t="s">
         <v>227</v>
       </c>
-      <c r="AE9" s="62" t="s">
+      <c r="AE9" s="61" t="s">
         <v>571</v>
       </c>
     </row>
@@ -4830,7 +4831,7 @@
       <c r="A10" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B10" s="56" t="s">
+      <c r="B10" s="55" t="s">
         <v>372</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -4908,7 +4909,7 @@
       <c r="AA10" s="30" t="s">
         <v>310</v>
       </c>
-      <c r="AB10" s="47" t="s">
+      <c r="AB10" s="46" t="s">
         <v>374</v>
       </c>
       <c r="AC10" s="30" t="s">
@@ -4917,7 +4918,7 @@
       <c r="AD10" s="30" t="s">
         <v>399</v>
       </c>
-      <c r="AE10" s="63" t="s">
+      <c r="AE10" s="62" t="s">
         <v>27</v>
       </c>
     </row>
@@ -4925,7 +4926,7 @@
       <c r="A11" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="B11" s="56" t="s">
+      <c r="B11" s="55" t="s">
         <v>269</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -4946,10 +4947,10 @@
       <c r="H11" s="31" t="s">
         <v>92</v>
       </c>
-      <c r="I11" s="53">
+      <c r="I11" s="52">
         <v>7.6649999999999999E-3</v>
       </c>
-      <c r="J11" s="53" t="s">
+      <c r="J11" s="52" t="s">
         <v>92</v>
       </c>
       <c r="K11" s="40" t="s">
@@ -5003,7 +5004,7 @@
       <c r="AA11" s="30" t="s">
         <v>270</v>
       </c>
-      <c r="AB11" s="47" t="s">
+      <c r="AB11" s="46" t="s">
         <v>420</v>
       </c>
       <c r="AC11" s="30" t="s">
@@ -5012,7 +5013,7 @@
       <c r="AD11" s="30" t="s">
         <v>426</v>
       </c>
-      <c r="AE11" s="64" t="s">
+      <c r="AE11" s="63" t="s">
         <v>572</v>
       </c>
     </row>
@@ -5020,7 +5021,7 @@
       <c r="A12" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B12" s="55" t="s">
+      <c r="B12" s="54" t="s">
         <v>192</v>
       </c>
       <c r="C12" s="4" t="s">
@@ -5098,7 +5099,7 @@
       <c r="AA12" s="34" t="s">
         <v>195</v>
       </c>
-      <c r="AB12" s="47" t="s">
+      <c r="AB12" s="46" t="s">
         <v>429</v>
       </c>
       <c r="AC12" s="34" t="s">
@@ -5107,7 +5108,7 @@
       <c r="AD12" s="34" t="s">
         <v>428</v>
       </c>
-      <c r="AE12" s="65" t="s">
+      <c r="AE12" s="64" t="s">
         <v>573</v>
       </c>
     </row>
@@ -5115,7 +5116,7 @@
       <c r="A13" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B13" s="55" t="s">
+      <c r="B13" s="54" t="s">
         <v>165</v>
       </c>
       <c r="C13" s="4" t="s">
@@ -5202,7 +5203,7 @@
       <c r="AD13" s="34" t="s">
         <v>386</v>
       </c>
-      <c r="AE13" s="61" t="s">
+      <c r="AE13" s="60" t="s">
         <v>570</v>
       </c>
     </row>
@@ -5210,7 +5211,7 @@
       <c r="A14" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="B14" s="55" t="s">
+      <c r="B14" s="54" t="s">
         <v>246</v>
       </c>
       <c r="C14" s="4" t="s">
@@ -5288,7 +5289,7 @@
       <c r="AA14" s="34" t="s">
         <v>416</v>
       </c>
-      <c r="AB14" s="47" t="s">
+      <c r="AB14" s="46" t="s">
         <v>415</v>
       </c>
       <c r="AC14" s="34" t="s">
@@ -5297,7 +5298,7 @@
       <c r="AD14" s="34" t="s">
         <v>414</v>
       </c>
-      <c r="AE14" s="65" t="s">
+      <c r="AE14" s="64" t="s">
         <v>573</v>
       </c>
     </row>
@@ -5305,7 +5306,7 @@
       <c r="A15" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B15" s="55" t="s">
+      <c r="B15" s="54" t="s">
         <v>173</v>
       </c>
       <c r="C15" s="4" t="s">
@@ -5381,7 +5382,7 @@
         <v>590</v>
       </c>
       <c r="AA15" s="34"/>
-      <c r="AB15" s="47" t="s">
+      <c r="AB15" s="46" t="s">
         <v>419</v>
       </c>
       <c r="AC15" s="34" t="s">
@@ -5390,7 +5391,7 @@
       <c r="AD15" s="34" t="s">
         <v>417</v>
       </c>
-      <c r="AE15" s="65" t="s">
+      <c r="AE15" s="64" t="s">
         <v>573</v>
       </c>
     </row>
@@ -5398,7 +5399,7 @@
       <c r="A16" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="B16" s="56" t="s">
+      <c r="B16" s="55" t="s">
         <v>289</v>
       </c>
       <c r="C16" s="4" t="s">
@@ -5476,7 +5477,7 @@
       <c r="AA16" s="30" t="s">
         <v>289</v>
       </c>
-      <c r="AB16" s="47" t="s">
+      <c r="AB16" s="46" t="s">
         <v>430</v>
       </c>
       <c r="AC16" s="30" t="s">
@@ -5485,7 +5486,7 @@
       <c r="AD16" s="30" t="s">
         <v>433</v>
       </c>
-      <c r="AE16" s="66" t="s">
+      <c r="AE16" s="65" t="s">
         <v>574</v>
       </c>
     </row>
@@ -5493,7 +5494,7 @@
       <c r="A17" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="B17" s="56" t="s">
+      <c r="B17" s="55" t="s">
         <v>253</v>
       </c>
       <c r="C17" s="4" t="s">
@@ -5511,19 +5512,19 @@
       <c r="G17" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="H17" s="52">
+      <c r="H17" s="51">
         <v>4.5999999999999999E-3</v>
       </c>
-      <c r="I17" s="52">
+      <c r="I17" s="51">
         <v>4.5999999999999999E-3</v>
       </c>
-      <c r="J17" s="52">
+      <c r="J17" s="51">
         <v>4.5999999999999999E-3</v>
       </c>
       <c r="K17" s="40" t="s">
         <v>92</v>
       </c>
-      <c r="L17" s="53">
+      <c r="L17" s="52">
         <v>4.5689E-2</v>
       </c>
       <c r="M17" s="40">
@@ -5580,7 +5581,7 @@
       <c r="AD17" s="30" t="s">
         <v>437</v>
       </c>
-      <c r="AE17" s="63" t="s">
+      <c r="AE17" s="62" t="s">
         <v>27</v>
       </c>
     </row>
@@ -5588,7 +5589,7 @@
       <c r="A18" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B18" s="56" t="s">
+      <c r="B18" s="55" t="s">
         <v>204</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -5675,7 +5676,7 @@
       <c r="AD18" s="30" t="s">
         <v>391</v>
       </c>
-      <c r="AE18" s="66" t="s">
+      <c r="AE18" s="65" t="s">
         <v>574</v>
       </c>
     </row>
@@ -5683,7 +5684,7 @@
       <c r="A19" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="B19" s="55" t="s">
+      <c r="B19" s="54" t="s">
         <v>99</v>
       </c>
       <c r="C19" s="4" t="s">
@@ -5761,7 +5762,7 @@
       <c r="AA19" s="34" t="s">
         <v>105</v>
       </c>
-      <c r="AB19" s="47" t="s">
+      <c r="AB19" s="46" t="s">
         <v>439</v>
       </c>
       <c r="AC19" s="34" t="s">
@@ -5770,7 +5771,7 @@
       <c r="AD19" s="34" t="s">
         <v>106</v>
       </c>
-      <c r="AE19" s="63" t="s">
+      <c r="AE19" s="62" t="s">
         <v>27</v>
       </c>
     </row>
@@ -5778,7 +5779,7 @@
       <c r="A20" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B20" s="55" t="s">
+      <c r="B20" s="54" t="s">
         <v>237</v>
       </c>
       <c r="C20" s="4" t="s">
@@ -5865,7 +5866,7 @@
       <c r="AD20" s="34" t="s">
         <v>441</v>
       </c>
-      <c r="AE20" s="67" t="s">
+      <c r="AE20" s="66" t="s">
         <v>575</v>
       </c>
     </row>
@@ -5873,7 +5874,7 @@
       <c r="A21" s="22" t="s">
         <v>126</v>
       </c>
-      <c r="B21" s="55" t="s">
+      <c r="B21" s="54" t="s">
         <v>305</v>
       </c>
       <c r="C21" s="4" t="s">
@@ -5891,7 +5892,7 @@
       <c r="G21" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="H21" s="54">
+      <c r="H21" s="53">
         <v>0.63600000000000001</v>
       </c>
       <c r="I21" s="41" t="s">
@@ -5903,7 +5904,7 @@
       <c r="K21" s="41" t="s">
         <v>92</v>
       </c>
-      <c r="L21" s="49">
+      <c r="L21" s="48">
         <v>6.3620479999999997</v>
       </c>
       <c r="M21" s="41" t="s">
@@ -5951,7 +5952,7 @@
       <c r="AA21" s="34" t="s">
         <v>306</v>
       </c>
-      <c r="AB21" s="47" t="s">
+      <c r="AB21" s="46" t="s">
         <v>444</v>
       </c>
       <c r="AC21" s="34" t="s">
@@ -5960,7 +5961,7 @@
       <c r="AD21" s="34" t="s">
         <v>307</v>
       </c>
-      <c r="AE21" s="66" t="s">
+      <c r="AE21" s="65" t="s">
         <v>574</v>
       </c>
     </row>
@@ -5968,7 +5969,7 @@
       <c r="A22" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="B22" s="56" t="s">
+      <c r="B22" s="55" t="s">
         <v>241</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -5986,7 +5987,7 @@
       <c r="G22" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="H22" s="53">
+      <c r="H22" s="52">
         <v>1.7904E-2</v>
       </c>
       <c r="I22" s="40">
@@ -6046,7 +6047,7 @@
       <c r="AA22" s="30" t="s">
         <v>245</v>
       </c>
-      <c r="AB22" s="47" t="s">
+      <c r="AB22" s="46" t="s">
         <v>445</v>
       </c>
       <c r="AC22" s="30" t="s">
@@ -6055,7 +6056,7 @@
       <c r="AD22" s="30" t="s">
         <v>447</v>
       </c>
-      <c r="AE22" s="65" t="s">
+      <c r="AE22" s="64" t="s">
         <v>573</v>
       </c>
     </row>
@@ -6063,7 +6064,7 @@
       <c r="A23" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="B23" s="55" t="s">
+      <c r="B23" s="54" t="s">
         <v>231</v>
       </c>
       <c r="C23" s="4" t="s">
@@ -6141,7 +6142,7 @@
       <c r="AA23" s="34" t="s">
         <v>233</v>
       </c>
-      <c r="AB23" s="47" t="s">
+      <c r="AB23" s="46" t="s">
         <v>450</v>
       </c>
       <c r="AC23" s="34" t="s">
@@ -6150,7 +6151,7 @@
       <c r="AD23" s="34" t="s">
         <v>452</v>
       </c>
-      <c r="AE23" s="66" t="s">
+      <c r="AE23" s="65" t="s">
         <v>574</v>
       </c>
     </row>
@@ -6158,7 +6159,7 @@
       <c r="A24" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="B24" s="55" t="s">
+      <c r="B24" s="54" t="s">
         <v>179</v>
       </c>
       <c r="C24" s="4" t="s">
@@ -6170,10 +6171,10 @@
       <c r="E24" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F24" s="42" t="s">
+      <c r="F24" s="71" t="s">
         <v>460</v>
       </c>
-      <c r="G24" s="42" t="s">
+      <c r="G24" s="71" t="s">
         <v>461</v>
       </c>
       <c r="H24" s="35">
@@ -6236,7 +6237,7 @@
       <c r="AA24" s="34" t="s">
         <v>181</v>
       </c>
-      <c r="AB24" s="47" t="s">
+      <c r="AB24" s="46" t="s">
         <v>465</v>
       </c>
       <c r="AC24" s="34" t="s">
@@ -6245,7 +6246,7 @@
       <c r="AD24" s="34" t="s">
         <v>463</v>
       </c>
-      <c r="AE24" s="62" t="s">
+      <c r="AE24" s="61" t="s">
         <v>571</v>
       </c>
     </row>
@@ -6253,7 +6254,7 @@
       <c r="A25" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="B25" s="55" t="s">
+      <c r="B25" s="54" t="s">
         <v>251</v>
       </c>
       <c r="C25" s="4" t="s">
@@ -6331,7 +6332,7 @@
       <c r="AA25" s="34" t="s">
         <v>252</v>
       </c>
-      <c r="AB25" s="47" t="s">
+      <c r="AB25" s="46" t="s">
         <v>456</v>
       </c>
       <c r="AC25" s="34" t="s">
@@ -6340,7 +6341,7 @@
       <c r="AD25" s="34" t="s">
         <v>458</v>
       </c>
-      <c r="AE25" s="66" t="s">
+      <c r="AE25" s="65" t="s">
         <v>574</v>
       </c>
     </row>
@@ -6348,7 +6349,7 @@
       <c r="A26" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B26" s="55" t="s">
+      <c r="B26" s="54" t="s">
         <v>259</v>
       </c>
       <c r="C26" s="34" t="s">
@@ -6366,7 +6367,7 @@
       <c r="G26" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="H26" s="54">
+      <c r="H26" s="53">
         <v>2.2800000000000001E-2</v>
       </c>
       <c r="I26" s="41" t="s">
@@ -6435,7 +6436,7 @@
       <c r="AD26" s="34" t="s">
         <v>264</v>
       </c>
-      <c r="AE26" s="62" t="s">
+      <c r="AE26" s="61" t="s">
         <v>571</v>
       </c>
     </row>
@@ -6443,7 +6444,7 @@
       <c r="A27" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B27" s="56" t="s">
+      <c r="B27" s="55" t="s">
         <v>169</v>
       </c>
       <c r="C27" s="2" t="s">
@@ -6530,7 +6531,7 @@
       <c r="AD27" s="30" t="s">
         <v>468</v>
       </c>
-      <c r="AE27" s="62" t="s">
+      <c r="AE27" s="61" t="s">
         <v>571</v>
       </c>
     </row>
@@ -6538,7 +6539,7 @@
       <c r="A28" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="B28" s="56" t="s">
+      <c r="B28" s="55" t="s">
         <v>146</v>
       </c>
       <c r="C28" s="2" t="s">
@@ -6616,7 +6617,7 @@
       <c r="AA28" s="30" t="s">
         <v>148</v>
       </c>
-      <c r="AB28" s="47" t="s">
+      <c r="AB28" s="46" t="s">
         <v>471</v>
       </c>
       <c r="AC28" s="30" t="s">
@@ -6625,7 +6626,7 @@
       <c r="AD28" s="30" t="s">
         <v>473</v>
       </c>
-      <c r="AE28" s="61" t="s">
+      <c r="AE28" s="60" t="s">
         <v>570</v>
       </c>
     </row>
@@ -6633,7 +6634,7 @@
       <c r="A29" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B29" s="56" t="s">
+      <c r="B29" s="55" t="s">
         <v>196</v>
       </c>
       <c r="C29" s="2" t="s">
@@ -6720,7 +6721,7 @@
       <c r="AD29" s="30" t="s">
         <v>476</v>
       </c>
-      <c r="AE29" s="61" t="s">
+      <c r="AE29" s="60" t="s">
         <v>570</v>
       </c>
     </row>
@@ -6728,7 +6729,7 @@
       <c r="A30" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="B30" s="55" t="s">
+      <c r="B30" s="54" t="s">
         <v>501</v>
       </c>
       <c r="C30" s="4" t="s">
@@ -6746,7 +6747,7 @@
       <c r="G30" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="H30" s="54">
+      <c r="H30" s="53">
         <v>4.5999999999999999E-2</v>
       </c>
       <c r="I30" s="41">
@@ -6806,7 +6807,7 @@
       <c r="AA30" s="34" t="s">
         <v>316</v>
       </c>
-      <c r="AB30" s="48" t="s">
+      <c r="AB30" s="47" t="s">
         <v>502</v>
       </c>
       <c r="AC30" s="34" t="s">
@@ -6815,7 +6816,7 @@
       <c r="AD30" s="34" t="s">
         <v>504</v>
       </c>
-      <c r="AE30" s="62" t="s">
+      <c r="AE30" s="61" t="s">
         <v>571</v>
       </c>
     </row>
@@ -6823,7 +6824,7 @@
       <c r="A31" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B31" s="55" t="s">
+      <c r="B31" s="54" t="s">
         <v>200</v>
       </c>
       <c r="C31" s="4" t="s">
@@ -6901,7 +6902,7 @@
       <c r="AA31" s="34" t="s">
         <v>202</v>
       </c>
-      <c r="AB31" s="71" t="s">
+      <c r="AB31" s="70" t="s">
         <v>203</v>
       </c>
       <c r="AC31" s="34" t="s">
@@ -6910,7 +6911,7 @@
       <c r="AD31" s="34" t="s">
         <v>412</v>
       </c>
-      <c r="AE31" s="61" t="s">
+      <c r="AE31" s="60" t="s">
         <v>570</v>
       </c>
     </row>
@@ -6918,7 +6919,7 @@
       <c r="A32" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B32" s="55" t="s">
+      <c r="B32" s="54" t="s">
         <v>277</v>
       </c>
       <c r="C32" s="4" t="s">
@@ -6996,7 +6997,7 @@
       <c r="AA32" s="34" t="s">
         <v>279</v>
       </c>
-      <c r="AB32" s="47" t="s">
+      <c r="AB32" s="46" t="s">
         <v>478</v>
       </c>
       <c r="AC32" s="34" t="s">
@@ -7005,7 +7006,7 @@
       <c r="AD32" s="34" t="s">
         <v>280</v>
       </c>
-      <c r="AE32" s="61" t="s">
+      <c r="AE32" s="60" t="s">
         <v>570</v>
       </c>
     </row>
@@ -7013,7 +7014,7 @@
       <c r="A33" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B33" s="56" t="s">
+      <c r="B33" s="55" t="s">
         <v>107</v>
       </c>
       <c r="C33" s="2" t="s">
@@ -7091,7 +7092,7 @@
       <c r="AA33" s="30" t="s">
         <v>113</v>
       </c>
-      <c r="AB33" s="47" t="s">
+      <c r="AB33" s="46" t="s">
         <v>481</v>
       </c>
       <c r="AC33" s="30" t="s">
@@ -7100,7 +7101,7 @@
       <c r="AD33" s="30" t="s">
         <v>480</v>
       </c>
-      <c r="AE33" s="67" t="s">
+      <c r="AE33" s="66" t="s">
         <v>575</v>
       </c>
     </row>
@@ -7108,7 +7109,7 @@
       <c r="A34" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B34" s="56" t="s">
+      <c r="B34" s="55" t="s">
         <v>293</v>
       </c>
       <c r="C34" s="2" t="s">
@@ -7184,7 +7185,7 @@
       <c r="AA34" s="30" t="s">
         <v>295</v>
       </c>
-      <c r="AB34" s="47" t="s">
+      <c r="AB34" s="46" t="s">
         <v>296</v>
       </c>
       <c r="AC34" s="30" t="s">
@@ -7193,7 +7194,7 @@
       <c r="AD34" s="30" t="s">
         <v>484</v>
       </c>
-      <c r="AE34" s="65" t="s">
+      <c r="AE34" s="64" t="s">
         <v>573</v>
       </c>
     </row>
@@ -7201,7 +7202,7 @@
       <c r="A35" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B35" s="55" t="s">
+      <c r="B35" s="54" t="s">
         <v>142</v>
       </c>
       <c r="C35" s="4" t="s">
@@ -7231,7 +7232,7 @@
       <c r="K35" s="41" t="s">
         <v>92</v>
       </c>
-      <c r="L35" s="49">
+      <c r="L35" s="48">
         <v>2.8</v>
       </c>
       <c r="M35" s="41">
@@ -7279,7 +7280,7 @@
       <c r="AA35" s="34" t="s">
         <v>145</v>
       </c>
-      <c r="AB35" s="47" t="s">
+      <c r="AB35" s="46" t="s">
         <v>485</v>
       </c>
       <c r="AC35" s="34" t="s">
@@ -7288,7 +7289,7 @@
       <c r="AD35" s="34" t="s">
         <v>377</v>
       </c>
-      <c r="AE35" s="63" t="s">
+      <c r="AE35" s="62" t="s">
         <v>27</v>
       </c>
     </row>
@@ -7296,7 +7297,7 @@
       <c r="A36" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B36" s="55" t="s">
+      <c r="B36" s="54" t="s">
         <v>114</v>
       </c>
       <c r="C36" s="2" t="s">
@@ -7335,7 +7336,7 @@
       <c r="N36" s="41" t="s">
         <v>92</v>
       </c>
-      <c r="O36" s="70" t="s">
+      <c r="O36" s="69" t="s">
         <v>92</v>
       </c>
       <c r="P36" s="36">
@@ -7374,7 +7375,7 @@
       <c r="AA36" s="34" t="s">
         <v>118</v>
       </c>
-      <c r="AB36" s="47" t="s">
+      <c r="AB36" s="46" t="s">
         <v>492</v>
       </c>
       <c r="AC36" s="34" t="s">
@@ -7383,7 +7384,7 @@
       <c r="AD36" s="34" t="s">
         <v>488</v>
       </c>
-      <c r="AE36" s="61" t="s">
+      <c r="AE36" s="60" t="s">
         <v>570</v>
       </c>
     </row>
@@ -7391,7 +7392,7 @@
       <c r="A37" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="B37" s="55" t="s">
+      <c r="B37" s="54" t="s">
         <v>284</v>
       </c>
       <c r="C37" s="4" t="s">
@@ -7409,7 +7410,7 @@
       <c r="G37" s="4" t="s">
         <v>286</v>
       </c>
-      <c r="H37" s="54">
+      <c r="H37" s="53">
         <v>5.0046999999999999E-3</v>
       </c>
       <c r="I37" s="41" t="s">
@@ -7421,16 +7422,16 @@
       <c r="K37" s="41" t="s">
         <v>92</v>
       </c>
-      <c r="L37" s="49">
+      <c r="L37" s="48">
         <v>5.0047000000000001E-2</v>
       </c>
       <c r="M37" s="41" t="s">
         <v>92</v>
       </c>
-      <c r="N37" s="54">
+      <c r="N37" s="53">
         <v>5.1711E-2</v>
       </c>
-      <c r="O37" s="69" t="s">
+      <c r="O37" s="68" t="s">
         <v>92</v>
       </c>
       <c r="P37" s="36">
@@ -7469,7 +7470,7 @@
       <c r="AA37" s="34" t="s">
         <v>288</v>
       </c>
-      <c r="AB37" s="47" t="s">
+      <c r="AB37" s="46" t="s">
         <v>491</v>
       </c>
       <c r="AC37" s="34" t="s">
@@ -7478,7 +7479,7 @@
       <c r="AD37" s="34" t="s">
         <v>490</v>
       </c>
-      <c r="AE37" s="61" t="s">
+      <c r="AE37" s="60" t="s">
         <v>570</v>
       </c>
     </row>
@@ -7486,7 +7487,7 @@
       <c r="A38" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B38" s="55" t="s">
+      <c r="B38" s="54" t="s">
         <v>336</v>
       </c>
       <c r="C38" s="2" t="s">
@@ -7564,7 +7565,7 @@
       <c r="AA38" s="34" t="s">
         <v>217</v>
       </c>
-      <c r="AB38" s="47" t="s">
+      <c r="AB38" s="46" t="s">
         <v>410</v>
       </c>
       <c r="AC38" s="34" t="s">
@@ -7573,7 +7574,7 @@
       <c r="AD38" s="34" t="s">
         <v>408</v>
       </c>
-      <c r="AE38" s="62" t="s">
+      <c r="AE38" s="61" t="s">
         <v>571</v>
       </c>
     </row>
@@ -7581,7 +7582,7 @@
       <c r="A39" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="B39" s="56" t="s">
+      <c r="B39" s="55" t="s">
         <v>312</v>
       </c>
       <c r="C39" s="2" t="s">
@@ -7657,7 +7658,7 @@
       <c r="AA39" s="30" t="s">
         <v>314</v>
       </c>
-      <c r="AB39" s="47" t="s">
+      <c r="AB39" s="46" t="s">
         <v>493</v>
       </c>
       <c r="AC39" s="30" t="s">
@@ -7666,7 +7667,7 @@
       <c r="AD39" s="30" t="s">
         <v>402</v>
       </c>
-      <c r="AE39" s="62" t="s">
+      <c r="AE39" s="61" t="s">
         <v>571</v>
       </c>
     </row>
@@ -7674,7 +7675,7 @@
       <c r="A40" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B40" s="56" t="s">
+      <c r="B40" s="55" t="s">
         <v>218</v>
       </c>
       <c r="C40" s="2" t="s">
@@ -7752,7 +7753,7 @@
       <c r="AA40" s="30" t="s">
         <v>222</v>
       </c>
-      <c r="AB40" s="47" t="s">
+      <c r="AB40" s="46" t="s">
         <v>223</v>
       </c>
       <c r="AC40" s="30" t="s">
@@ -7761,7 +7762,7 @@
       <c r="AD40" s="30" t="s">
         <v>495</v>
       </c>
-      <c r="AE40" s="65" t="s">
+      <c r="AE40" s="64" t="s">
         <v>573</v>
       </c>
     </row>
@@ -7769,7 +7770,7 @@
       <c r="A41" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B41" s="56" t="s">
+      <c r="B41" s="55" t="s">
         <v>88</v>
       </c>
       <c r="C41" s="2" t="s">
@@ -7847,7 +7848,7 @@
       <c r="AA41" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="AB41" s="47" t="s">
+      <c r="AB41" s="46" t="s">
         <v>498</v>
       </c>
       <c r="AC41" s="30" t="s">
@@ -7856,7 +7857,7 @@
       <c r="AD41" s="30" t="s">
         <v>497</v>
       </c>
-      <c r="AE41" s="67" t="s">
+      <c r="AE41" s="66" t="s">
         <v>575</v>
       </c>
     </row>
@@ -7864,7 +7865,7 @@
       <c r="A42" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B42" s="55" t="s">
+      <c r="B42" s="54" t="s">
         <v>134</v>
       </c>
       <c r="C42" s="2" t="s">
@@ -7942,7 +7943,7 @@
       <c r="AA42" s="34" t="s">
         <v>134</v>
       </c>
-      <c r="AB42" s="47" t="s">
+      <c r="AB42" s="46" t="s">
         <v>401</v>
       </c>
       <c r="AC42" s="34" t="s">
@@ -7951,7 +7952,7 @@
       <c r="AD42" s="34" t="s">
         <v>400</v>
       </c>
-      <c r="AE42" s="61" t="s">
+      <c r="AE42" s="60" t="s">
         <v>570</v>
       </c>
     </row>
@@ -7959,7 +7960,7 @@
       <c r="A43" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B43" s="55" t="s">
+      <c r="B43" s="54" t="s">
         <v>379</v>
       </c>
       <c r="C43" s="4" t="s">
@@ -7989,7 +7990,7 @@
       <c r="K43" s="41" t="s">
         <v>92</v>
       </c>
-      <c r="L43" s="50">
+      <c r="L43" s="49">
         <v>31.381101000000001</v>
       </c>
       <c r="M43" s="41" t="s">
@@ -8037,7 +8038,7 @@
       <c r="AA43" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="AB43" s="48" t="s">
+      <c r="AB43" s="47" t="s">
         <v>381</v>
       </c>
       <c r="AC43" s="34" t="s">
@@ -8046,7 +8047,7 @@
       <c r="AD43" s="34" t="s">
         <v>383</v>
       </c>
-      <c r="AE43" s="61" t="s">
+      <c r="AE43" s="60" t="s">
         <v>570</v>
       </c>
     </row>
@@ -8054,7 +8055,7 @@
       <c r="A44" s="22" t="s">
         <v>126</v>
       </c>
-      <c r="B44" s="55" t="s">
+      <c r="B44" s="54" t="s">
         <v>127</v>
       </c>
       <c r="C44" s="4" t="s">
@@ -8132,7 +8133,7 @@
       <c r="AA44" s="34" t="s">
         <v>129</v>
       </c>
-      <c r="AB44" s="47" t="s">
+      <c r="AB44" s="46" t="s">
         <v>506</v>
       </c>
       <c r="AC44" s="34" t="s">
@@ -8141,7 +8142,7 @@
       <c r="AD44" s="34" t="s">
         <v>508</v>
       </c>
-      <c r="AE44" s="61" t="s">
+      <c r="AE44" s="60" t="s">
         <v>570</v>
       </c>
     </row>
@@ -8149,7 +8150,7 @@
       <c r="A45" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="B45" s="55" t="s">
+      <c r="B45" s="54" t="s">
         <v>267</v>
       </c>
       <c r="C45" s="4" t="s">
@@ -8227,7 +8228,7 @@
       <c r="AA45" s="34" t="s">
         <v>268</v>
       </c>
-      <c r="AB45" s="47" t="s">
+      <c r="AB45" s="46" t="s">
         <v>509</v>
       </c>
       <c r="AC45" s="34" t="s">
@@ -8236,7 +8237,7 @@
       <c r="AD45" s="34" t="s">
         <v>513</v>
       </c>
-      <c r="AE45" s="65" t="s">
+      <c r="AE45" s="64" t="s">
         <v>573</v>
       </c>
     </row>
@@ -8244,7 +8245,7 @@
       <c r="A46" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B46" s="57" t="s">
+      <c r="B46" s="56" t="s">
         <v>212</v>
       </c>
       <c r="C46" s="2" t="s">
@@ -8274,7 +8275,7 @@
       <c r="K46" s="40" t="s">
         <v>92</v>
       </c>
-      <c r="L46" s="51">
+      <c r="L46" s="50">
         <v>6.8833489999999999</v>
       </c>
       <c r="M46" s="40">
@@ -8322,7 +8323,7 @@
       <c r="AA46" s="30" t="s">
         <v>215</v>
       </c>
-      <c r="AB46" s="47" t="s">
+      <c r="AB46" s="46" t="s">
         <v>406</v>
       </c>
       <c r="AC46" s="30" t="s">
@@ -8331,15 +8332,15 @@
       <c r="AD46" s="30" t="s">
         <v>405</v>
       </c>
-      <c r="AE46" s="63" t="s">
-        <v>27</v>
+      <c r="AE46" s="64" t="s">
+        <v>573</v>
       </c>
     </row>
     <row r="47" spans="1:31" ht="114" x14ac:dyDescent="0.3">
       <c r="A47" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="B47" s="56" t="s">
+      <c r="B47" s="55" t="s">
         <v>153</v>
       </c>
       <c r="C47" s="2" t="s">
@@ -8357,7 +8358,7 @@
       <c r="G47" s="2" t="s">
         <v>515</v>
       </c>
-      <c r="H47" s="53">
+      <c r="H47" s="52">
         <v>1.55E-2</v>
       </c>
       <c r="I47" s="40" t="s">
@@ -8417,7 +8418,7 @@
       <c r="AA47" s="30" t="s">
         <v>155</v>
       </c>
-      <c r="AB47" s="47" t="s">
+      <c r="AB47" s="46" t="s">
         <v>518</v>
       </c>
       <c r="AC47" s="30" t="s">
@@ -8426,7 +8427,7 @@
       <c r="AD47" s="30" t="s">
         <v>517</v>
       </c>
-      <c r="AE47" s="66" t="s">
+      <c r="AE47" s="65" t="s">
         <v>574</v>
       </c>
     </row>
@@ -8434,7 +8435,7 @@
       <c r="A48" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B48" s="55" t="s">
+      <c r="B48" s="54" t="s">
         <v>346</v>
       </c>
       <c r="C48" s="2" t="s">
@@ -8512,7 +8513,7 @@
       <c r="AA48" s="34" t="s">
         <v>311</v>
       </c>
-      <c r="AB48" s="48" t="s">
+      <c r="AB48" s="47" t="s">
         <v>350</v>
       </c>
       <c r="AC48" s="34" t="s">
@@ -8521,7 +8522,7 @@
       <c r="AD48" s="34" t="s">
         <v>349</v>
       </c>
-      <c r="AE48" s="62" t="s">
+      <c r="AE48" s="61" t="s">
         <v>571</v>
       </c>
     </row>
@@ -8529,7 +8530,7 @@
       <c r="A49" s="22" t="s">
         <v>126</v>
       </c>
-      <c r="B49" s="55" t="s">
+      <c r="B49" s="54" t="s">
         <v>149</v>
       </c>
       <c r="C49" s="4" t="s">
@@ -8547,7 +8548,7 @@
       <c r="G49" s="4" t="s">
         <v>521</v>
       </c>
-      <c r="H49" s="54">
+      <c r="H49" s="53">
         <v>6.7077999999999999E-2</v>
       </c>
       <c r="I49" s="41" t="s">
@@ -8559,7 +8560,7 @@
       <c r="K49" s="41" t="s">
         <v>92</v>
       </c>
-      <c r="L49" s="49">
+      <c r="L49" s="48">
         <v>0.67078000000000004</v>
       </c>
       <c r="M49" s="41" t="s">
@@ -8607,7 +8608,7 @@
       <c r="AA49" s="34" t="s">
         <v>152</v>
       </c>
-      <c r="AB49" s="47" t="s">
+      <c r="AB49" s="46" t="s">
         <v>522</v>
       </c>
       <c r="AC49" s="34" t="s">
@@ -8616,7 +8617,7 @@
       <c r="AD49" s="34" t="s">
         <v>524</v>
       </c>
-      <c r="AE49" s="65" t="s">
+      <c r="AE49" s="64" t="s">
         <v>573</v>
       </c>
     </row>
@@ -8624,7 +8625,7 @@
       <c r="A50" s="22" t="s">
         <v>126</v>
       </c>
-      <c r="B50" s="55" t="s">
+      <c r="B50" s="54" t="s">
         <v>209</v>
       </c>
       <c r="C50" s="34" t="s">
@@ -8648,7 +8649,7 @@
       <c r="I50" s="41"/>
       <c r="J50" s="41"/>
       <c r="K50" s="41"/>
-      <c r="L50" s="49">
+      <c r="L50" s="48">
         <v>2.4073790000000002</v>
       </c>
       <c r="M50" s="41"/>
@@ -8690,7 +8691,7 @@
       <c r="AA50" s="34" t="s">
         <v>211</v>
       </c>
-      <c r="AB50" s="47" t="s">
+      <c r="AB50" s="46" t="s">
         <v>526</v>
       </c>
       <c r="AC50" s="34" t="s">
@@ -8699,7 +8700,7 @@
       <c r="AD50" s="34" t="s">
         <v>528</v>
       </c>
-      <c r="AE50" s="66" t="s">
+      <c r="AE50" s="65" t="s">
         <v>574</v>
       </c>
     </row>
@@ -8707,7 +8708,7 @@
       <c r="A51" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="B51" s="56" t="s">
+      <c r="B51" s="55" t="s">
         <v>182</v>
       </c>
       <c r="C51" s="2" t="s">
@@ -8728,16 +8729,16 @@
       <c r="H51" s="31">
         <v>0.27411429999999998</v>
       </c>
-      <c r="I51" s="58">
+      <c r="I51" s="57">
         <v>0.33400000000000002</v>
       </c>
       <c r="J51" s="40" t="s">
         <v>92</v>
       </c>
-      <c r="K51" s="58">
+      <c r="K51" s="57">
         <v>0.33400000000000002</v>
       </c>
-      <c r="L51" s="59">
+      <c r="L51" s="58">
         <v>2.7411430000000001</v>
       </c>
       <c r="M51" s="40">
@@ -8785,7 +8786,7 @@
       <c r="AA51" s="30" t="s">
         <v>184</v>
       </c>
-      <c r="AB51" s="47" t="s">
+      <c r="AB51" s="46" t="s">
         <v>530</v>
       </c>
       <c r="AC51" s="30" t="s">
@@ -8794,7 +8795,7 @@
       <c r="AD51" s="30" t="s">
         <v>532</v>
       </c>
-      <c r="AE51" s="66" t="s">
+      <c r="AE51" s="65" t="s">
         <v>574</v>
       </c>
     </row>
@@ -8802,7 +8803,7 @@
       <c r="A52" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B52" s="55" t="s">
+      <c r="B52" s="54" t="s">
         <v>156</v>
       </c>
       <c r="C52" s="2" t="s">
@@ -8880,7 +8881,7 @@
       <c r="AA52" s="34" t="s">
         <v>159</v>
       </c>
-      <c r="AB52" s="47" t="s">
+      <c r="AB52" s="46" t="s">
         <v>160</v>
       </c>
       <c r="AC52" s="34" t="s">
@@ -8889,7 +8890,7 @@
       <c r="AD52" s="34" t="s">
         <v>162</v>
       </c>
-      <c r="AE52" s="67" t="s">
+      <c r="AE52" s="66" t="s">
         <v>575</v>
       </c>
     </row>
@@ -8897,7 +8898,7 @@
       <c r="A53" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="B53" s="56" t="s">
+      <c r="B53" s="55" t="s">
         <v>234</v>
       </c>
       <c r="C53" s="4" t="s">
@@ -8975,7 +8976,7 @@
       <c r="AA53" s="30" t="s">
         <v>236</v>
       </c>
-      <c r="AB53" s="47" t="s">
+      <c r="AB53" s="46" t="s">
         <v>537</v>
       </c>
       <c r="AC53" s="30" t="s">
@@ -8984,7 +8985,7 @@
       <c r="AD53" s="30" t="s">
         <v>540</v>
       </c>
-      <c r="AE53" s="68" t="s">
+      <c r="AE53" s="67" t="s">
         <v>29</v>
       </c>
     </row>
@@ -8992,7 +8993,7 @@
       <c r="A54" s="23" t="s">
         <v>163</v>
       </c>
-      <c r="B54" s="56" t="s">
+      <c r="B54" s="55" t="s">
         <v>275</v>
       </c>
       <c r="C54" s="2" t="s">
@@ -9070,7 +9071,7 @@
       <c r="AA54" s="30" t="s">
         <v>276</v>
       </c>
-      <c r="AB54" s="47" t="s">
+      <c r="AB54" s="46" t="s">
         <v>543</v>
       </c>
       <c r="AC54" s="30" t="s">
@@ -9079,7 +9080,7 @@
       <c r="AD54" s="30" t="s">
         <v>545</v>
       </c>
-      <c r="AE54" s="66" t="s">
+      <c r="AE54" s="65" t="s">
         <v>574</v>
       </c>
     </row>
@@ -9087,7 +9088,7 @@
       <c r="A55" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B55" s="56" t="s">
+      <c r="B55" s="55" t="s">
         <v>265</v>
       </c>
       <c r="C55" s="2" t="s">
@@ -9163,7 +9164,7 @@
         <v>594</v>
       </c>
       <c r="AA55" s="30"/>
-      <c r="AB55" s="47" t="s">
+      <c r="AB55" s="46" t="s">
         <v>266</v>
       </c>
       <c r="AC55" s="30" t="s">
@@ -9172,7 +9173,7 @@
       <c r="AD55" s="30" t="s">
         <v>389</v>
       </c>
-      <c r="AE55" s="61" t="s">
+      <c r="AE55" s="60" t="s">
         <v>570</v>
       </c>
     </row>
@@ -9180,7 +9181,7 @@
       <c r="A56" s="23" t="s">
         <v>163</v>
       </c>
-      <c r="B56" s="56" t="s">
+      <c r="B56" s="55" t="s">
         <v>190</v>
       </c>
       <c r="C56" s="2" t="s">
@@ -9258,7 +9259,7 @@
       <c r="AA56" s="30" t="s">
         <v>191</v>
       </c>
-      <c r="AB56" s="47" t="s">
+      <c r="AB56" s="46" t="s">
         <v>552</v>
       </c>
       <c r="AC56" s="30" t="s">
@@ -9267,7 +9268,7 @@
       <c r="AD56" s="30" t="s">
         <v>554</v>
       </c>
-      <c r="AE56" s="65" t="s">
+      <c r="AE56" s="64" t="s">
         <v>573</v>
       </c>
     </row>
@@ -9275,7 +9276,7 @@
       <c r="A57" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B57" s="56" t="s">
+      <c r="B57" s="55" t="s">
         <v>302</v>
       </c>
       <c r="C57" s="2" t="s">
@@ -9362,7 +9363,7 @@
       <c r="AD57" s="30" t="s">
         <v>558</v>
       </c>
-      <c r="AE57" s="61" t="s">
+      <c r="AE57" s="60" t="s">
         <v>570</v>
       </c>
     </row>
@@ -9370,7 +9371,7 @@
       <c r="A58" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="B58" s="56" t="s">
+      <c r="B58" s="55" t="s">
         <v>228</v>
       </c>
       <c r="C58" s="4" t="s">
@@ -9388,7 +9389,7 @@
       <c r="G58" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="H58" s="53">
+      <c r="H58" s="52">
         <v>7.8E-2</v>
       </c>
       <c r="I58" s="40" t="s">
@@ -9400,7 +9401,7 @@
       <c r="K58" s="40" t="s">
         <v>92</v>
       </c>
-      <c r="L58" s="60">
+      <c r="L58" s="59">
         <v>0.784304</v>
       </c>
       <c r="M58" s="40" t="s">
@@ -9448,7 +9449,7 @@
       <c r="AA58" s="30" t="s">
         <v>230</v>
       </c>
-      <c r="AB58" s="47" t="s">
+      <c r="AB58" s="46" t="s">
         <v>566</v>
       </c>
       <c r="AC58" s="30" t="s">
@@ -9457,7 +9458,7 @@
       <c r="AD58" s="30" t="s">
         <v>568</v>
       </c>
-      <c r="AE58" s="61" t="s">
+      <c r="AE58" s="60" t="s">
         <v>570</v>
       </c>
     </row>
@@ -9465,7 +9466,7 @@
       <c r="A59" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B59" s="55" t="s">
+      <c r="B59" s="54" t="s">
         <v>297</v>
       </c>
       <c r="C59" s="4" t="s">
@@ -9483,7 +9484,7 @@
       <c r="G59" s="4" t="s">
         <v>298</v>
       </c>
-      <c r="H59" s="54">
+      <c r="H59" s="53">
         <v>8.5999999999999993E-2</v>
       </c>
       <c r="I59" s="41">
@@ -9552,7 +9553,7 @@
       <c r="AD59" s="34" t="s">
         <v>301</v>
       </c>
-      <c r="AE59" s="62" t="s">
+      <c r="AE59" s="61" t="s">
         <v>571</v>
       </c>
     </row>
@@ -9560,7 +9561,7 @@
       <c r="A60" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="B60" s="55" t="s">
+      <c r="B60" s="54" t="s">
         <v>185</v>
       </c>
       <c r="C60" s="4" t="s">
@@ -9638,7 +9639,7 @@
       <c r="AA60" s="34" t="s">
         <v>188</v>
       </c>
-      <c r="AB60" s="47" t="s">
+      <c r="AB60" s="46" t="s">
         <v>561</v>
       </c>
       <c r="AC60" s="34" t="s">
@@ -9647,7 +9648,7 @@
       <c r="AD60" s="34" t="s">
         <v>189</v>
       </c>
-      <c r="AE60" s="61" t="s">
+      <c r="AE60" s="60" t="s">
         <v>570</v>
       </c>
     </row>
@@ -9655,7 +9656,7 @@
       <c r="A61" s="22" t="s">
         <v>126</v>
       </c>
-      <c r="B61" s="55" t="s">
+      <c r="B61" s="54" t="s">
         <v>271</v>
       </c>
       <c r="C61" s="2" t="s">
@@ -9733,7 +9734,7 @@
       <c r="AA61" s="34" t="s">
         <v>273</v>
       </c>
-      <c r="AB61" s="47" t="s">
+      <c r="AB61" s="46" t="s">
         <v>564</v>
       </c>
       <c r="AC61" s="34" t="s">
@@ -9742,7 +9743,7 @@
       <c r="AD61" s="34" t="s">
         <v>274</v>
       </c>
-      <c r="AE61" s="66" t="s">
+      <c r="AE61" s="65" t="s">
         <v>574</v>
       </c>
     </row>
@@ -9821,6 +9822,314 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D4FF1D5-A91D-4300-B515-F6FD45A4A36E}">
+  <dimension ref="A1:A60"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="40">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="31">
+        <v>0.112</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="35" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="31">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="40">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" s="41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" s="40">
+        <v>0.78300000000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" s="52">
+        <v>7.6649999999999999E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" s="41">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" s="41">
+        <v>0.57999999999999996</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" s="41">
+        <v>6.4000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" s="41">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A15" s="40">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" s="51">
+        <v>4.5999999999999999E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" s="40">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" s="41">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" s="41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" s="41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" s="40">
+        <v>1.2999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" s="41">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" s="41">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" s="41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" s="41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" s="40">
+        <v>0.19500000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" s="40">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28" s="40">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" s="41">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A30" s="41">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31" s="41">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A32" s="40">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" s="40">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" s="41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35" s="41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36" s="41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A37" s="41">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38" s="40">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A39" s="40">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A40" s="40">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A41" s="41">
+        <v>0.36599999999999999</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A42" s="41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A43" s="41">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A44" s="41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A45" s="40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A46" s="40" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A47" s="41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A48" s="41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" s="41"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50" s="57">
+        <v>0.33400000000000002</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A51" s="41">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A52" s="40">
+        <v>3.4000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A53" s="40">
+        <v>0.126</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A54" s="40" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A55" s="40">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A56" s="40" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A57" s="40" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A58" s="41">
+        <v>5.6000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A59" s="41">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A60" s="41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor rgb="FF888888"/>
@@ -9835,162 +10144,155 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="76" t="s">
+      <c r="A1" s="86" t="s">
         <v>317</v>
       </c>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="79" t="s">
+      <c r="A3" s="72" t="s">
         <v>318</v>
       </c>
-      <c r="B3" s="75"/>
-      <c r="C3" s="75"/>
-      <c r="D3" s="75"/>
-      <c r="E3" s="75"/>
+      <c r="B3" s="73"/>
+      <c r="C3" s="73"/>
+      <c r="D3" s="73"/>
+      <c r="E3" s="73"/>
     </row>
     <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="83" t="s">
+      <c r="A4" s="92" t="s">
         <v>319</v>
       </c>
-      <c r="B4" s="73"/>
-      <c r="C4" s="74" t="s">
+      <c r="B4" s="76"/>
+      <c r="C4" s="81" t="s">
         <v>320</v>
       </c>
-      <c r="D4" s="75"/>
-      <c r="E4" s="75"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="73"/>
     </row>
     <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="80" t="s">
+      <c r="A5" s="89" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="73"/>
-      <c r="C5" s="74" t="s">
+      <c r="B5" s="76"/>
+      <c r="C5" s="81" t="s">
         <v>321</v>
       </c>
-      <c r="D5" s="75"/>
-      <c r="E5" s="75"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="73"/>
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="77" t="s">
+      <c r="A6" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="73"/>
-      <c r="C6" s="74" t="s">
+      <c r="B6" s="76"/>
+      <c r="C6" s="81" t="s">
         <v>322</v>
       </c>
-      <c r="D6" s="75"/>
-      <c r="E6" s="75"/>
+      <c r="D6" s="73"/>
+      <c r="E6" s="73"/>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="78" t="s">
+      <c r="A7" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="73"/>
-      <c r="C7" s="74" t="s">
+      <c r="B7" s="76"/>
+      <c r="C7" s="81" t="s">
         <v>323</v>
       </c>
-      <c r="D7" s="75"/>
-      <c r="E7" s="75"/>
+      <c r="D7" s="73"/>
+      <c r="E7" s="73"/>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="82" t="s">
+      <c r="A8" s="91" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="73"/>
-      <c r="C8" s="74" t="s">
+      <c r="B8" s="76"/>
+      <c r="C8" s="81" t="s">
         <v>324</v>
       </c>
-      <c r="D8" s="75"/>
-      <c r="E8" s="75"/>
+      <c r="D8" s="73"/>
+      <c r="E8" s="73"/>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="86" t="s">
+      <c r="A9" s="84" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="73"/>
-      <c r="C9" s="74" t="s">
+      <c r="B9" s="76"/>
+      <c r="C9" s="81" t="s">
         <v>325</v>
       </c>
-      <c r="D9" s="75"/>
-      <c r="E9" s="75"/>
+      <c r="D9" s="73"/>
+      <c r="E9" s="73"/>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="84" t="s">
+      <c r="A10" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="73"/>
-      <c r="C10" s="74" t="s">
+      <c r="B10" s="76"/>
+      <c r="C10" s="81" t="s">
         <v>326</v>
       </c>
-      <c r="D10" s="75"/>
-      <c r="E10" s="75"/>
+      <c r="D10" s="73"/>
+      <c r="E10" s="73"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="79" t="s">
+      <c r="A12" s="72" t="s">
         <v>327</v>
       </c>
-      <c r="B12" s="75"/>
-      <c r="C12" s="75"/>
-      <c r="D12" s="75"/>
-      <c r="E12" s="75"/>
+      <c r="B12" s="73"/>
+      <c r="C12" s="73"/>
+      <c r="D12" s="73"/>
+      <c r="E12" s="73"/>
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="85" t="s">
+      <c r="A13" s="83" t="s">
         <v>328</v>
       </c>
-      <c r="B13" s="73"/>
-      <c r="C13" s="74" t="s">
+      <c r="B13" s="76"/>
+      <c r="C13" s="81" t="s">
         <v>329</v>
       </c>
-      <c r="D13" s="75"/>
-      <c r="E13" s="75"/>
+      <c r="D13" s="73"/>
+      <c r="E13" s="73"/>
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="81" t="s">
+      <c r="A14" s="90" t="s">
         <v>330</v>
       </c>
-      <c r="B14" s="73"/>
-      <c r="C14" s="74" t="s">
+      <c r="B14" s="76"/>
+      <c r="C14" s="81" t="s">
         <v>331</v>
       </c>
-      <c r="D14" s="75"/>
-      <c r="E14" s="75"/>
+      <c r="D14" s="73"/>
+      <c r="E14" s="73"/>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="72" t="s">
+      <c r="A15" s="85" t="s">
         <v>332</v>
       </c>
-      <c r="B15" s="73"/>
-      <c r="C15" s="74" t="s">
+      <c r="B15" s="76"/>
+      <c r="C15" s="81" t="s">
         <v>333</v>
       </c>
-      <c r="D15" s="75"/>
-      <c r="E15" s="75"/>
+      <c r="D15" s="73"/>
+      <c r="E15" s="73"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="44" t="s">
+      <c r="A18" s="43" t="s">
         <v>334</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="43"/>
+      <c r="A19" s="42"/>
       <c r="B19" t="s">
         <v>335</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C10:E10"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="A1:E1"/>
@@ -10007,6 +10309,13 @@
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C6:E6"/>
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C10:E10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -10014,12 +10323,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10264,20 +10575,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CBE187-A7DE-4A9A-99BE-7485C92477B0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10302,18 +10620,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CBE187-A7DE-4A9A-99BE-7485C92477B0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
modified:   excel_data/Innovation_Fund_Projects_data - 130426.xlsx
</commit_message>
<xml_diff>
--- a/excel_data/Innovation_Fund_Projects_data - 130426.xlsx
+++ b/excel_data/Innovation_Fund_Projects_data - 130426.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zeplatform-my.sharepoint.com/personal/salman_muhammad_zeplatform_eu/Documents/Technical/IF mapping tool/if-map/excel_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1739" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFEA8AE1-D4F1-4A6E-B791-DE0730027B57}"/>
+  <xr:revisionPtr revIDLastSave="1781" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7873DA73-896B-4666-B4BC-58612B8B545B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
     <sheet name="IF Projects" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="4" r:id="rId3"/>
-    <sheet name="Legend" sheetId="3" r:id="rId4"/>
+    <sheet name="Legend" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'IF Projects'!$A$1:$AE$61</definedName>
@@ -694,7 +693,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1321" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1303" uniqueCount="597">
   <si>
     <t>EU Innovation Fund — CCS/CCU Project Portfolio Summary</t>
   </si>
@@ -1494,12 +1493,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://ec.europa.eu/assets/cinea/project_fiches/innovation_fund/101132987.pdf </t>
-  </si>
-  <si>
-    <t>Norwegian e-fuel pilot converting blast furnace gas into synthetic fuels via P2X, achieving &gt;99% GHG reduction.</t>
-  </si>
-  <si>
-    <t>Power-to-Liquid e-fuels: post-combustion amine CO₂ capture from ferro/silicon-manganese plant; PEM electrolysis green H₂; Fischer-Tropsch synthesis → e-SAF/liquid fuels; 22 kt/yr CO₂ input; small refinery pilot</t>
   </si>
   <si>
     <t>StarFish</t>
@@ -2494,6 +2487,18 @@
   </si>
   <si>
     <t>CO₂ Storage Site</t>
+  </si>
+  <si>
+    <t>E-Fuel Pilot is a Power-to-Liquid synthetic fuel project developed by Nordic Electrofuel AS at Herøya Industrial Park in Porsgrunn, Norway. The plant uses captured CO₂ from a local ammonia plant, renewable electricity and hydrogen to produce about 8,000 tonnes per year of synthetic hydrocarbons (syncrude) for aviation and other hard-to-abate transport uses. The project is backed by a €40 million Innovation Fund grant and is expected to deliver 228,163 tonnes CO₂e of avoided emissions over its first 10 years of operation.</t>
+  </si>
+  <si>
+    <t>The project applies a Power-to-Liquid route in which captured CO₂ from a local ammonia plant is combined with renewable hydrogen and converted through reverse water-gas shift (RWGS) to synthesis gas, followed by Fischer-Tropsch synthesis to produce approximately 8,000 t/year of synthetic hydrocarbons (syncrude). Public project sources describe carbon utilisation close to 100% and include a Safire reactor / gas-gas syngas cooler concept to improve heat recovery and process efficiency; no geological CO₂ storage component is indicated.</t>
+  </si>
+  <si>
+    <t>Fertilisers</t>
+  </si>
+  <si>
+    <t>Metals &amp; Mining</t>
   </si>
 </sst>
 </file>
@@ -2861,7 +2866,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3073,6 +3078,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -3446,40 +3454,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
+      <c r="F1" s="74"/>
+      <c r="G1" s="74"/>
+      <c r="H1" s="74"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="80" t="s">
+      <c r="A2" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
+      <c r="B2" s="74"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="74"/>
+      <c r="G2" s="74"/>
+      <c r="H2" s="74"/>
     </row>
     <row r="4" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="72" t="s">
+      <c r="A4" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="73"/>
-      <c r="C4" s="73"/>
-      <c r="D4" s="73"/>
-      <c r="E4" s="73"/>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73"/>
-      <c r="H4" s="73"/>
+      <c r="B4" s="74"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="74"/>
+      <c r="F4" s="74"/>
+      <c r="G4" s="74"/>
+      <c r="H4" s="74"/>
     </row>
     <row r="5" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3496,12 +3504,12 @@
       <c r="B6" s="3">
         <v>62</v>
       </c>
-      <c r="C6" s="73"/>
-      <c r="D6" s="73"/>
-      <c r="E6" s="73"/>
-      <c r="F6" s="73"/>
-      <c r="G6" s="73"/>
-      <c r="H6" s="73"/>
+      <c r="C6" s="74"/>
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="74"/>
+      <c r="G6" s="74"/>
+      <c r="H6" s="74"/>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
@@ -3510,12 +3518,12 @@
       <c r="B7" s="5">
         <v>16</v>
       </c>
-      <c r="C7" s="73"/>
-      <c r="D7" s="73"/>
-      <c r="E7" s="73"/>
-      <c r="F7" s="73"/>
-      <c r="G7" s="73"/>
-      <c r="H7" s="73"/>
+      <c r="C7" s="74"/>
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
+      <c r="F7" s="74"/>
+      <c r="G7" s="74"/>
+      <c r="H7" s="74"/>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -3524,12 +3532,12 @@
       <c r="B8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="73"/>
-      <c r="D8" s="73"/>
-      <c r="E8" s="73"/>
-      <c r="F8" s="73"/>
-      <c r="G8" s="73"/>
-      <c r="H8" s="73"/>
+      <c r="C8" s="74"/>
+      <c r="D8" s="74"/>
+      <c r="E8" s="74"/>
+      <c r="F8" s="74"/>
+      <c r="G8" s="74"/>
+      <c r="H8" s="74"/>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
@@ -3538,12 +3546,12 @@
       <c r="B9" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="73"/>
-      <c r="D9" s="73"/>
-      <c r="E9" s="73"/>
-      <c r="F9" s="73"/>
-      <c r="G9" s="73"/>
-      <c r="H9" s="73"/>
+      <c r="C9" s="74"/>
+      <c r="D9" s="74"/>
+      <c r="E9" s="74"/>
+      <c r="F9" s="74"/>
+      <c r="G9" s="74"/>
+      <c r="H9" s="74"/>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -3552,12 +3560,12 @@
       <c r="B10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="73"/>
-      <c r="D10" s="73"/>
-      <c r="E10" s="73"/>
-      <c r="F10" s="73"/>
-      <c r="G10" s="73"/>
-      <c r="H10" s="73"/>
+      <c r="C10" s="74"/>
+      <c r="D10" s="74"/>
+      <c r="E10" s="74"/>
+      <c r="F10" s="74"/>
+      <c r="G10" s="74"/>
+      <c r="H10" s="74"/>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
@@ -3566,12 +3574,12 @@
       <c r="B11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="73"/>
-      <c r="D11" s="73"/>
-      <c r="E11" s="73"/>
-      <c r="F11" s="73"/>
-      <c r="G11" s="73"/>
-      <c r="H11" s="73"/>
+      <c r="C11" s="74"/>
+      <c r="D11" s="74"/>
+      <c r="E11" s="74"/>
+      <c r="F11" s="74"/>
+      <c r="G11" s="74"/>
+      <c r="H11" s="74"/>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
@@ -3580,24 +3588,24 @@
       <c r="B12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="73"/>
-      <c r="D12" s="73"/>
-      <c r="E12" s="73"/>
-      <c r="F12" s="73"/>
-      <c r="G12" s="73"/>
-      <c r="H12" s="73"/>
+      <c r="C12" s="74"/>
+      <c r="D12" s="74"/>
+      <c r="E12" s="74"/>
+      <c r="F12" s="74"/>
+      <c r="G12" s="74"/>
+      <c r="H12" s="74"/>
     </row>
     <row r="15" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="72" t="s">
+      <c r="A15" s="73" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="73"/>
-      <c r="C15" s="73"/>
-      <c r="D15" s="73"/>
-      <c r="E15" s="73"/>
-      <c r="F15" s="73"/>
-      <c r="G15" s="73"/>
-      <c r="H15" s="73"/>
+      <c r="B15" s="74"/>
+      <c r="C15" s="74"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="74"/>
+      <c r="F15" s="74"/>
+      <c r="G15" s="74"/>
+      <c r="H15" s="74"/>
     </row>
     <row r="16" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -3606,14 +3614,14 @@
       <c r="B16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="79" t="s">
+      <c r="C16" s="80" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="75"/>
-      <c r="E16" s="75"/>
-      <c r="F16" s="75"/>
-      <c r="G16" s="75"/>
-      <c r="H16" s="76"/>
+      <c r="D16" s="76"/>
+      <c r="E16" s="76"/>
+      <c r="F16" s="76"/>
+      <c r="G16" s="76"/>
+      <c r="H16" s="77"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
@@ -3622,14 +3630,14 @@
       <c r="B17" s="9">
         <v>21</v>
       </c>
-      <c r="C17" s="74" t="s">
+      <c r="C17" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="75"/>
-      <c r="E17" s="75"/>
-      <c r="F17" s="75"/>
-      <c r="G17" s="75"/>
-      <c r="H17" s="76"/>
+      <c r="D17" s="76"/>
+      <c r="E17" s="76"/>
+      <c r="F17" s="76"/>
+      <c r="G17" s="76"/>
+      <c r="H17" s="77"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
@@ -3638,14 +3646,14 @@
       <c r="B18" s="11">
         <v>20</v>
       </c>
-      <c r="C18" s="78" t="s">
+      <c r="C18" s="79" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="75"/>
-      <c r="E18" s="75"/>
-      <c r="F18" s="75"/>
-      <c r="G18" s="75"/>
-      <c r="H18" s="76"/>
+      <c r="D18" s="76"/>
+      <c r="E18" s="76"/>
+      <c r="F18" s="76"/>
+      <c r="G18" s="76"/>
+      <c r="H18" s="77"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -3654,14 +3662,14 @@
       <c r="B19" s="13">
         <v>10</v>
       </c>
-      <c r="C19" s="74" t="s">
+      <c r="C19" s="75" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="75"/>
-      <c r="E19" s="75"/>
-      <c r="F19" s="75"/>
-      <c r="G19" s="75"/>
-      <c r="H19" s="76"/>
+      <c r="D19" s="76"/>
+      <c r="E19" s="76"/>
+      <c r="F19" s="76"/>
+      <c r="G19" s="76"/>
+      <c r="H19" s="77"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
@@ -3670,14 +3678,14 @@
       <c r="B20" s="15">
         <v>4</v>
       </c>
-      <c r="C20" s="78" t="s">
+      <c r="C20" s="79" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="75"/>
-      <c r="E20" s="75"/>
-      <c r="F20" s="75"/>
-      <c r="G20" s="75"/>
-      <c r="H20" s="76"/>
+      <c r="D20" s="76"/>
+      <c r="E20" s="76"/>
+      <c r="F20" s="76"/>
+      <c r="G20" s="76"/>
+      <c r="H20" s="77"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
@@ -3686,14 +3694,14 @@
       <c r="B21" s="17">
         <v>3</v>
       </c>
-      <c r="C21" s="74" t="s">
+      <c r="C21" s="75" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="75"/>
-      <c r="E21" s="75"/>
-      <c r="F21" s="75"/>
-      <c r="G21" s="75"/>
-      <c r="H21" s="76"/>
+      <c r="D21" s="76"/>
+      <c r="E21" s="76"/>
+      <c r="F21" s="76"/>
+      <c r="G21" s="76"/>
+      <c r="H21" s="77"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="16" t="s">
@@ -3702,14 +3710,14 @@
       <c r="B22" s="17">
         <v>1</v>
       </c>
-      <c r="C22" s="78" t="s">
+      <c r="C22" s="79" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="75"/>
-      <c r="E22" s="75"/>
-      <c r="F22" s="75"/>
-      <c r="G22" s="75"/>
-      <c r="H22" s="76"/>
+      <c r="D22" s="76"/>
+      <c r="E22" s="76"/>
+      <c r="F22" s="76"/>
+      <c r="G22" s="76"/>
+      <c r="H22" s="77"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="16" t="s">
@@ -3718,14 +3726,14 @@
       <c r="B23" s="17">
         <v>1</v>
       </c>
-      <c r="C23" s="74" t="s">
+      <c r="C23" s="75" t="s">
         <v>34</v>
       </c>
-      <c r="D23" s="75"/>
-      <c r="E23" s="75"/>
-      <c r="F23" s="75"/>
-      <c r="G23" s="75"/>
-      <c r="H23" s="76"/>
+      <c r="D23" s="76"/>
+      <c r="E23" s="76"/>
+      <c r="F23" s="76"/>
+      <c r="G23" s="76"/>
+      <c r="H23" s="77"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="s">
@@ -3734,14 +3742,14 @@
       <c r="B24" s="19">
         <v>1</v>
       </c>
-      <c r="C24" s="78" t="s">
+      <c r="C24" s="79" t="s">
         <v>36</v>
       </c>
-      <c r="D24" s="75"/>
-      <c r="E24" s="75"/>
-      <c r="F24" s="75"/>
-      <c r="G24" s="75"/>
-      <c r="H24" s="76"/>
+      <c r="D24" s="76"/>
+      <c r="E24" s="76"/>
+      <c r="F24" s="76"/>
+      <c r="G24" s="76"/>
+      <c r="H24" s="77"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="20" t="s">
@@ -3750,26 +3758,26 @@
       <c r="B25" s="21">
         <v>1</v>
       </c>
-      <c r="C25" s="74" t="s">
+      <c r="C25" s="75" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="75"/>
-      <c r="E25" s="75"/>
-      <c r="F25" s="75"/>
-      <c r="G25" s="75"/>
-      <c r="H25" s="76"/>
+      <c r="D25" s="76"/>
+      <c r="E25" s="76"/>
+      <c r="F25" s="76"/>
+      <c r="G25" s="76"/>
+      <c r="H25" s="77"/>
     </row>
     <row r="28" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="72" t="s">
+      <c r="A28" s="73" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="73"/>
-      <c r="C28" s="73"/>
-      <c r="D28" s="73"/>
-      <c r="E28" s="73"/>
-      <c r="F28" s="73"/>
-      <c r="G28" s="73"/>
-      <c r="H28" s="73"/>
+      <c r="B28" s="74"/>
+      <c r="C28" s="74"/>
+      <c r="D28" s="74"/>
+      <c r="E28" s="74"/>
+      <c r="F28" s="74"/>
+      <c r="G28" s="74"/>
+      <c r="H28" s="74"/>
     </row>
     <row r="29" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -4022,10 +4030,10 @@
         <v>74</v>
       </c>
       <c r="Q1" s="28" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="R1" s="28" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="S1" s="28" t="s">
         <v>75</v>
@@ -4129,7 +4137,7 @@
         <v>220123498</v>
       </c>
       <c r="U2" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V2" s="24">
         <v>57.062100000000001</v>
@@ -4144,22 +4152,22 @@
         <v>139</v>
       </c>
       <c r="Z2" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA2" s="30" t="s">
         <v>140</v>
       </c>
       <c r="AB2" s="46" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="AC2" s="30" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="AD2" s="30" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="AE2" s="60" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="3" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -4167,7 +4175,7 @@
         <v>141</v>
       </c>
       <c r="B3" s="55" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>242</v>
@@ -4224,7 +4232,7 @@
         <v>31238542</v>
       </c>
       <c r="U3" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V3" s="24">
         <v>44.464755134852901</v>
@@ -4236,10 +4244,10 @@
         <v>95</v>
       </c>
       <c r="Y3" s="30" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="Z3" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA3" s="30" t="s">
         <v>92</v>
@@ -4248,13 +4256,13 @@
         <v>250</v>
       </c>
       <c r="AC3" s="30" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="AD3" s="30" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="AE3" s="61" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="4" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -4262,7 +4270,7 @@
         <v>98</v>
       </c>
       <c r="B4" s="54" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>108</v>
@@ -4274,10 +4282,10 @@
         <v>52</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="H4" s="35" t="s">
         <v>92</v>
@@ -4319,7 +4327,7 @@
         <v>3168000</v>
       </c>
       <c r="U4" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V4" s="26">
         <v>43.327720234653299</v>
@@ -4331,22 +4339,22 @@
         <v>95</v>
       </c>
       <c r="Y4" s="34" t="s">
+        <v>340</v>
+      </c>
+      <c r="Z4" s="34" t="s">
+        <v>589</v>
+      </c>
+      <c r="AA4" s="34" t="s">
+        <v>290</v>
+      </c>
+      <c r="AB4" s="46" t="s">
+        <v>349</v>
+      </c>
+      <c r="AC4" s="34" t="s">
+        <v>341</v>
+      </c>
+      <c r="AD4" s="34" t="s">
         <v>342</v>
-      </c>
-      <c r="Z4" s="34" t="s">
-        <v>591</v>
-      </c>
-      <c r="AA4" s="34" t="s">
-        <v>292</v>
-      </c>
-      <c r="AB4" s="46" t="s">
-        <v>351</v>
-      </c>
-      <c r="AC4" s="34" t="s">
-        <v>343</v>
-      </c>
-      <c r="AD4" s="34" t="s">
-        <v>344</v>
       </c>
       <c r="AE4" s="62" t="s">
         <v>27</v>
@@ -4357,13 +4365,13 @@
         <v>119</v>
       </c>
       <c r="B5" s="55" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>108</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>42</v>
@@ -4399,7 +4407,7 @@
         <v>92</v>
       </c>
       <c r="P5" s="32" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="Q5" s="32">
         <v>2030</v>
@@ -4414,7 +4422,7 @@
         <v>170000000</v>
       </c>
       <c r="U5" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V5" s="24">
         <v>46.809800000000003</v>
@@ -4429,22 +4437,22 @@
         <v>177</v>
       </c>
       <c r="Z5" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA5" s="30" t="s">
         <v>178</v>
       </c>
       <c r="AB5" s="46" t="s">
+        <v>354</v>
+      </c>
+      <c r="AC5" s="30" t="s">
+        <v>355</v>
+      </c>
+      <c r="AD5" s="30" t="s">
         <v>356</v>
       </c>
-      <c r="AC5" s="30" t="s">
-        <v>357</v>
-      </c>
-      <c r="AD5" s="30" t="s">
-        <v>358</v>
-      </c>
       <c r="AE5" s="63" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="6" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -4452,10 +4460,10 @@
         <v>141</v>
       </c>
       <c r="B6" s="55" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="D6" s="30" t="s">
         <v>150</v>
@@ -4464,10 +4472,10 @@
         <v>45</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="H6" s="31">
         <v>2.5999999999999999E-2</v>
@@ -4509,7 +4517,7 @@
         <v>7958244</v>
       </c>
       <c r="U6" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V6" s="23" t="s">
         <v>92</v>
@@ -4524,22 +4532,22 @@
         <v>92</v>
       </c>
       <c r="Z6" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA6" s="30" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="AB6" s="46" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="AC6" s="30" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="AD6" s="30" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="AE6" s="64" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="7" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -4604,7 +4612,7 @@
         <v>189694949</v>
       </c>
       <c r="U7" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V7" s="24">
         <v>43.232830995956597</v>
@@ -4616,25 +4624,25 @@
         <v>132</v>
       </c>
       <c r="Y7" s="30" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="Z7" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA7" s="30" t="s">
         <v>133</v>
       </c>
       <c r="AB7" s="46" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="AC7" s="30" t="s">
+        <v>361</v>
+      </c>
+      <c r="AD7" s="30" t="s">
         <v>363</v>
       </c>
-      <c r="AD7" s="30" t="s">
-        <v>365</v>
-      </c>
       <c r="AE7" s="63" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="8" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -4684,7 +4692,7 @@
         <v>92</v>
       </c>
       <c r="P8" s="32" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="Q8" s="32">
         <v>2029</v>
@@ -4696,10 +4704,10 @@
         <v>122</v>
       </c>
       <c r="T8" s="33" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="U8" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V8" s="24">
         <v>50.575420999999999</v>
@@ -4714,22 +4722,22 @@
         <v>123</v>
       </c>
       <c r="Z8" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA8" s="30" t="s">
         <v>124</v>
       </c>
       <c r="AB8" s="46" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="AC8" s="30" t="s">
         <v>125</v>
       </c>
       <c r="AD8" s="30" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="AE8" s="63" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="9" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -4740,19 +4748,19 @@
         <v>224</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D9" s="34" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>50</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="H9" s="35">
         <v>2.5819174</v>
@@ -4794,7 +4802,7 @@
         <v>169300000</v>
       </c>
       <c r="U9" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V9" s="26">
         <v>37.960247145532399</v>
@@ -4806,25 +4814,25 @@
         <v>95</v>
       </c>
       <c r="Y9" s="34" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="Z9" s="34" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="AA9" s="34" t="s">
         <v>226</v>
       </c>
       <c r="AB9" s="46" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="AC9" s="34" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="AD9" s="34" t="s">
         <v>227</v>
       </c>
       <c r="AE9" s="61" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="10" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -4832,22 +4840,22 @@
         <v>87</v>
       </c>
       <c r="B10" s="55" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>58</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="H10" s="31" t="s">
         <v>92</v>
@@ -4901,22 +4909,22 @@
         <v>95</v>
       </c>
       <c r="Y10" s="30" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="Z10" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA10" s="30" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="AB10" s="46" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="AC10" s="30" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="AD10" s="30" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="AE10" s="62" t="s">
         <v>27</v>
@@ -4927,10 +4935,10 @@
         <v>126</v>
       </c>
       <c r="B11" s="55" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="D11" s="30" t="s">
         <v>150</v>
@@ -4939,10 +4947,10 @@
         <v>46</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="H11" s="31" t="s">
         <v>92</v>
@@ -4981,10 +4989,10 @@
         <v>122</v>
       </c>
       <c r="T11" s="33" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="U11" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V11" s="24">
         <v>59.592303479664103</v>
@@ -4996,25 +5004,25 @@
         <v>244</v>
       </c>
       <c r="Y11" s="30" t="s">
+        <v>422</v>
+      </c>
+      <c r="Z11" s="30" t="s">
+        <v>588</v>
+      </c>
+      <c r="AA11" s="30" t="s">
+        <v>268</v>
+      </c>
+      <c r="AB11" s="46" t="s">
+        <v>418</v>
+      </c>
+      <c r="AC11" s="30" t="s">
+        <v>423</v>
+      </c>
+      <c r="AD11" s="30" t="s">
         <v>424</v>
       </c>
-      <c r="Z11" s="30" t="s">
-        <v>590</v>
-      </c>
-      <c r="AA11" s="30" t="s">
-        <v>270</v>
-      </c>
-      <c r="AB11" s="46" t="s">
-        <v>420</v>
-      </c>
-      <c r="AC11" s="30" t="s">
-        <v>425</v>
-      </c>
-      <c r="AD11" s="30" t="s">
-        <v>426</v>
-      </c>
       <c r="AE11" s="63" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="12" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -5094,22 +5102,22 @@
         <v>194</v>
       </c>
       <c r="Z12" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA12" s="34" t="s">
         <v>195</v>
       </c>
       <c r="AB12" s="46" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="AC12" s="34" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="AD12" s="34" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="AE12" s="64" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="13" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5186,10 +5194,10 @@
         <v>95</v>
       </c>
       <c r="Y13" s="34" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="Z13" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA13" s="34" t="s">
         <v>167</v>
@@ -5198,13 +5206,13 @@
         <v>168</v>
       </c>
       <c r="AC13" s="34" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="AD13" s="34" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="AE13" s="60" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="14" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -5215,7 +5223,7 @@
         <v>246</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="D14" s="34" t="s">
         <v>109</v>
@@ -5269,7 +5277,7 @@
         <v>23635998</v>
       </c>
       <c r="U14" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V14" s="26">
         <v>44.826999999999998</v>
@@ -5284,22 +5292,22 @@
         <v>248</v>
       </c>
       <c r="Z14" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA14" s="34" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="AB14" s="46" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="AC14" s="34" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="AD14" s="34" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="AE14" s="64" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="15" spans="1:31" ht="148.19999999999999" x14ac:dyDescent="0.3">
@@ -5364,7 +5372,7 @@
         <v>119682059</v>
       </c>
       <c r="U15" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V15" s="26">
         <v>43.186100000000003</v>
@@ -5379,20 +5387,20 @@
         <v>176</v>
       </c>
       <c r="Z15" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA15" s="34"/>
       <c r="AB15" s="46" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="AC15" s="34" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="AD15" s="34" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="AE15" s="64" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="16" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5400,7 +5408,7 @@
         <v>119</v>
       </c>
       <c r="B16" s="55" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>108</v>
@@ -5412,10 +5420,10 @@
         <v>59</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="H16" s="31" t="s">
         <v>92</v>
@@ -5454,10 +5462,10 @@
         <v>122</v>
       </c>
       <c r="T16" s="33" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="U16" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V16" s="24">
         <v>45.290985428950698</v>
@@ -5469,25 +5477,25 @@
         <v>244</v>
       </c>
       <c r="Y16" s="30" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="Z16" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA16" s="30" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="AB16" s="46" t="s">
+        <v>428</v>
+      </c>
+      <c r="AC16" s="30" t="s">
         <v>430</v>
       </c>
-      <c r="AC16" s="30" t="s">
-        <v>432</v>
-      </c>
       <c r="AD16" s="30" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="AE16" s="65" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="17" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5510,7 +5518,7 @@
         <v>254</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="H17" s="51">
         <v>4.5999999999999999E-3</v>
@@ -5552,7 +5560,7 @@
         <v>30497000</v>
       </c>
       <c r="U17" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V17" s="23">
         <v>51.870851200822599</v>
@@ -5564,10 +5572,10 @@
         <v>244</v>
       </c>
       <c r="Y17" s="30" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="Z17" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA17" s="30" t="s">
         <v>255</v>
@@ -5576,10 +5584,10 @@
         <v>256</v>
       </c>
       <c r="AC17" s="30" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="AD17" s="30" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="AE17" s="62" t="s">
         <v>27</v>
@@ -5647,7 +5655,7 @@
         <v>157000000</v>
       </c>
       <c r="U18" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V18" s="24">
         <v>52.489100000000001</v>
@@ -5662,7 +5670,7 @@
         <v>206</v>
       </c>
       <c r="Z18" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA18" s="30" t="s">
         <v>207</v>
@@ -5671,13 +5679,13 @@
         <v>208</v>
       </c>
       <c r="AC18" s="30" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="AD18" s="30" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="AE18" s="65" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="19" spans="1:31" ht="57" x14ac:dyDescent="0.3">
@@ -5742,7 +5750,7 @@
         <v>4265136</v>
       </c>
       <c r="U19" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V19" s="26">
         <v>50.569000000000003</v>
@@ -5757,13 +5765,13 @@
         <v>104</v>
       </c>
       <c r="Z19" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA19" s="34" t="s">
         <v>105</v>
       </c>
       <c r="AB19" s="46" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="AC19" s="34" t="s">
         <v>105</v>
@@ -5783,10 +5791,10 @@
         <v>237</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>49</v>
@@ -5795,7 +5803,7 @@
         <v>235</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="H20" s="35">
         <v>2.11</v>
@@ -5852,7 +5860,7 @@
         <v>238</v>
       </c>
       <c r="Z20" s="34" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="AA20" s="34" t="s">
         <v>239</v>
@@ -5861,13 +5869,13 @@
         <v>240</v>
       </c>
       <c r="AC20" s="34" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="AD20" s="34" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="AE20" s="66" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="21" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5875,13 +5883,13 @@
         <v>126</v>
       </c>
       <c r="B21" s="54" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D21" s="34" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>52</v>
@@ -5920,10 +5928,10 @@
         <v>2025</v>
       </c>
       <c r="Q21" s="36" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="R21" s="36" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="S21" s="22" t="s">
         <v>122</v>
@@ -5932,7 +5940,7 @@
         <v>25400000</v>
       </c>
       <c r="U21" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V21" s="26">
         <v>41.352637812781921</v>
@@ -5944,25 +5952,25 @@
         <v>132</v>
       </c>
       <c r="Y21" s="30" t="s">
+        <v>440</v>
+      </c>
+      <c r="Z21" s="34" t="s">
+        <v>590</v>
+      </c>
+      <c r="AA21" s="34" t="s">
+        <v>304</v>
+      </c>
+      <c r="AB21" s="46" t="s">
         <v>442</v>
       </c>
-      <c r="Z21" s="34" t="s">
-        <v>592</v>
-      </c>
-      <c r="AA21" s="34" t="s">
-        <v>306</v>
-      </c>
-      <c r="AB21" s="46" t="s">
-        <v>444</v>
-      </c>
       <c r="AC21" s="34" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="AD21" s="34" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="AE21" s="65" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="22" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6039,25 +6047,25 @@
         <v>244</v>
       </c>
       <c r="Y22" s="29" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="Z22" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA22" s="30" t="s">
         <v>245</v>
       </c>
       <c r="AB22" s="46" t="s">
+        <v>443</v>
+      </c>
+      <c r="AC22" s="30" t="s">
+        <v>444</v>
+      </c>
+      <c r="AD22" s="30" t="s">
         <v>445</v>
       </c>
-      <c r="AC22" s="30" t="s">
-        <v>446</v>
-      </c>
-      <c r="AD22" s="30" t="s">
-        <v>447</v>
-      </c>
       <c r="AE22" s="64" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="23" spans="1:31" ht="136.80000000000001" x14ac:dyDescent="0.3">
@@ -6077,10 +6085,10 @@
         <v>57</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="H23" s="35">
         <v>0.56499999999999995</v>
@@ -6134,25 +6142,25 @@
         <v>95</v>
       </c>
       <c r="Y23" s="34" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="Z23" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA23" s="34" t="s">
         <v>233</v>
       </c>
       <c r="AB23" s="46" t="s">
+        <v>448</v>
+      </c>
+      <c r="AC23" s="34" t="s">
+        <v>449</v>
+      </c>
+      <c r="AD23" s="34" t="s">
         <v>450</v>
       </c>
-      <c r="AC23" s="34" t="s">
-        <v>451</v>
-      </c>
-      <c r="AD23" s="34" t="s">
-        <v>452</v>
-      </c>
       <c r="AE23" s="65" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="24" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6163,7 +6171,7 @@
         <v>179</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>219</v>
+        <v>358</v>
       </c>
       <c r="D24" s="34" t="s">
         <v>150</v>
@@ -6172,10 +6180,10 @@
         <v>42</v>
       </c>
       <c r="F24" s="71" t="s">
-        <v>460</v>
-      </c>
-      <c r="G24" s="71" t="s">
-        <v>461</v>
+        <v>458</v>
+      </c>
+      <c r="G24" s="72" t="s">
+        <v>459</v>
       </c>
       <c r="H24" s="35">
         <v>0.2</v>
@@ -6229,25 +6237,25 @@
         <v>180</v>
       </c>
       <c r="Y24" s="34" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="Z24" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA24" s="34" t="s">
         <v>181</v>
       </c>
       <c r="AB24" s="46" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="AC24" s="34" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="AD24" s="34" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="AE24" s="61" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="25" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -6267,10 +6275,10 @@
         <v>56</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="H25" s="35">
         <v>1</v>
@@ -6312,7 +6320,7 @@
         <v>216000000</v>
       </c>
       <c r="U25" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V25" s="26">
         <v>45.686354081466597</v>
@@ -6324,28 +6332,28 @@
         <v>244</v>
       </c>
       <c r="Y25" s="34" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="Z25" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA25" s="34" t="s">
         <v>252</v>
       </c>
       <c r="AB25" s="46" t="s">
+        <v>454</v>
+      </c>
+      <c r="AC25" s="34" t="s">
+        <v>455</v>
+      </c>
+      <c r="AD25" s="34" t="s">
         <v>456</v>
       </c>
-      <c r="AC25" s="34" t="s">
-        <v>457</v>
-      </c>
-      <c r="AD25" s="34" t="s">
-        <v>458</v>
-      </c>
       <c r="AE25" s="65" t="s">
-        <v>574</v>
-      </c>
-    </row>
-    <row r="26" spans="1:31" ht="45.6" x14ac:dyDescent="0.3">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="26" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
       <c r="A26" s="22" t="s">
         <v>87</v>
       </c>
@@ -6353,7 +6361,7 @@
         <v>259</v>
       </c>
       <c r="C26" s="34" t="s">
-        <v>219</v>
+        <v>595</v>
       </c>
       <c r="D26" s="34" t="s">
         <v>150</v>
@@ -6395,10 +6403,10 @@
         <v>2024</v>
       </c>
       <c r="Q26" s="36">
-        <v>2028</v>
+        <v>2030</v>
       </c>
       <c r="R26" s="36">
-        <v>2033</v>
+        <v>2040</v>
       </c>
       <c r="S26" s="22" t="s">
         <v>111</v>
@@ -6407,7 +6415,7 @@
         <v>40000000</v>
       </c>
       <c r="U26" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V26" s="22">
         <v>59.121267699503399</v>
@@ -6419,10 +6427,10 @@
         <v>244</v>
       </c>
       <c r="Y26" s="34" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="Z26" s="34" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="AA26" s="34" t="s">
         <v>261</v>
@@ -6431,13 +6439,13 @@
         <v>262</v>
       </c>
       <c r="AC26" s="34" t="s">
-        <v>263</v>
+        <v>593</v>
       </c>
       <c r="AD26" s="34" t="s">
-        <v>264</v>
-      </c>
-      <c r="AE26" s="61" t="s">
-        <v>571</v>
+        <v>594</v>
+      </c>
+      <c r="AE26" s="60" t="s">
+        <v>568</v>
       </c>
     </row>
     <row r="27" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -6448,7 +6456,7 @@
         <v>169</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="D27" s="30" t="s">
         <v>150</v>
@@ -6460,7 +6468,7 @@
         <v>170</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="H27" s="31">
         <v>0.23252429999999999</v>
@@ -6514,10 +6522,10 @@
         <v>95</v>
       </c>
       <c r="Y27" s="30" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="Z27" s="30" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="AA27" s="30" t="s">
         <v>171</v>
@@ -6526,13 +6534,13 @@
         <v>172</v>
       </c>
       <c r="AC27" s="30" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="AD27" s="30" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="AE27" s="61" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="28" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -6543,10 +6551,10 @@
         <v>146</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>54</v>
@@ -6609,25 +6617,25 @@
         <v>132</v>
       </c>
       <c r="Y28" s="30" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="Z28" s="30" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="AA28" s="30" t="s">
         <v>148</v>
       </c>
       <c r="AB28" s="46" t="s">
+        <v>469</v>
+      </c>
+      <c r="AC28" s="30" t="s">
+        <v>470</v>
+      </c>
+      <c r="AD28" s="30" t="s">
         <v>471</v>
       </c>
-      <c r="AC28" s="30" t="s">
-        <v>472</v>
-      </c>
-      <c r="AD28" s="30" t="s">
-        <v>473</v>
-      </c>
       <c r="AE28" s="60" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="29" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -6692,7 +6700,7 @@
         <v>228721666</v>
       </c>
       <c r="U29" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V29" s="24">
         <v>51.297800000000002</v>
@@ -6704,10 +6712,10 @@
         <v>180</v>
       </c>
       <c r="Y29" s="30" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="Z29" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA29" s="30" t="s">
         <v>198</v>
@@ -6716,13 +6724,13 @@
         <v>199</v>
       </c>
       <c r="AC29" s="30" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="AD29" s="30" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="AE29" s="60" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="30" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6730,22 +6738,22 @@
         <v>163</v>
       </c>
       <c r="B30" s="54" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="D30" s="34" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>58</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="H30" s="53">
         <v>4.5999999999999999E-2</v>
@@ -6787,7 +6795,7 @@
         <v>29500000</v>
       </c>
       <c r="U30" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V30" s="22">
         <v>60.618241659279597</v>
@@ -6799,25 +6807,25 @@
         <v>244</v>
       </c>
       <c r="Y30" s="34" t="s">
+        <v>498</v>
+      </c>
+      <c r="Z30" s="34" t="s">
+        <v>588</v>
+      </c>
+      <c r="AA30" s="34" t="s">
+        <v>314</v>
+      </c>
+      <c r="AB30" s="47" t="s">
         <v>500</v>
       </c>
-      <c r="Z30" s="34" t="s">
-        <v>590</v>
-      </c>
-      <c r="AA30" s="34" t="s">
-        <v>316</v>
-      </c>
-      <c r="AB30" s="47" t="s">
+      <c r="AC30" s="34" t="s">
+        <v>501</v>
+      </c>
+      <c r="AD30" s="34" t="s">
         <v>502</v>
       </c>
-      <c r="AC30" s="34" t="s">
-        <v>503</v>
-      </c>
-      <c r="AD30" s="34" t="s">
-        <v>504</v>
-      </c>
       <c r="AE30" s="61" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="31" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6882,7 +6890,7 @@
         <v>191000000</v>
       </c>
       <c r="U31" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V31" s="26">
         <v>51.618000000000002</v>
@@ -6897,7 +6905,7 @@
         <v>201</v>
       </c>
       <c r="Z31" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA31" s="34" t="s">
         <v>202</v>
@@ -6906,13 +6914,13 @@
         <v>203</v>
       </c>
       <c r="AC31" s="34" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="AD31" s="34" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="AE31" s="60" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="32" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6920,7 +6928,7 @@
         <v>87</v>
       </c>
       <c r="B32" s="54" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>108</v>
@@ -6932,10 +6940,10 @@
         <v>45</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="H32" s="35">
         <v>1</v>
@@ -6989,25 +6997,25 @@
         <v>95</v>
       </c>
       <c r="Y32" s="34" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="Z32" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA32" s="34" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="AB32" s="46" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="AC32" s="34" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="AD32" s="34" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="AE32" s="60" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="33" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7087,22 +7095,22 @@
         <v>112</v>
       </c>
       <c r="Z33" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA33" s="30" t="s">
         <v>113</v>
       </c>
       <c r="AB33" s="46" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="AC33" s="30" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="AD33" s="30" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="AE33" s="66" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="34" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7110,19 +7118,19 @@
         <v>87</v>
       </c>
       <c r="B34" s="55" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>89</v>
+        <v>225</v>
       </c>
       <c r="D34" s="30" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>52</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="G34" s="2"/>
       <c r="H34" s="31">
@@ -7165,7 +7173,7 @@
         <v>122900000</v>
       </c>
       <c r="U34" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V34" s="23">
         <v>43.151000000000003</v>
@@ -7177,25 +7185,25 @@
         <v>244</v>
       </c>
       <c r="Y34" s="30" t="s">
+        <v>480</v>
+      </c>
+      <c r="Z34" s="30" t="s">
+        <v>591</v>
+      </c>
+      <c r="AA34" s="30" t="s">
+        <v>293</v>
+      </c>
+      <c r="AB34" s="46" t="s">
+        <v>294</v>
+      </c>
+      <c r="AC34" s="30" t="s">
+        <v>481</v>
+      </c>
+      <c r="AD34" s="30" t="s">
         <v>482</v>
       </c>
-      <c r="Z34" s="30" t="s">
-        <v>593</v>
-      </c>
-      <c r="AA34" s="30" t="s">
-        <v>295</v>
-      </c>
-      <c r="AB34" s="46" t="s">
-        <v>296</v>
-      </c>
-      <c r="AC34" s="30" t="s">
-        <v>483</v>
-      </c>
-      <c r="AD34" s="30" t="s">
-        <v>484</v>
-      </c>
       <c r="AE34" s="64" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="35" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7206,10 +7214,10 @@
         <v>142</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>54</v>
@@ -7218,7 +7226,7 @@
         <v>143</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="H35" s="35">
         <v>0.28144999999999998</v>
@@ -7275,19 +7283,19 @@
         <v>144</v>
       </c>
       <c r="Z35" s="34" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="AA35" s="34" t="s">
         <v>145</v>
       </c>
       <c r="AB35" s="46" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="AC35" s="34" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="AD35" s="34" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="AE35" s="62" t="s">
         <v>27</v>
@@ -7301,7 +7309,7 @@
         <v>114</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="D36" s="34" t="s">
         <v>109</v>
@@ -7355,7 +7363,7 @@
         <v>159000000</v>
       </c>
       <c r="U36" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V36" s="26">
         <v>51.1339349</v>
@@ -7367,25 +7375,25 @@
         <v>95</v>
       </c>
       <c r="Y36" s="34" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="Z36" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA36" s="34" t="s">
         <v>118</v>
       </c>
       <c r="AB36" s="46" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="AC36" s="34" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="AD36" s="34" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="AE36" s="60" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="37" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7393,22 +7401,22 @@
         <v>163</v>
       </c>
       <c r="B37" s="54" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>45</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="H37" s="53">
         <v>5.0046999999999999E-3</v>
@@ -7450,7 +7458,7 @@
         <v>26498650</v>
       </c>
       <c r="U37" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V37" s="26">
         <v>50.529000000000003</v>
@@ -7462,25 +7470,25 @@
         <v>95</v>
       </c>
       <c r="Y37" s="34" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="Z37" s="34" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="AA37" s="34" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="AB37" s="46" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="AC37" s="34" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="AD37" s="34" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="AE37" s="60" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="38" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7488,7 +7496,7 @@
         <v>87</v>
       </c>
       <c r="B38" s="54" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>108</v>
@@ -7545,7 +7553,7 @@
         <v>234000000</v>
       </c>
       <c r="U38" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V38" s="26">
         <v>38.129899999999999</v>
@@ -7557,25 +7565,25 @@
         <v>95</v>
       </c>
       <c r="Y38" s="34" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="Z38" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA38" s="34" t="s">
         <v>217</v>
       </c>
       <c r="AB38" s="46" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="AC38" s="34" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="AD38" s="34" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="AE38" s="61" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="39" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7583,10 +7591,10 @@
         <v>141</v>
       </c>
       <c r="B39" s="55" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="D39" s="34" t="s">
         <v>109</v>
@@ -7595,7 +7603,7 @@
         <v>58</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="G39" s="2"/>
       <c r="H39" s="31">
@@ -7650,25 +7658,25 @@
         <v>180</v>
       </c>
       <c r="Y39" s="30" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="Z39" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA39" s="30" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="AB39" s="46" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="AC39" s="30" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="AD39" s="30" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="AE39" s="61" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="40" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7682,7 +7690,7 @@
         <v>219</v>
       </c>
       <c r="D40" s="30" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>50</v>
@@ -7733,7 +7741,7 @@
         <v>127000000</v>
       </c>
       <c r="U40" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V40" s="24">
         <v>37.916800000000002</v>
@@ -7748,7 +7756,7 @@
         <v>221</v>
       </c>
       <c r="Z40" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA40" s="30" t="s">
         <v>222</v>
@@ -7757,13 +7765,13 @@
         <v>223</v>
       </c>
       <c r="AC40" s="30" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="AD40" s="30" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="AE40" s="64" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="41" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -7843,22 +7851,22 @@
         <v>96</v>
       </c>
       <c r="Z41" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA41" s="30" t="s">
         <v>97</v>
       </c>
       <c r="AB41" s="46" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="AC41" s="30" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="AD41" s="30" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="AE41" s="66" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="42" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -7923,7 +7931,7 @@
         <v>117000000</v>
       </c>
       <c r="U42" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V42" s="26">
         <v>44.968299999999999</v>
@@ -7938,22 +7946,22 @@
         <v>136</v>
       </c>
       <c r="Z42" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA42" s="34" t="s">
         <v>134</v>
       </c>
       <c r="AB42" s="46" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="AC42" s="34" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="AD42" s="34" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="AE42" s="60" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="43" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7961,13 +7969,13 @@
         <v>87</v>
       </c>
       <c r="B43" s="54" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="D43" s="30" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>43</v>
@@ -8018,7 +8026,7 @@
         <v>118000000</v>
       </c>
       <c r="U43" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V43" s="26">
         <v>51.976999999999997</v>
@@ -8033,22 +8041,22 @@
         <v>258</v>
       </c>
       <c r="Z43" s="34" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="AA43" s="34" t="s">
         <v>92</v>
       </c>
       <c r="AB43" s="47" t="s">
+        <v>379</v>
+      </c>
+      <c r="AC43" s="34" t="s">
+        <v>380</v>
+      </c>
+      <c r="AD43" s="34" t="s">
         <v>381</v>
       </c>
-      <c r="AC43" s="34" t="s">
-        <v>382</v>
-      </c>
-      <c r="AD43" s="34" t="s">
-        <v>383</v>
-      </c>
       <c r="AE43" s="60" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="44" spans="1:31" ht="68.400000000000006" x14ac:dyDescent="0.3">
@@ -8113,7 +8121,7 @@
         <v>36000000</v>
       </c>
       <c r="U44" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V44" s="26">
         <v>50.406342306737002</v>
@@ -8125,25 +8133,25 @@
         <v>95</v>
       </c>
       <c r="Y44" s="34" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="Z44" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA44" s="34" t="s">
         <v>129</v>
       </c>
       <c r="AB44" s="46" t="s">
+        <v>504</v>
+      </c>
+      <c r="AC44" s="34" t="s">
+        <v>505</v>
+      </c>
+      <c r="AD44" s="34" t="s">
         <v>506</v>
       </c>
-      <c r="AC44" s="34" t="s">
-        <v>507</v>
-      </c>
-      <c r="AD44" s="34" t="s">
-        <v>508</v>
-      </c>
       <c r="AE44" s="60" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="45" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -8151,19 +8159,19 @@
         <v>163</v>
       </c>
       <c r="B45" s="54" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="D45" s="34" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>46</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="G45" s="4" t="s">
         <v>92</v>
@@ -8208,7 +8216,7 @@
         <v>13000000</v>
       </c>
       <c r="U45" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V45" s="22">
         <v>59.2181</v>
@@ -8220,25 +8228,25 @@
         <v>244</v>
       </c>
       <c r="Y45" s="34" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="Z45" s="34" t="s">
         <v>225</v>
       </c>
       <c r="AA45" s="34" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="AB45" s="46" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="AC45" s="34" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="AD45" s="34" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="AE45" s="64" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="46" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8318,22 +8326,22 @@
         <v>214</v>
       </c>
       <c r="Z46" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA46" s="30" t="s">
         <v>215</v>
       </c>
       <c r="AB46" s="46" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="AC46" s="30" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="AD46" s="30" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="AE46" s="64" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="47" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8344,7 +8352,7 @@
         <v>153</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>219</v>
+        <v>358</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>150</v>
@@ -8353,10 +8361,10 @@
         <v>55</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="H47" s="52">
         <v>1.55E-2</v>
@@ -8413,22 +8421,22 @@
         <v>154</v>
       </c>
       <c r="Z47" s="30" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="AA47" s="30" t="s">
         <v>155</v>
       </c>
       <c r="AB47" s="46" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="AC47" s="30" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="AD47" s="30" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="AE47" s="65" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="48" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -8436,7 +8444,7 @@
         <v>87</v>
       </c>
       <c r="B48" s="54" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>89</v>
@@ -8448,10 +8456,10 @@
         <v>58</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="H48" s="35">
         <v>0.40600000000000003</v>
@@ -8493,7 +8501,7 @@
         <v>97000000</v>
       </c>
       <c r="U48" s="37" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="V48" s="22">
         <v>58.099057767351503</v>
@@ -8505,25 +8513,25 @@
         <v>244</v>
       </c>
       <c r="Y48" s="34" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="Z48" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA48" s="34" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="AB48" s="47" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="AC48" s="34" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="AD48" s="34" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="AE48" s="61" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="49" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -8543,10 +8551,10 @@
         <v>54</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="H49" s="53">
         <v>6.7077999999999999E-2</v>
@@ -8588,7 +8596,7 @@
         <v>40000000</v>
       </c>
       <c r="U49" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V49" s="26">
         <v>56.787056035485499</v>
@@ -8603,22 +8611,22 @@
         <v>151</v>
       </c>
       <c r="Z49" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA49" s="34" t="s">
         <v>152</v>
       </c>
       <c r="AB49" s="46" t="s">
+        <v>520</v>
+      </c>
+      <c r="AC49" s="34" t="s">
+        <v>521</v>
+      </c>
+      <c r="AD49" s="34" t="s">
         <v>522</v>
       </c>
-      <c r="AC49" s="34" t="s">
-        <v>523</v>
-      </c>
-      <c r="AD49" s="34" t="s">
-        <v>524</v>
-      </c>
       <c r="AE49" s="64" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="50" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -8632,7 +8640,7 @@
         <v>225</v>
       </c>
       <c r="D50" s="34" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>48</v>
@@ -8671,7 +8679,7 @@
         <v>19458418</v>
       </c>
       <c r="U50" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V50" s="26">
         <v>48.096166502584701</v>
@@ -8683,7 +8691,7 @@
         <v>132</v>
       </c>
       <c r="Y50" s="34" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="Z50" s="34" t="s">
         <v>225</v>
@@ -8692,16 +8700,16 @@
         <v>211</v>
       </c>
       <c r="AB50" s="46" t="s">
+        <v>524</v>
+      </c>
+      <c r="AC50" s="34" t="s">
+        <v>525</v>
+      </c>
+      <c r="AD50" s="34" t="s">
         <v>526</v>
       </c>
-      <c r="AC50" s="34" t="s">
-        <v>527</v>
-      </c>
-      <c r="AD50" s="34" t="s">
-        <v>528</v>
-      </c>
       <c r="AE50" s="65" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="51" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -8712,7 +8720,7 @@
         <v>182</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="D51" s="30" t="s">
         <v>150</v>
@@ -8721,10 +8729,10 @@
         <v>42</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="G51" s="30" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="H51" s="31">
         <v>0.27411429999999998</v>
@@ -8778,25 +8786,25 @@
         <v>132</v>
       </c>
       <c r="Y51" s="30" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="Z51" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA51" s="30" t="s">
         <v>184</v>
       </c>
       <c r="AB51" s="46" t="s">
+        <v>528</v>
+      </c>
+      <c r="AC51" s="30" t="s">
+        <v>529</v>
+      </c>
+      <c r="AD51" s="30" t="s">
         <v>530</v>
       </c>
-      <c r="AC51" s="30" t="s">
-        <v>531</v>
-      </c>
-      <c r="AD51" s="30" t="s">
-        <v>532</v>
-      </c>
       <c r="AE51" s="65" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="52" spans="1:31" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -8861,7 +8869,7 @@
         <v>88286266</v>
       </c>
       <c r="U52" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V52" s="26">
         <v>60.306100000000001</v>
@@ -8876,7 +8884,7 @@
         <v>158</v>
       </c>
       <c r="Z52" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA52" s="34" t="s">
         <v>159</v>
@@ -8891,7 +8899,7 @@
         <v>162</v>
       </c>
       <c r="AE52" s="66" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="53" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8902,7 +8910,7 @@
         <v>234</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>109</v>
@@ -8914,7 +8922,7 @@
         <v>235</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H53" s="31">
         <v>1.72E-2</v>
@@ -8956,7 +8964,7 @@
         <v>3867988</v>
       </c>
       <c r="U53" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V53" s="24">
         <v>64.037112316635401</v>
@@ -8968,22 +8976,22 @@
         <v>95</v>
       </c>
       <c r="Y53" s="30" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="Z53" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA53" s="30" t="s">
         <v>236</v>
       </c>
       <c r="AB53" s="46" t="s">
+        <v>535</v>
+      </c>
+      <c r="AC53" s="30" t="s">
         <v>537</v>
       </c>
-      <c r="AC53" s="30" t="s">
-        <v>539</v>
-      </c>
       <c r="AD53" s="30" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="AE53" s="67" t="s">
         <v>29</v>
@@ -8994,22 +9002,22 @@
         <v>163</v>
       </c>
       <c r="B54" s="55" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>219</v>
+        <v>596</v>
       </c>
       <c r="D54" s="30" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>46</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="G54" s="30" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="H54" s="31">
         <v>0.16981750000000001</v>
@@ -9051,7 +9059,7 @@
         <v>40000000</v>
       </c>
       <c r="U54" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V54" s="24">
         <v>59.127044152710397</v>
@@ -9063,25 +9071,25 @@
         <v>132</v>
       </c>
       <c r="Y54" s="30" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="Z54" s="30" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA54" s="30" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="AB54" s="46" t="s">
+        <v>541</v>
+      </c>
+      <c r="AC54" s="30" t="s">
+        <v>542</v>
+      </c>
+      <c r="AD54" s="30" t="s">
         <v>543</v>
       </c>
-      <c r="AC54" s="30" t="s">
-        <v>544</v>
-      </c>
-      <c r="AD54" s="30" t="s">
-        <v>545</v>
-      </c>
       <c r="AE54" s="65" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="55" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -9089,22 +9097,22 @@
         <v>87</v>
       </c>
       <c r="B55" s="55" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="D55" s="30" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>46</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="H55" s="31">
         <v>4.2</v>
@@ -9146,7 +9154,7 @@
         <v>225000000</v>
       </c>
       <c r="U55" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V55" s="23">
         <v>57.788622470324199</v>
@@ -9158,23 +9166,23 @@
         <v>132</v>
       </c>
       <c r="Y55" s="30" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="Z55" s="30" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="AA55" s="30"/>
       <c r="AB55" s="46" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="AC55" s="30" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="AD55" s="30" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="AE55" s="60" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="56" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -9185,7 +9193,7 @@
         <v>190</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>219</v>
+        <v>108</v>
       </c>
       <c r="D56" s="30" t="s">
         <v>150</v>
@@ -9194,10 +9202,10 @@
         <v>42</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="H56" s="31">
         <v>0.17</v>
@@ -9251,25 +9259,25 @@
         <v>95</v>
       </c>
       <c r="Y56" s="30" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="Z56" s="30" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="AA56" s="30" t="s">
         <v>191</v>
       </c>
       <c r="AB56" s="46" t="s">
+        <v>550</v>
+      </c>
+      <c r="AC56" s="30" t="s">
+        <v>551</v>
+      </c>
+      <c r="AD56" s="30" t="s">
         <v>552</v>
       </c>
-      <c r="AC56" s="30" t="s">
-        <v>553</v>
-      </c>
-      <c r="AD56" s="30" t="s">
-        <v>554</v>
-      </c>
       <c r="AE56" s="64" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="57" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -9277,22 +9285,22 @@
         <v>87</v>
       </c>
       <c r="B57" s="55" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="D57" s="30" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>52</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="H57" s="31">
         <v>2</v>
@@ -9334,7 +9342,7 @@
         <v>205061582</v>
       </c>
       <c r="U57" s="33" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V57" s="24">
         <v>40.8482802817337</v>
@@ -9346,25 +9354,25 @@
         <v>132</v>
       </c>
       <c r="Y57" s="30" t="s">
+        <v>554</v>
+      </c>
+      <c r="Z57" s="30" t="s">
+        <v>592</v>
+      </c>
+      <c r="AA57" s="30" t="s">
+        <v>301</v>
+      </c>
+      <c r="AB57" s="25" t="s">
+        <v>302</v>
+      </c>
+      <c r="AC57" s="30" t="s">
+        <v>555</v>
+      </c>
+      <c r="AD57" s="30" t="s">
         <v>556</v>
       </c>
-      <c r="Z57" s="30" t="s">
-        <v>594</v>
-      </c>
-      <c r="AA57" s="30" t="s">
-        <v>303</v>
-      </c>
-      <c r="AB57" s="25" t="s">
-        <v>304</v>
-      </c>
-      <c r="AC57" s="30" t="s">
-        <v>557</v>
-      </c>
-      <c r="AD57" s="30" t="s">
-        <v>558</v>
-      </c>
       <c r="AE57" s="60" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="58" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -9375,10 +9383,10 @@
         <v>228</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>89</v>
+        <v>225</v>
       </c>
       <c r="D58" s="34" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>50</v>
@@ -9441,7 +9449,7 @@
         <v>132</v>
       </c>
       <c r="Y58" s="30" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="Z58" s="30" t="s">
         <v>225</v>
@@ -9450,16 +9458,16 @@
         <v>230</v>
       </c>
       <c r="AB58" s="46" t="s">
+        <v>564</v>
+      </c>
+      <c r="AC58" s="30" t="s">
+        <v>565</v>
+      </c>
+      <c r="AD58" s="30" t="s">
         <v>566</v>
       </c>
-      <c r="AC58" s="30" t="s">
-        <v>567</v>
-      </c>
-      <c r="AD58" s="30" t="s">
+      <c r="AE58" s="60" t="s">
         <v>568</v>
-      </c>
-      <c r="AE58" s="60" t="s">
-        <v>570</v>
       </c>
     </row>
     <row r="59" spans="1:31" ht="68.400000000000006" x14ac:dyDescent="0.3">
@@ -9467,10 +9475,10 @@
         <v>87</v>
       </c>
       <c r="B59" s="54" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>219</v>
+        <v>358</v>
       </c>
       <c r="D59" s="34" t="s">
         <v>150</v>
@@ -9479,10 +9487,10 @@
         <v>52</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="H59" s="53">
         <v>8.5999999999999993E-2</v>
@@ -9536,25 +9544,25 @@
         <v>244</v>
       </c>
       <c r="Y59" s="34" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="Z59" s="34" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="AA59" s="34" t="s">
+        <v>297</v>
+      </c>
+      <c r="AB59" s="27" t="s">
+        <v>298</v>
+      </c>
+      <c r="AC59" s="34" t="s">
+        <v>558</v>
+      </c>
+      <c r="AD59" s="34" t="s">
         <v>299</v>
       </c>
-      <c r="AB59" s="27" t="s">
-        <v>300</v>
-      </c>
-      <c r="AC59" s="34" t="s">
-        <v>560</v>
-      </c>
-      <c r="AD59" s="34" t="s">
-        <v>301</v>
-      </c>
       <c r="AE59" s="61" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="60" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -9634,22 +9642,22 @@
         <v>187</v>
       </c>
       <c r="Z60" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AA60" s="34" t="s">
         <v>188</v>
       </c>
       <c r="AB60" s="46" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="AC60" s="34" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="AD60" s="34" t="s">
         <v>189</v>
       </c>
       <c r="AE60" s="60" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="61" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -9657,22 +9665,22 @@
         <v>126</v>
       </c>
       <c r="B61" s="54" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C61" s="2" t="s">
         <v>242</v>
       </c>
       <c r="D61" s="34" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="E61" s="4" t="s">
         <v>46</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="H61" s="35">
         <v>0.1</v>
@@ -9714,7 +9722,7 @@
         <v>26200000</v>
       </c>
       <c r="U61" s="37" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="V61" s="26">
         <v>60.45333865137971</v>
@@ -9726,33 +9734,29 @@
         <v>244</v>
       </c>
       <c r="Y61" s="34" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="Z61" s="34" t="s">
         <v>225</v>
       </c>
       <c r="AA61" s="34" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="AB61" s="46" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="AC61" s="34" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="AD61" s="34" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="AE61" s="65" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AE61" xr:uid="{00000000-0009-0000-0000-000001000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AE61">
-      <sortCondition ref="B1:B61"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:AE61" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <hyperlinks>
     <hyperlink ref="AB2" r:id="rId1" xr:uid="{732997D1-2192-49C8-AD3C-37FF6D9C50FB}"/>
     <hyperlink ref="AB3" r:id="rId2" xr:uid="{6D3D26FD-6440-42D0-915E-7DC5B096846A}"/>
@@ -9822,314 +9826,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D4FF1D5-A91D-4300-B515-F6FD45A4A36E}">
-  <dimension ref="A1:A60"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" s="40">
-        <v>1.4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31">
-        <v>0.112</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="41" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="35" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" s="31">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" s="40">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" s="41" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" s="40">
-        <v>0.78300000000000003</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" s="52">
-        <v>7.6649999999999999E-3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" s="41">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" s="41">
-        <v>0.57999999999999996</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" s="41">
-        <v>6.4000000000000001E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A14" s="41">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A15" s="40">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A16" s="51">
-        <v>4.5999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" s="40">
-        <v>1.3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" s="41">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A19" s="41" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A20" s="41" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A21" s="40">
-        <v>1.2999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A22" s="41">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A23" s="41">
-        <v>0.35</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A24" s="41">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A25" s="41" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A26" s="40">
-        <v>0.19500000000000001</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A27" s="40">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A28" s="40">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A29" s="41">
-        <v>0.16</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A30" s="41">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A31" s="41">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A32" s="40">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A33" s="40">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" s="41" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A35" s="41" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A36" s="41" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A37" s="41">
-        <v>1.9</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A38" s="40">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A39" s="40">
-        <v>0.85</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A40" s="40">
-        <v>1.4</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A41" s="41">
-        <v>0.36599999999999999</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A42" s="41" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A43" s="41">
-        <v>7.0000000000000007E-2</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A44" s="41" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A45" s="40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="40" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A47" s="41" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A48" s="41" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="41"/>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A50" s="57">
-        <v>0.33400000000000002</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A51" s="41">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A52" s="40">
-        <v>3.4000000000000002E-2</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A53" s="40">
-        <v>0.126</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A54" s="40" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A55" s="40">
-        <v>0.16</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A56" s="40" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A57" s="40" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A58" s="41">
-        <v>5.6000000000000001E-2</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A59" s="41">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A60" s="41" t="s">
-        <v>92</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor rgb="FF888888"/>
@@ -10144,151 +9840,151 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="86" t="s">
+      <c r="A1" s="87" t="s">
+        <v>315</v>
+      </c>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="73" t="s">
+        <v>316</v>
+      </c>
+      <c r="B3" s="74"/>
+      <c r="C3" s="74"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
+    </row>
+    <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="93" t="s">
         <v>317</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="72" t="s">
+      <c r="B4" s="77"/>
+      <c r="C4" s="82" t="s">
         <v>318</v>
       </c>
-      <c r="B3" s="73"/>
-      <c r="C3" s="73"/>
-      <c r="D3" s="73"/>
-      <c r="E3" s="73"/>
-    </row>
-    <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="92" t="s">
+      <c r="D4" s="74"/>
+      <c r="E4" s="74"/>
+    </row>
+    <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="90" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="77"/>
+      <c r="C5" s="82" t="s">
         <v>319</v>
       </c>
-      <c r="B4" s="76"/>
-      <c r="C4" s="81" t="s">
+      <c r="D5" s="74"/>
+      <c r="E5" s="74"/>
+    </row>
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="88" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="77"/>
+      <c r="C6" s="82" t="s">
         <v>320</v>
       </c>
-      <c r="D4" s="73"/>
-      <c r="E4" s="73"/>
-    </row>
-    <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="89" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="76"/>
-      <c r="C5" s="81" t="s">
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
+    </row>
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="89" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="77"/>
+      <c r="C7" s="82" t="s">
         <v>321</v>
       </c>
-      <c r="D5" s="73"/>
-      <c r="E5" s="73"/>
-    </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="87" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="76"/>
-      <c r="C6" s="81" t="s">
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
+    </row>
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="92" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="77"/>
+      <c r="C8" s="82" t="s">
         <v>322</v>
       </c>
-      <c r="D6" s="73"/>
-      <c r="E6" s="73"/>
-    </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="88" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="76"/>
-      <c r="C7" s="81" t="s">
+      <c r="D8" s="74"/>
+      <c r="E8" s="74"/>
+    </row>
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="85" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="77"/>
+      <c r="C9" s="82" t="s">
         <v>323</v>
       </c>
-      <c r="D7" s="73"/>
-      <c r="E7" s="73"/>
-    </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="91" t="s">
-        <v>35</v>
-      </c>
-      <c r="B8" s="76"/>
-      <c r="C8" s="81" t="s">
+      <c r="D9" s="74"/>
+      <c r="E9" s="74"/>
+    </row>
+    <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="83" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="77"/>
+      <c r="C10" s="82" t="s">
         <v>324</v>
       </c>
-      <c r="D8" s="73"/>
-      <c r="E8" s="73"/>
-    </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="84" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" s="76"/>
-      <c r="C9" s="81" t="s">
+      <c r="D10" s="74"/>
+      <c r="E10" s="74"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="73" t="s">
         <v>325</v>
       </c>
-      <c r="D9" s="73"/>
-      <c r="E9" s="73"/>
-    </row>
-    <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="82" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="76"/>
-      <c r="C10" s="81" t="s">
+      <c r="B12" s="74"/>
+      <c r="C12" s="74"/>
+      <c r="D12" s="74"/>
+      <c r="E12" s="74"/>
+    </row>
+    <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="84" t="s">
         <v>326</v>
       </c>
-      <c r="D10" s="73"/>
-      <c r="E10" s="73"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="72" t="s">
+      <c r="B13" s="77"/>
+      <c r="C13" s="82" t="s">
         <v>327</v>
       </c>
-      <c r="B12" s="73"/>
-      <c r="C12" s="73"/>
-      <c r="D12" s="73"/>
-      <c r="E12" s="73"/>
-    </row>
-    <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="83" t="s">
+      <c r="D13" s="74"/>
+      <c r="E13" s="74"/>
+    </row>
+    <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="91" t="s">
         <v>328</v>
       </c>
-      <c r="B13" s="76"/>
-      <c r="C13" s="81" t="s">
+      <c r="B14" s="77"/>
+      <c r="C14" s="82" t="s">
         <v>329</v>
       </c>
-      <c r="D13" s="73"/>
-      <c r="E13" s="73"/>
-    </row>
-    <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="90" t="s">
+      <c r="D14" s="74"/>
+      <c r="E14" s="74"/>
+    </row>
+    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="86" t="s">
         <v>330</v>
       </c>
-      <c r="B14" s="76"/>
-      <c r="C14" s="81" t="s">
+      <c r="B15" s="77"/>
+      <c r="C15" s="82" t="s">
         <v>331</v>
       </c>
-      <c r="D14" s="73"/>
-      <c r="E14" s="73"/>
-    </row>
-    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="85" t="s">
-        <v>332</v>
-      </c>
-      <c r="B15" s="76"/>
-      <c r="C15" s="81" t="s">
-        <v>333</v>
-      </c>
-      <c r="D15" s="73"/>
-      <c r="E15" s="73"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="74"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="43" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="42"/>
       <c r="B19" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modified:   excel_data/Innovation_Fund_Projects_data - 130426.xlsx 	modified:   public/data/projects.json
</commit_message>
<xml_diff>
--- a/excel_data/Innovation_Fund_Projects_data - 130426.xlsx
+++ b/excel_data/Innovation_Fund_Projects_data - 130426.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zeplatform-my.sharepoint.com/personal/salman_muhammad_zeplatform_eu/Documents/Technical/IF mapping tool/if-map/excel_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1784" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE9D5AE8-4961-471E-AC0D-44C6E1046072}"/>
+  <xr:revisionPtr revIDLastSave="1785" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{334CC654-21D2-4062-9E5A-3DCAF21C241F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1462,9 +1462,6 @@
     <t>DREAM</t>
   </si>
   <si>
-    <t>Decarbonisation of the Rezzato and Mazzano cement plant</t>
-  </si>
-  <si>
     <t>CFCPILOT4CCS</t>
   </si>
   <si>
@@ -2499,6 +2496,9 @@
   </si>
   <si>
     <t>Via Gardesana, 84, 25086 Rezzato BS, Italy</t>
+  </si>
+  <si>
+    <t>Decarbonisation of the Rezzato and Mazzano cement plant in taly</t>
   </si>
 </sst>
 </file>
@@ -3082,27 +3082,36 @@
     <xf numFmtId="0" fontId="3" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3124,15 +3133,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3454,40 +3454,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="79" t="s">
+      <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
+      <c r="F1" s="74"/>
+      <c r="G1" s="74"/>
+      <c r="H1" s="74"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="76"/>
-      <c r="C2" s="76"/>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="76"/>
+      <c r="B2" s="74"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="74"/>
+      <c r="G2" s="74"/>
+      <c r="H2" s="74"/>
     </row>
     <row r="4" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="78" t="s">
+      <c r="A4" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="76"/>
-      <c r="C4" s="76"/>
-      <c r="D4" s="76"/>
-      <c r="E4" s="76"/>
-      <c r="F4" s="76"/>
-      <c r="G4" s="76"/>
-      <c r="H4" s="76"/>
+      <c r="B4" s="74"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="74"/>
+      <c r="F4" s="74"/>
+      <c r="G4" s="74"/>
+      <c r="H4" s="74"/>
     </row>
     <row r="5" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3504,12 +3504,12 @@
       <c r="B6" s="3">
         <v>62</v>
       </c>
-      <c r="C6" s="76"/>
-      <c r="D6" s="76"/>
-      <c r="E6" s="76"/>
-      <c r="F6" s="76"/>
-      <c r="G6" s="76"/>
-      <c r="H6" s="76"/>
+      <c r="C6" s="74"/>
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="74"/>
+      <c r="G6" s="74"/>
+      <c r="H6" s="74"/>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
@@ -3518,12 +3518,12 @@
       <c r="B7" s="5">
         <v>16</v>
       </c>
-      <c r="C7" s="76"/>
-      <c r="D7" s="76"/>
-      <c r="E7" s="76"/>
-      <c r="F7" s="76"/>
-      <c r="G7" s="76"/>
-      <c r="H7" s="76"/>
+      <c r="C7" s="74"/>
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
+      <c r="F7" s="74"/>
+      <c r="G7" s="74"/>
+      <c r="H7" s="74"/>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -3532,12 +3532,12 @@
       <c r="B8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="76"/>
-      <c r="D8" s="76"/>
-      <c r="E8" s="76"/>
-      <c r="F8" s="76"/>
-      <c r="G8" s="76"/>
-      <c r="H8" s="76"/>
+      <c r="C8" s="74"/>
+      <c r="D8" s="74"/>
+      <c r="E8" s="74"/>
+      <c r="F8" s="74"/>
+      <c r="G8" s="74"/>
+      <c r="H8" s="74"/>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
@@ -3546,12 +3546,12 @@
       <c r="B9" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="76"/>
-      <c r="D9" s="76"/>
-      <c r="E9" s="76"/>
-      <c r="F9" s="76"/>
-      <c r="G9" s="76"/>
-      <c r="H9" s="76"/>
+      <c r="C9" s="74"/>
+      <c r="D9" s="74"/>
+      <c r="E9" s="74"/>
+      <c r="F9" s="74"/>
+      <c r="G9" s="74"/>
+      <c r="H9" s="74"/>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -3560,12 +3560,12 @@
       <c r="B10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="76"/>
-      <c r="D10" s="76"/>
-      <c r="E10" s="76"/>
-      <c r="F10" s="76"/>
-      <c r="G10" s="76"/>
-      <c r="H10" s="76"/>
+      <c r="C10" s="74"/>
+      <c r="D10" s="74"/>
+      <c r="E10" s="74"/>
+      <c r="F10" s="74"/>
+      <c r="G10" s="74"/>
+      <c r="H10" s="74"/>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
@@ -3574,12 +3574,12 @@
       <c r="B11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="76"/>
-      <c r="D11" s="76"/>
-      <c r="E11" s="76"/>
-      <c r="F11" s="76"/>
-      <c r="G11" s="76"/>
-      <c r="H11" s="76"/>
+      <c r="C11" s="74"/>
+      <c r="D11" s="74"/>
+      <c r="E11" s="74"/>
+      <c r="F11" s="74"/>
+      <c r="G11" s="74"/>
+      <c r="H11" s="74"/>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
@@ -3588,24 +3588,24 @@
       <c r="B12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="76"/>
-      <c r="D12" s="76"/>
-      <c r="E12" s="76"/>
-      <c r="F12" s="76"/>
-      <c r="G12" s="76"/>
-      <c r="H12" s="76"/>
+      <c r="C12" s="74"/>
+      <c r="D12" s="74"/>
+      <c r="E12" s="74"/>
+      <c r="F12" s="74"/>
+      <c r="G12" s="74"/>
+      <c r="H12" s="74"/>
     </row>
     <row r="15" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="78" t="s">
+      <c r="A15" s="73" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="76"/>
-      <c r="C15" s="76"/>
-      <c r="D15" s="76"/>
-      <c r="E15" s="76"/>
-      <c r="F15" s="76"/>
-      <c r="G15" s="76"/>
-      <c r="H15" s="76"/>
+      <c r="B15" s="74"/>
+      <c r="C15" s="74"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="74"/>
+      <c r="F15" s="74"/>
+      <c r="G15" s="74"/>
+      <c r="H15" s="74"/>
     </row>
     <row r="16" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -3617,11 +3617,11 @@
       <c r="C16" s="80" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="74"/>
-      <c r="E16" s="74"/>
-      <c r="F16" s="74"/>
-      <c r="G16" s="74"/>
-      <c r="H16" s="75"/>
+      <c r="D16" s="76"/>
+      <c r="E16" s="76"/>
+      <c r="F16" s="76"/>
+      <c r="G16" s="76"/>
+      <c r="H16" s="77"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
@@ -3630,14 +3630,14 @@
       <c r="B17" s="9">
         <v>21</v>
       </c>
-      <c r="C17" s="73" t="s">
+      <c r="C17" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="74"/>
-      <c r="E17" s="74"/>
-      <c r="F17" s="74"/>
-      <c r="G17" s="74"/>
-      <c r="H17" s="75"/>
+      <c r="D17" s="76"/>
+      <c r="E17" s="76"/>
+      <c r="F17" s="76"/>
+      <c r="G17" s="76"/>
+      <c r="H17" s="77"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
@@ -3646,14 +3646,14 @@
       <c r="B18" s="11">
         <v>20</v>
       </c>
-      <c r="C18" s="77" t="s">
+      <c r="C18" s="79" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="74"/>
-      <c r="E18" s="74"/>
-      <c r="F18" s="74"/>
-      <c r="G18" s="74"/>
-      <c r="H18" s="75"/>
+      <c r="D18" s="76"/>
+      <c r="E18" s="76"/>
+      <c r="F18" s="76"/>
+      <c r="G18" s="76"/>
+      <c r="H18" s="77"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -3662,14 +3662,14 @@
       <c r="B19" s="13">
         <v>10</v>
       </c>
-      <c r="C19" s="73" t="s">
+      <c r="C19" s="75" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="74"/>
-      <c r="E19" s="74"/>
-      <c r="F19" s="74"/>
-      <c r="G19" s="74"/>
-      <c r="H19" s="75"/>
+      <c r="D19" s="76"/>
+      <c r="E19" s="76"/>
+      <c r="F19" s="76"/>
+      <c r="G19" s="76"/>
+      <c r="H19" s="77"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
@@ -3678,14 +3678,14 @@
       <c r="B20" s="15">
         <v>4</v>
       </c>
-      <c r="C20" s="77" t="s">
+      <c r="C20" s="79" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="74"/>
-      <c r="E20" s="74"/>
-      <c r="F20" s="74"/>
-      <c r="G20" s="74"/>
-      <c r="H20" s="75"/>
+      <c r="D20" s="76"/>
+      <c r="E20" s="76"/>
+      <c r="F20" s="76"/>
+      <c r="G20" s="76"/>
+      <c r="H20" s="77"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
@@ -3694,14 +3694,14 @@
       <c r="B21" s="17">
         <v>3</v>
       </c>
-      <c r="C21" s="73" t="s">
+      <c r="C21" s="75" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="74"/>
-      <c r="E21" s="74"/>
-      <c r="F21" s="74"/>
-      <c r="G21" s="74"/>
-      <c r="H21" s="75"/>
+      <c r="D21" s="76"/>
+      <c r="E21" s="76"/>
+      <c r="F21" s="76"/>
+      <c r="G21" s="76"/>
+      <c r="H21" s="77"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="16" t="s">
@@ -3710,14 +3710,14 @@
       <c r="B22" s="17">
         <v>1</v>
       </c>
-      <c r="C22" s="77" t="s">
+      <c r="C22" s="79" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="74"/>
-      <c r="E22" s="74"/>
-      <c r="F22" s="74"/>
-      <c r="G22" s="74"/>
-      <c r="H22" s="75"/>
+      <c r="D22" s="76"/>
+      <c r="E22" s="76"/>
+      <c r="F22" s="76"/>
+      <c r="G22" s="76"/>
+      <c r="H22" s="77"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="16" t="s">
@@ -3726,14 +3726,14 @@
       <c r="B23" s="17">
         <v>1</v>
       </c>
-      <c r="C23" s="73" t="s">
+      <c r="C23" s="75" t="s">
         <v>34</v>
       </c>
-      <c r="D23" s="74"/>
-      <c r="E23" s="74"/>
-      <c r="F23" s="74"/>
-      <c r="G23" s="74"/>
-      <c r="H23" s="75"/>
+      <c r="D23" s="76"/>
+      <c r="E23" s="76"/>
+      <c r="F23" s="76"/>
+      <c r="G23" s="76"/>
+      <c r="H23" s="77"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="s">
@@ -3742,14 +3742,14 @@
       <c r="B24" s="19">
         <v>1</v>
       </c>
-      <c r="C24" s="77" t="s">
+      <c r="C24" s="79" t="s">
         <v>36</v>
       </c>
-      <c r="D24" s="74"/>
-      <c r="E24" s="74"/>
-      <c r="F24" s="74"/>
-      <c r="G24" s="74"/>
-      <c r="H24" s="75"/>
+      <c r="D24" s="76"/>
+      <c r="E24" s="76"/>
+      <c r="F24" s="76"/>
+      <c r="G24" s="76"/>
+      <c r="H24" s="77"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="20" t="s">
@@ -3758,26 +3758,26 @@
       <c r="B25" s="21">
         <v>1</v>
       </c>
-      <c r="C25" s="73" t="s">
+      <c r="C25" s="75" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="74"/>
-      <c r="E25" s="74"/>
-      <c r="F25" s="74"/>
-      <c r="G25" s="74"/>
-      <c r="H25" s="75"/>
+      <c r="D25" s="76"/>
+      <c r="E25" s="76"/>
+      <c r="F25" s="76"/>
+      <c r="G25" s="76"/>
+      <c r="H25" s="77"/>
     </row>
     <row r="28" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="78" t="s">
+      <c r="A28" s="73" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="76"/>
-      <c r="C28" s="76"/>
-      <c r="D28" s="76"/>
-      <c r="E28" s="76"/>
-      <c r="F28" s="76"/>
-      <c r="G28" s="76"/>
-      <c r="H28" s="76"/>
+      <c r="B28" s="74"/>
+      <c r="C28" s="74"/>
+      <c r="D28" s="74"/>
+      <c r="E28" s="74"/>
+      <c r="F28" s="74"/>
+      <c r="G28" s="74"/>
+      <c r="H28" s="74"/>
     </row>
     <row r="29" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -3921,6 +3921,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="C19:H19"/>
     <mergeCell ref="A1:H1"/>
@@ -3937,12 +3943,6 @@
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="C6:H6"/>
     <mergeCell ref="C24:H24"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C23:H23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4030,10 +4030,10 @@
         <v>74</v>
       </c>
       <c r="Q1" s="28" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="R1" s="28" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="S1" s="28" t="s">
         <v>75</v>
@@ -4137,7 +4137,7 @@
         <v>220123498</v>
       </c>
       <c r="U2" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V2" s="24">
         <v>57.062100000000001</v>
@@ -4152,22 +4152,22 @@
         <v>139</v>
       </c>
       <c r="Z2" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA2" s="30" t="s">
         <v>140</v>
       </c>
       <c r="AB2" s="46" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="AC2" s="30" t="s">
+        <v>336</v>
+      </c>
+      <c r="AD2" s="30" t="s">
         <v>337</v>
       </c>
-      <c r="AD2" s="30" t="s">
-        <v>338</v>
-      </c>
       <c r="AE2" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="3" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -4175,7 +4175,7 @@
         <v>141</v>
       </c>
       <c r="B3" s="55" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>242</v>
@@ -4232,7 +4232,7 @@
         <v>31238542</v>
       </c>
       <c r="U3" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V3" s="24">
         <v>44.464755134852901</v>
@@ -4244,10 +4244,10 @@
         <v>95</v>
       </c>
       <c r="Y3" s="30" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="Z3" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA3" s="30" t="s">
         <v>92</v>
@@ -4256,13 +4256,13 @@
         <v>250</v>
       </c>
       <c r="AC3" s="30" t="s">
+        <v>393</v>
+      </c>
+      <c r="AD3" s="30" t="s">
         <v>394</v>
       </c>
-      <c r="AD3" s="30" t="s">
-        <v>395</v>
-      </c>
       <c r="AE3" s="61" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="4" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -4270,7 +4270,7 @@
         <v>98</v>
       </c>
       <c r="B4" s="54" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>108</v>
@@ -4282,10 +4282,10 @@
         <v>52</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="H4" s="35" t="s">
         <v>92</v>
@@ -4327,7 +4327,7 @@
         <v>3168000</v>
       </c>
       <c r="U4" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V4" s="26">
         <v>43.327720234653299</v>
@@ -4339,22 +4339,22 @@
         <v>95</v>
       </c>
       <c r="Y4" s="34" t="s">
+        <v>339</v>
+      </c>
+      <c r="Z4" s="34" t="s">
+        <v>587</v>
+      </c>
+      <c r="AA4" s="34" t="s">
+        <v>289</v>
+      </c>
+      <c r="AB4" s="46" t="s">
+        <v>348</v>
+      </c>
+      <c r="AC4" s="34" t="s">
         <v>340</v>
       </c>
-      <c r="Z4" s="34" t="s">
-        <v>588</v>
-      </c>
-      <c r="AA4" s="34" t="s">
-        <v>290</v>
-      </c>
-      <c r="AB4" s="46" t="s">
-        <v>349</v>
-      </c>
-      <c r="AC4" s="34" t="s">
+      <c r="AD4" s="34" t="s">
         <v>341</v>
-      </c>
-      <c r="AD4" s="34" t="s">
-        <v>342</v>
       </c>
       <c r="AE4" s="62" t="s">
         <v>27</v>
@@ -4365,13 +4365,13 @@
         <v>119</v>
       </c>
       <c r="B5" s="55" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>108</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>42</v>
@@ -4407,7 +4407,7 @@
         <v>92</v>
       </c>
       <c r="P5" s="32" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="Q5" s="32">
         <v>2030</v>
@@ -4422,7 +4422,7 @@
         <v>170000000</v>
       </c>
       <c r="U5" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V5" s="24">
         <v>46.809800000000003</v>
@@ -4437,22 +4437,22 @@
         <v>177</v>
       </c>
       <c r="Z5" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA5" s="30" t="s">
         <v>178</v>
       </c>
       <c r="AB5" s="46" t="s">
+        <v>353</v>
+      </c>
+      <c r="AC5" s="30" t="s">
         <v>354</v>
       </c>
-      <c r="AC5" s="30" t="s">
+      <c r="AD5" s="30" t="s">
         <v>355</v>
       </c>
-      <c r="AD5" s="30" t="s">
-        <v>356</v>
-      </c>
       <c r="AE5" s="63" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="6" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -4460,10 +4460,10 @@
         <v>141</v>
       </c>
       <c r="B6" s="55" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D6" s="30" t="s">
         <v>150</v>
@@ -4472,10 +4472,10 @@
         <v>45</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="H6" s="31">
         <v>2.5999999999999999E-2</v>
@@ -4517,7 +4517,7 @@
         <v>7958244</v>
       </c>
       <c r="U6" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V6" s="23" t="s">
         <v>92</v>
@@ -4532,22 +4532,22 @@
         <v>92</v>
       </c>
       <c r="Z6" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA6" s="30" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="AB6" s="46" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="AC6" s="30" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="AD6" s="30" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="AE6" s="64" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="7" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -4612,7 +4612,7 @@
         <v>189694949</v>
       </c>
       <c r="U7" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V7" s="24">
         <v>43.232830995956597</v>
@@ -4624,25 +4624,25 @@
         <v>132</v>
       </c>
       <c r="Y7" s="30" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="Z7" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA7" s="30" t="s">
         <v>133</v>
       </c>
       <c r="AB7" s="46" t="s">
+        <v>361</v>
+      </c>
+      <c r="AC7" s="30" t="s">
+        <v>360</v>
+      </c>
+      <c r="AD7" s="30" t="s">
         <v>362</v>
       </c>
-      <c r="AC7" s="30" t="s">
-        <v>361</v>
-      </c>
-      <c r="AD7" s="30" t="s">
-        <v>363</v>
-      </c>
       <c r="AE7" s="63" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="8" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -4692,7 +4692,7 @@
         <v>92</v>
       </c>
       <c r="P8" s="32" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="Q8" s="32">
         <v>2029</v>
@@ -4704,10 +4704,10 @@
         <v>122</v>
       </c>
       <c r="T8" s="33" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="U8" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V8" s="24">
         <v>50.575420999999999</v>
@@ -4722,22 +4722,22 @@
         <v>123</v>
       </c>
       <c r="Z8" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA8" s="30" t="s">
         <v>124</v>
       </c>
       <c r="AB8" s="46" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AC8" s="30" t="s">
         <v>125</v>
       </c>
       <c r="AD8" s="30" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="AE8" s="63" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="9" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -4748,19 +4748,19 @@
         <v>224</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D9" s="34" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>50</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="H9" s="35">
         <v>2.5819174</v>
@@ -4802,7 +4802,7 @@
         <v>169300000</v>
       </c>
       <c r="U9" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V9" s="26">
         <v>37.960247145532399</v>
@@ -4814,25 +4814,25 @@
         <v>95</v>
       </c>
       <c r="Y9" s="34" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="Z9" s="34" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="AA9" s="34" t="s">
         <v>226</v>
       </c>
       <c r="AB9" s="46" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="AC9" s="34" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AD9" s="34" t="s">
         <v>227</v>
       </c>
       <c r="AE9" s="61" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="10" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -4840,22 +4840,22 @@
         <v>87</v>
       </c>
       <c r="B10" s="55" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>58</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H10" s="31" t="s">
         <v>92</v>
@@ -4909,22 +4909,22 @@
         <v>95</v>
       </c>
       <c r="Y10" s="30" t="s">
+        <v>306</v>
+      </c>
+      <c r="Z10" s="30" t="s">
+        <v>586</v>
+      </c>
+      <c r="AA10" s="30" t="s">
         <v>307</v>
       </c>
-      <c r="Z10" s="30" t="s">
-        <v>587</v>
-      </c>
-      <c r="AA10" s="30" t="s">
-        <v>308</v>
-      </c>
       <c r="AB10" s="46" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="AC10" s="30" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="AD10" s="30" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="AE10" s="62" t="s">
         <v>27</v>
@@ -4935,10 +4935,10 @@
         <v>126</v>
       </c>
       <c r="B11" s="55" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D11" s="30" t="s">
         <v>150</v>
@@ -4947,10 +4947,10 @@
         <v>46</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="H11" s="31" t="s">
         <v>92</v>
@@ -4989,10 +4989,10 @@
         <v>122</v>
       </c>
       <c r="T11" s="33" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="U11" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V11" s="24">
         <v>59.592303479664103</v>
@@ -5004,25 +5004,25 @@
         <v>244</v>
       </c>
       <c r="Y11" s="30" t="s">
+        <v>421</v>
+      </c>
+      <c r="Z11" s="30" t="s">
+        <v>586</v>
+      </c>
+      <c r="AA11" s="30" t="s">
+        <v>267</v>
+      </c>
+      <c r="AB11" s="46" t="s">
+        <v>417</v>
+      </c>
+      <c r="AC11" s="30" t="s">
         <v>422</v>
       </c>
-      <c r="Z11" s="30" t="s">
-        <v>587</v>
-      </c>
-      <c r="AA11" s="30" t="s">
-        <v>268</v>
-      </c>
-      <c r="AB11" s="46" t="s">
-        <v>418</v>
-      </c>
-      <c r="AC11" s="30" t="s">
+      <c r="AD11" s="30" t="s">
         <v>423</v>
       </c>
-      <c r="AD11" s="30" t="s">
-        <v>424</v>
-      </c>
       <c r="AE11" s="63" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="12" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -5102,22 +5102,22 @@
         <v>194</v>
       </c>
       <c r="Z12" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA12" s="34" t="s">
         <v>195</v>
       </c>
       <c r="AB12" s="46" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="AC12" s="34" t="s">
+        <v>424</v>
+      </c>
+      <c r="AD12" s="34" t="s">
         <v>425</v>
       </c>
-      <c r="AD12" s="34" t="s">
-        <v>426</v>
-      </c>
       <c r="AE12" s="64" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="13" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5194,10 +5194,10 @@
         <v>95</v>
       </c>
       <c r="Y13" s="34" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="Z13" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA13" s="34" t="s">
         <v>167</v>
@@ -5206,13 +5206,13 @@
         <v>168</v>
       </c>
       <c r="AC13" s="34" t="s">
+        <v>382</v>
+      </c>
+      <c r="AD13" s="34" t="s">
         <v>383</v>
       </c>
-      <c r="AD13" s="34" t="s">
-        <v>384</v>
-      </c>
       <c r="AE13" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="14" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -5223,7 +5223,7 @@
         <v>246</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="D14" s="34" t="s">
         <v>109</v>
@@ -5277,7 +5277,7 @@
         <v>23635998</v>
       </c>
       <c r="U14" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V14" s="26">
         <v>44.826999999999998</v>
@@ -5292,22 +5292,22 @@
         <v>248</v>
       </c>
       <c r="Z14" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA14" s="34" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="AB14" s="46" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="AC14" s="34" t="s">
+        <v>410</v>
+      </c>
+      <c r="AD14" s="34" t="s">
         <v>411</v>
       </c>
-      <c r="AD14" s="34" t="s">
-        <v>412</v>
-      </c>
       <c r="AE14" s="64" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="15" spans="1:31" ht="148.19999999999999" x14ac:dyDescent="0.3">
@@ -5372,7 +5372,7 @@
         <v>119682059</v>
       </c>
       <c r="U15" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V15" s="26">
         <v>43.186100000000003</v>
@@ -5387,20 +5387,20 @@
         <v>176</v>
       </c>
       <c r="Z15" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA15" s="34"/>
       <c r="AB15" s="46" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="AC15" s="34" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="AD15" s="34" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="AE15" s="64" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="16" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5408,7 +5408,7 @@
         <v>119</v>
       </c>
       <c r="B16" s="55" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>108</v>
@@ -5420,10 +5420,10 @@
         <v>59</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="H16" s="31" t="s">
         <v>92</v>
@@ -5462,10 +5462,10 @@
         <v>122</v>
       </c>
       <c r="T16" s="33" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="U16" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V16" s="24">
         <v>45.290985428950698</v>
@@ -5477,25 +5477,25 @@
         <v>244</v>
       </c>
       <c r="Y16" s="30" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="Z16" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA16" s="30" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="AB16" s="46" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="AC16" s="30" t="s">
+        <v>429</v>
+      </c>
+      <c r="AD16" s="30" t="s">
         <v>430</v>
       </c>
-      <c r="AD16" s="30" t="s">
-        <v>431</v>
-      </c>
       <c r="AE16" s="65" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="17" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5503,7 +5503,7 @@
         <v>98</v>
       </c>
       <c r="B17" s="55" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>219</v>
@@ -5515,10 +5515,10 @@
         <v>43</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="H17" s="51">
         <v>4.5999999999999999E-3</v>
@@ -5560,7 +5560,7 @@
         <v>30497000</v>
       </c>
       <c r="U17" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V17" s="23">
         <v>51.870851200822599</v>
@@ -5572,22 +5572,22 @@
         <v>244</v>
       </c>
       <c r="Y17" s="30" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="Z17" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA17" s="30" t="s">
+        <v>254</v>
+      </c>
+      <c r="AB17" s="25" t="s">
         <v>255</v>
       </c>
-      <c r="AB17" s="25" t="s">
-        <v>256</v>
-      </c>
       <c r="AC17" s="30" t="s">
+        <v>433</v>
+      </c>
+      <c r="AD17" s="30" t="s">
         <v>434</v>
-      </c>
-      <c r="AD17" s="30" t="s">
-        <v>435</v>
       </c>
       <c r="AE17" s="62" t="s">
         <v>27</v>
@@ -5655,7 +5655,7 @@
         <v>157000000</v>
       </c>
       <c r="U18" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V18" s="24">
         <v>52.489100000000001</v>
@@ -5670,7 +5670,7 @@
         <v>206</v>
       </c>
       <c r="Z18" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA18" s="30" t="s">
         <v>207</v>
@@ -5679,13 +5679,13 @@
         <v>208</v>
       </c>
       <c r="AC18" s="30" t="s">
+        <v>387</v>
+      </c>
+      <c r="AD18" s="30" t="s">
         <v>388</v>
       </c>
-      <c r="AD18" s="30" t="s">
-        <v>389</v>
-      </c>
       <c r="AE18" s="65" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="19" spans="1:31" ht="57" x14ac:dyDescent="0.3">
@@ -5750,7 +5750,7 @@
         <v>4265136</v>
       </c>
       <c r="U19" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V19" s="26">
         <v>50.569000000000003</v>
@@ -5765,13 +5765,13 @@
         <v>104</v>
       </c>
       <c r="Z19" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA19" s="34" t="s">
         <v>105</v>
       </c>
       <c r="AB19" s="46" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="AC19" s="34" t="s">
         <v>105</v>
@@ -5791,10 +5791,10 @@
         <v>237</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>49</v>
@@ -5803,7 +5803,7 @@
         <v>235</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="H20" s="35">
         <v>2.11</v>
@@ -5860,7 +5860,7 @@
         <v>238</v>
       </c>
       <c r="Z20" s="34" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="AA20" s="34" t="s">
         <v>239</v>
@@ -5869,13 +5869,13 @@
         <v>240</v>
       </c>
       <c r="AC20" s="34" t="s">
+        <v>437</v>
+      </c>
+      <c r="AD20" s="34" t="s">
         <v>438</v>
       </c>
-      <c r="AD20" s="34" t="s">
-        <v>439</v>
-      </c>
       <c r="AE20" s="66" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="21" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5883,13 +5883,13 @@
         <v>126</v>
       </c>
       <c r="B21" s="54" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D21" s="34" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>52</v>
@@ -5928,10 +5928,10 @@
         <v>2025</v>
       </c>
       <c r="Q21" s="36" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="R21" s="36" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="S21" s="22" t="s">
         <v>122</v>
@@ -5940,7 +5940,7 @@
         <v>25400000</v>
       </c>
       <c r="U21" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V21" s="26">
         <v>41.352637812781921</v>
@@ -5952,25 +5952,25 @@
         <v>132</v>
       </c>
       <c r="Y21" s="30" t="s">
+        <v>439</v>
+      </c>
+      <c r="Z21" s="34" t="s">
+        <v>588</v>
+      </c>
+      <c r="AA21" s="34" t="s">
+        <v>303</v>
+      </c>
+      <c r="AB21" s="46" t="s">
+        <v>441</v>
+      </c>
+      <c r="AC21" s="34" t="s">
         <v>440</v>
       </c>
-      <c r="Z21" s="34" t="s">
-        <v>589</v>
-      </c>
-      <c r="AA21" s="34" t="s">
+      <c r="AD21" s="34" t="s">
         <v>304</v>
       </c>
-      <c r="AB21" s="46" t="s">
-        <v>442</v>
-      </c>
-      <c r="AC21" s="34" t="s">
-        <v>441</v>
-      </c>
-      <c r="AD21" s="34" t="s">
-        <v>305</v>
-      </c>
       <c r="AE21" s="65" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="22" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6047,25 +6047,25 @@
         <v>244</v>
       </c>
       <c r="Y22" s="29" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="Z22" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA22" s="30" t="s">
         <v>245</v>
       </c>
       <c r="AB22" s="46" t="s">
+        <v>442</v>
+      </c>
+      <c r="AC22" s="30" t="s">
         <v>443</v>
       </c>
-      <c r="AC22" s="30" t="s">
+      <c r="AD22" s="30" t="s">
         <v>444</v>
       </c>
-      <c r="AD22" s="30" t="s">
-        <v>445</v>
-      </c>
       <c r="AE22" s="64" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="23" spans="1:31" ht="136.80000000000001" x14ac:dyDescent="0.3">
@@ -6085,10 +6085,10 @@
         <v>57</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="H23" s="35">
         <v>0.56499999999999995</v>
@@ -6142,25 +6142,25 @@
         <v>95</v>
       </c>
       <c r="Y23" s="34" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="Z23" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA23" s="34" t="s">
         <v>233</v>
       </c>
       <c r="AB23" s="46" t="s">
+        <v>447</v>
+      </c>
+      <c r="AC23" s="34" t="s">
         <v>448</v>
       </c>
-      <c r="AC23" s="34" t="s">
+      <c r="AD23" s="34" t="s">
         <v>449</v>
       </c>
-      <c r="AD23" s="34" t="s">
-        <v>450</v>
-      </c>
       <c r="AE23" s="65" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="24" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6171,7 +6171,7 @@
         <v>179</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D24" s="34" t="s">
         <v>150</v>
@@ -6180,10 +6180,10 @@
         <v>42</v>
       </c>
       <c r="F24" s="71" t="s">
+        <v>456</v>
+      </c>
+      <c r="G24" s="72" t="s">
         <v>457</v>
-      </c>
-      <c r="G24" s="72" t="s">
-        <v>458</v>
       </c>
       <c r="H24" s="35">
         <v>0.2</v>
@@ -6237,25 +6237,25 @@
         <v>180</v>
       </c>
       <c r="Y24" s="34" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="Z24" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA24" s="34" t="s">
         <v>181</v>
       </c>
       <c r="AB24" s="46" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="AC24" s="34" t="s">
+        <v>458</v>
+      </c>
+      <c r="AD24" s="34" t="s">
         <v>459</v>
       </c>
-      <c r="AD24" s="34" t="s">
-        <v>460</v>
-      </c>
       <c r="AE24" s="61" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="25" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -6275,10 +6275,10 @@
         <v>56</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="H25" s="35">
         <v>1</v>
@@ -6320,7 +6320,7 @@
         <v>216000000</v>
       </c>
       <c r="U25" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V25" s="26">
         <v>45.515127894849797</v>
@@ -6332,25 +6332,25 @@
         <v>244</v>
       </c>
       <c r="Y25" s="34" t="s">
+        <v>595</v>
+      </c>
+      <c r="Z25" s="34" t="s">
+        <v>586</v>
+      </c>
+      <c r="AA25" s="34" t="s">
         <v>596</v>
       </c>
-      <c r="Z25" s="34" t="s">
-        <v>587</v>
-      </c>
-      <c r="AA25" s="34" t="s">
-        <v>252</v>
-      </c>
       <c r="AB25" s="46" t="s">
+        <v>452</v>
+      </c>
+      <c r="AC25" s="34" t="s">
         <v>453</v>
       </c>
-      <c r="AC25" s="34" t="s">
+      <c r="AD25" s="34" t="s">
         <v>454</v>
       </c>
-      <c r="AD25" s="34" t="s">
-        <v>455</v>
-      </c>
       <c r="AE25" s="65" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="26" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6358,10 +6358,10 @@
         <v>87</v>
       </c>
       <c r="B26" s="54" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C26" s="34" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="D26" s="34" t="s">
         <v>150</v>
@@ -6370,7 +6370,7 @@
         <v>46</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G26" s="4" t="s">
         <v>93</v>
@@ -6415,7 +6415,7 @@
         <v>40000000</v>
       </c>
       <c r="U26" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V26" s="22">
         <v>59.121267699503399</v>
@@ -6427,25 +6427,25 @@
         <v>244</v>
       </c>
       <c r="Y26" s="34" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="Z26" s="34" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="AA26" s="34" t="s">
+        <v>260</v>
+      </c>
+      <c r="AB26" s="27" t="s">
         <v>261</v>
       </c>
-      <c r="AB26" s="27" t="s">
-        <v>262</v>
-      </c>
       <c r="AC26" s="34" t="s">
+        <v>591</v>
+      </c>
+      <c r="AD26" s="34" t="s">
         <v>592</v>
       </c>
-      <c r="AD26" s="34" t="s">
-        <v>593</v>
-      </c>
       <c r="AE26" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="27" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -6468,7 +6468,7 @@
         <v>170</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="H27" s="31">
         <v>0.23252429999999999</v>
@@ -6522,10 +6522,10 @@
         <v>95</v>
       </c>
       <c r="Y27" s="30" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="Z27" s="30" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="AA27" s="30" t="s">
         <v>171</v>
@@ -6534,13 +6534,13 @@
         <v>172</v>
       </c>
       <c r="AC27" s="30" t="s">
+        <v>463</v>
+      </c>
+      <c r="AD27" s="30" t="s">
         <v>464</v>
       </c>
-      <c r="AD27" s="30" t="s">
-        <v>465</v>
-      </c>
       <c r="AE27" s="61" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="28" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -6554,7 +6554,7 @@
         <v>225</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>54</v>
@@ -6617,25 +6617,25 @@
         <v>132</v>
       </c>
       <c r="Y28" s="30" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="Z28" s="30" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="AA28" s="30" t="s">
         <v>148</v>
       </c>
       <c r="AB28" s="46" t="s">
+        <v>467</v>
+      </c>
+      <c r="AC28" s="30" t="s">
         <v>468</v>
       </c>
-      <c r="AC28" s="30" t="s">
+      <c r="AD28" s="30" t="s">
         <v>469</v>
       </c>
-      <c r="AD28" s="30" t="s">
-        <v>470</v>
-      </c>
       <c r="AE28" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="29" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -6700,7 +6700,7 @@
         <v>228721666</v>
       </c>
       <c r="U29" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V29" s="24">
         <v>51.297800000000002</v>
@@ -6712,10 +6712,10 @@
         <v>180</v>
       </c>
       <c r="Y29" s="30" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="Z29" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA29" s="30" t="s">
         <v>198</v>
@@ -6724,13 +6724,13 @@
         <v>199</v>
       </c>
       <c r="AC29" s="30" t="s">
+        <v>471</v>
+      </c>
+      <c r="AD29" s="30" t="s">
         <v>472</v>
       </c>
-      <c r="AD29" s="30" t="s">
-        <v>473</v>
-      </c>
       <c r="AE29" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="30" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6738,22 +6738,22 @@
         <v>163</v>
       </c>
       <c r="B30" s="54" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="D30" s="34" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>58</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H30" s="53">
         <v>4.5999999999999999E-2</v>
@@ -6795,7 +6795,7 @@
         <v>29500000</v>
       </c>
       <c r="U30" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V30" s="22">
         <v>60.618241659279597</v>
@@ -6807,25 +6807,25 @@
         <v>244</v>
       </c>
       <c r="Y30" s="34" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="Z30" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA30" s="34" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="AB30" s="47" t="s">
+        <v>498</v>
+      </c>
+      <c r="AC30" s="34" t="s">
         <v>499</v>
       </c>
-      <c r="AC30" s="34" t="s">
+      <c r="AD30" s="34" t="s">
         <v>500</v>
       </c>
-      <c r="AD30" s="34" t="s">
-        <v>501</v>
-      </c>
       <c r="AE30" s="61" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="31" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6890,7 +6890,7 @@
         <v>191000000</v>
       </c>
       <c r="U31" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V31" s="26">
         <v>51.618000000000002</v>
@@ -6905,7 +6905,7 @@
         <v>201</v>
       </c>
       <c r="Z31" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA31" s="34" t="s">
         <v>202</v>
@@ -6914,13 +6914,13 @@
         <v>203</v>
       </c>
       <c r="AC31" s="34" t="s">
+        <v>408</v>
+      </c>
+      <c r="AD31" s="34" t="s">
         <v>409</v>
       </c>
-      <c r="AD31" s="34" t="s">
-        <v>410</v>
-      </c>
       <c r="AE31" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="32" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6928,7 +6928,7 @@
         <v>87</v>
       </c>
       <c r="B32" s="54" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>108</v>
@@ -6940,10 +6940,10 @@
         <v>45</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H32" s="35">
         <v>1</v>
@@ -6997,25 +6997,25 @@
         <v>95</v>
       </c>
       <c r="Y32" s="34" t="s">
+        <v>473</v>
+      </c>
+      <c r="Z32" s="34" t="s">
+        <v>586</v>
+      </c>
+      <c r="AA32" s="34" t="s">
+        <v>276</v>
+      </c>
+      <c r="AB32" s="46" t="s">
         <v>474</v>
       </c>
-      <c r="Z32" s="34" t="s">
-        <v>587</v>
-      </c>
-      <c r="AA32" s="34" t="s">
+      <c r="AC32" s="34" t="s">
+        <v>390</v>
+      </c>
+      <c r="AD32" s="34" t="s">
         <v>277</v>
       </c>
-      <c r="AB32" s="46" t="s">
-        <v>475</v>
-      </c>
-      <c r="AC32" s="34" t="s">
-        <v>391</v>
-      </c>
-      <c r="AD32" s="34" t="s">
-        <v>278</v>
-      </c>
       <c r="AE32" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="33" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7095,22 +7095,22 @@
         <v>112</v>
       </c>
       <c r="Z33" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA33" s="30" t="s">
         <v>113</v>
       </c>
       <c r="AB33" s="46" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="AC33" s="30" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD33" s="30" t="s">
         <v>476</v>
       </c>
-      <c r="AD33" s="30" t="s">
-        <v>477</v>
-      </c>
       <c r="AE33" s="66" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="34" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7118,19 +7118,19 @@
         <v>87</v>
       </c>
       <c r="B34" s="55" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>225</v>
       </c>
       <c r="D34" s="30" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>52</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="G34" s="2"/>
       <c r="H34" s="31">
@@ -7173,7 +7173,7 @@
         <v>122900000</v>
       </c>
       <c r="U34" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V34" s="23">
         <v>43.151000000000003</v>
@@ -7185,25 +7185,25 @@
         <v>244</v>
       </c>
       <c r="Y34" s="30" t="s">
+        <v>478</v>
+      </c>
+      <c r="Z34" s="30" t="s">
+        <v>589</v>
+      </c>
+      <c r="AA34" s="30" t="s">
+        <v>292</v>
+      </c>
+      <c r="AB34" s="46" t="s">
+        <v>293</v>
+      </c>
+      <c r="AC34" s="30" t="s">
         <v>479</v>
       </c>
-      <c r="Z34" s="30" t="s">
-        <v>590</v>
-      </c>
-      <c r="AA34" s="30" t="s">
-        <v>293</v>
-      </c>
-      <c r="AB34" s="46" t="s">
-        <v>294</v>
-      </c>
-      <c r="AC34" s="30" t="s">
+      <c r="AD34" s="30" t="s">
         <v>480</v>
       </c>
-      <c r="AD34" s="30" t="s">
-        <v>481</v>
-      </c>
       <c r="AE34" s="64" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="35" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7214,10 +7214,10 @@
         <v>142</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>54</v>
@@ -7226,7 +7226,7 @@
         <v>143</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="H35" s="35">
         <v>0.28144999999999998</v>
@@ -7283,19 +7283,19 @@
         <v>144</v>
       </c>
       <c r="Z35" s="34" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="AA35" s="34" t="s">
         <v>145</v>
       </c>
       <c r="AB35" s="46" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="AC35" s="34" t="s">
+        <v>373</v>
+      </c>
+      <c r="AD35" s="34" t="s">
         <v>374</v>
-      </c>
-      <c r="AD35" s="34" t="s">
-        <v>375</v>
       </c>
       <c r="AE35" s="62" t="s">
         <v>27</v>
@@ -7309,7 +7309,7 @@
         <v>114</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="D36" s="34" t="s">
         <v>109</v>
@@ -7363,7 +7363,7 @@
         <v>159000000</v>
       </c>
       <c r="U36" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V36" s="26">
         <v>51.1339349</v>
@@ -7375,25 +7375,25 @@
         <v>95</v>
       </c>
       <c r="Y36" s="34" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="Z36" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA36" s="34" t="s">
         <v>118</v>
       </c>
       <c r="AB36" s="46" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="AC36" s="34" t="s">
+        <v>483</v>
+      </c>
+      <c r="AD36" s="34" t="s">
         <v>484</v>
       </c>
-      <c r="AD36" s="34" t="s">
-        <v>485</v>
-      </c>
       <c r="AE36" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="37" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7401,22 +7401,22 @@
         <v>163</v>
       </c>
       <c r="B37" s="54" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>45</v>
       </c>
       <c r="F37" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="G37" s="4" t="s">
         <v>283</v>
-      </c>
-      <c r="G37" s="4" t="s">
-        <v>284</v>
       </c>
       <c r="H37" s="53">
         <v>5.0046999999999999E-3</v>
@@ -7458,7 +7458,7 @@
         <v>26498650</v>
       </c>
       <c r="U37" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V37" s="26">
         <v>50.529000000000003</v>
@@ -7470,25 +7470,25 @@
         <v>95</v>
       </c>
       <c r="Y37" s="34" t="s">
+        <v>284</v>
+      </c>
+      <c r="Z37" s="34" t="s">
+        <v>588</v>
+      </c>
+      <c r="AA37" s="34" t="s">
         <v>285</v>
       </c>
-      <c r="Z37" s="34" t="s">
-        <v>589</v>
-      </c>
-      <c r="AA37" s="34" t="s">
-        <v>286</v>
-      </c>
       <c r="AB37" s="46" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="AC37" s="34" t="s">
+        <v>485</v>
+      </c>
+      <c r="AD37" s="34" t="s">
         <v>486</v>
       </c>
-      <c r="AD37" s="34" t="s">
-        <v>487</v>
-      </c>
       <c r="AE37" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="38" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7496,7 +7496,7 @@
         <v>87</v>
       </c>
       <c r="B38" s="54" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>108</v>
@@ -7553,7 +7553,7 @@
         <v>234000000</v>
       </c>
       <c r="U38" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V38" s="26">
         <v>38.129899999999999</v>
@@ -7565,25 +7565,25 @@
         <v>95</v>
       </c>
       <c r="Y38" s="34" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="Z38" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA38" s="34" t="s">
         <v>217</v>
       </c>
       <c r="AB38" s="46" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="AC38" s="34" t="s">
+        <v>404</v>
+      </c>
+      <c r="AD38" s="34" t="s">
         <v>405</v>
       </c>
-      <c r="AD38" s="34" t="s">
-        <v>406</v>
-      </c>
       <c r="AE38" s="61" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="39" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7591,10 +7591,10 @@
         <v>141</v>
       </c>
       <c r="B39" s="55" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="D39" s="34" t="s">
         <v>109</v>
@@ -7603,7 +7603,7 @@
         <v>58</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="G39" s="2"/>
       <c r="H39" s="31">
@@ -7658,25 +7658,25 @@
         <v>180</v>
       </c>
       <c r="Y39" s="30" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="Z39" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA39" s="30" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="AB39" s="46" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="AC39" s="30" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="AD39" s="30" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="AE39" s="61" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="40" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7690,7 +7690,7 @@
         <v>219</v>
       </c>
       <c r="D40" s="30" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>50</v>
@@ -7741,7 +7741,7 @@
         <v>127000000</v>
       </c>
       <c r="U40" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V40" s="24">
         <v>37.916800000000002</v>
@@ -7756,7 +7756,7 @@
         <v>221</v>
       </c>
       <c r="Z40" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA40" s="30" t="s">
         <v>222</v>
@@ -7765,13 +7765,13 @@
         <v>223</v>
       </c>
       <c r="AC40" s="30" t="s">
+        <v>490</v>
+      </c>
+      <c r="AD40" s="30" t="s">
         <v>491</v>
       </c>
-      <c r="AD40" s="30" t="s">
-        <v>492</v>
-      </c>
       <c r="AE40" s="64" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="41" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -7851,22 +7851,22 @@
         <v>96</v>
       </c>
       <c r="Z41" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA41" s="30" t="s">
         <v>97</v>
       </c>
       <c r="AB41" s="46" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="AC41" s="30" t="s">
+        <v>492</v>
+      </c>
+      <c r="AD41" s="30" t="s">
         <v>493</v>
       </c>
-      <c r="AD41" s="30" t="s">
-        <v>494</v>
-      </c>
       <c r="AE41" s="66" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="42" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -7931,7 +7931,7 @@
         <v>117000000</v>
       </c>
       <c r="U42" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V42" s="26">
         <v>44.968299999999999</v>
@@ -7946,22 +7946,22 @@
         <v>136</v>
       </c>
       <c r="Z42" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA42" s="34" t="s">
         <v>134</v>
       </c>
       <c r="AB42" s="46" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="AC42" s="34" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="AD42" s="34" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="AE42" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="43" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7969,19 +7969,19 @@
         <v>87</v>
       </c>
       <c r="B43" s="54" t="s">
+        <v>376</v>
+      </c>
+      <c r="C43" s="4" t="s">
         <v>377</v>
       </c>
-      <c r="C43" s="4" t="s">
-        <v>378</v>
-      </c>
       <c r="D43" s="30" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>43</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G43" s="4" t="s">
         <v>92</v>
@@ -8026,7 +8026,7 @@
         <v>118000000</v>
       </c>
       <c r="U43" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V43" s="26">
         <v>51.976999999999997</v>
@@ -8038,25 +8038,25 @@
         <v>95</v>
       </c>
       <c r="Y43" s="34" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="Z43" s="34" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="AA43" s="34" t="s">
         <v>92</v>
       </c>
       <c r="AB43" s="47" t="s">
+        <v>378</v>
+      </c>
+      <c r="AC43" s="34" t="s">
         <v>379</v>
       </c>
-      <c r="AC43" s="34" t="s">
+      <c r="AD43" s="34" t="s">
         <v>380</v>
       </c>
-      <c r="AD43" s="34" t="s">
-        <v>381</v>
-      </c>
       <c r="AE43" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="44" spans="1:31" ht="68.400000000000006" x14ac:dyDescent="0.3">
@@ -8121,7 +8121,7 @@
         <v>36000000</v>
       </c>
       <c r="U44" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V44" s="26">
         <v>50.406342306737002</v>
@@ -8133,25 +8133,25 @@
         <v>95</v>
       </c>
       <c r="Y44" s="34" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="Z44" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA44" s="34" t="s">
         <v>129</v>
       </c>
       <c r="AB44" s="46" t="s">
+        <v>502</v>
+      </c>
+      <c r="AC44" s="34" t="s">
         <v>503</v>
       </c>
-      <c r="AC44" s="34" t="s">
+      <c r="AD44" s="34" t="s">
         <v>504</v>
       </c>
-      <c r="AD44" s="34" t="s">
-        <v>505</v>
-      </c>
       <c r="AE44" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="45" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -8159,19 +8159,19 @@
         <v>163</v>
       </c>
       <c r="B45" s="54" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D45" s="34" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>46</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="G45" s="4" t="s">
         <v>92</v>
@@ -8216,7 +8216,7 @@
         <v>13000000</v>
       </c>
       <c r="U45" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V45" s="22">
         <v>59.2181</v>
@@ -8228,25 +8228,25 @@
         <v>244</v>
       </c>
       <c r="Y45" s="34" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="Z45" s="34" t="s">
         <v>225</v>
       </c>
       <c r="AA45" s="34" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="AB45" s="46" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="AC45" s="34" t="s">
+        <v>508</v>
+      </c>
+      <c r="AD45" s="34" t="s">
         <v>509</v>
       </c>
-      <c r="AD45" s="34" t="s">
-        <v>510</v>
-      </c>
       <c r="AE45" s="64" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="46" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8326,22 +8326,22 @@
         <v>214</v>
       </c>
       <c r="Z46" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA46" s="30" t="s">
         <v>215</v>
       </c>
       <c r="AB46" s="46" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="AC46" s="30" t="s">
+        <v>401</v>
+      </c>
+      <c r="AD46" s="30" t="s">
         <v>402</v>
       </c>
-      <c r="AD46" s="30" t="s">
-        <v>403</v>
-      </c>
       <c r="AE46" s="64" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="47" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8352,7 +8352,7 @@
         <v>153</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D47" s="30" t="s">
         <v>150</v>
@@ -8361,10 +8361,10 @@
         <v>55</v>
       </c>
       <c r="F47" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="G47" s="2" t="s">
         <v>511</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>512</v>
       </c>
       <c r="H47" s="52">
         <v>1.55E-2</v>
@@ -8421,22 +8421,22 @@
         <v>154</v>
       </c>
       <c r="Z47" s="30" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="AA47" s="30" t="s">
         <v>155</v>
       </c>
       <c r="AB47" s="46" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="AC47" s="30" t="s">
+        <v>512</v>
+      </c>
+      <c r="AD47" s="30" t="s">
         <v>513</v>
       </c>
-      <c r="AD47" s="30" t="s">
-        <v>514</v>
-      </c>
       <c r="AE47" s="65" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="48" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -8444,7 +8444,7 @@
         <v>87</v>
       </c>
       <c r="B48" s="54" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>89</v>
@@ -8456,10 +8456,10 @@
         <v>58</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="H48" s="35">
         <v>0.40600000000000003</v>
@@ -8501,7 +8501,7 @@
         <v>97000000</v>
       </c>
       <c r="U48" s="37" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="V48" s="22">
         <v>58.099057767351503</v>
@@ -8513,25 +8513,25 @@
         <v>244</v>
       </c>
       <c r="Y48" s="34" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="Z48" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA48" s="34" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="AB48" s="47" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="AC48" s="34" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="AD48" s="34" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="AE48" s="61" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="49" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -8551,10 +8551,10 @@
         <v>54</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="H49" s="53">
         <v>6.7077999999999999E-2</v>
@@ -8596,7 +8596,7 @@
         <v>40000000</v>
       </c>
       <c r="U49" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V49" s="26">
         <v>56.787056035485499</v>
@@ -8611,22 +8611,22 @@
         <v>151</v>
       </c>
       <c r="Z49" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA49" s="34" t="s">
         <v>152</v>
       </c>
       <c r="AB49" s="46" t="s">
+        <v>518</v>
+      </c>
+      <c r="AC49" s="34" t="s">
         <v>519</v>
       </c>
-      <c r="AC49" s="34" t="s">
+      <c r="AD49" s="34" t="s">
         <v>520</v>
       </c>
-      <c r="AD49" s="34" t="s">
-        <v>521</v>
-      </c>
       <c r="AE49" s="64" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="50" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -8640,7 +8640,7 @@
         <v>225</v>
       </c>
       <c r="D50" s="34" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>48</v>
@@ -8679,7 +8679,7 @@
         <v>19458418</v>
       </c>
       <c r="U50" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V50" s="26">
         <v>48.096166502584701</v>
@@ -8691,7 +8691,7 @@
         <v>132</v>
       </c>
       <c r="Y50" s="34" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="Z50" s="34" t="s">
         <v>225</v>
@@ -8700,16 +8700,16 @@
         <v>211</v>
       </c>
       <c r="AB50" s="46" t="s">
+        <v>522</v>
+      </c>
+      <c r="AC50" s="34" t="s">
         <v>523</v>
       </c>
-      <c r="AC50" s="34" t="s">
+      <c r="AD50" s="34" t="s">
         <v>524</v>
       </c>
-      <c r="AD50" s="34" t="s">
-        <v>525</v>
-      </c>
       <c r="AE50" s="65" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="51" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -8729,10 +8729,10 @@
         <v>42</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="G51" s="30" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H51" s="31">
         <v>0.27411429999999998</v>
@@ -8786,25 +8786,25 @@
         <v>132</v>
       </c>
       <c r="Y51" s="30" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="Z51" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA51" s="30" t="s">
         <v>184</v>
       </c>
       <c r="AB51" s="46" t="s">
+        <v>526</v>
+      </c>
+      <c r="AC51" s="30" t="s">
         <v>527</v>
       </c>
-      <c r="AC51" s="30" t="s">
+      <c r="AD51" s="30" t="s">
         <v>528</v>
       </c>
-      <c r="AD51" s="30" t="s">
-        <v>529</v>
-      </c>
       <c r="AE51" s="65" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="52" spans="1:31" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -8869,7 +8869,7 @@
         <v>88286266</v>
       </c>
       <c r="U52" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V52" s="26">
         <v>60.306100000000001</v>
@@ -8884,7 +8884,7 @@
         <v>158</v>
       </c>
       <c r="Z52" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA52" s="34" t="s">
         <v>159</v>
@@ -8899,7 +8899,7 @@
         <v>162</v>
       </c>
       <c r="AE52" s="66" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="53" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8910,7 +8910,7 @@
         <v>234</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>109</v>
@@ -8922,7 +8922,7 @@
         <v>235</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="H53" s="31">
         <v>1.72E-2</v>
@@ -8964,7 +8964,7 @@
         <v>3867988</v>
       </c>
       <c r="U53" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V53" s="24">
         <v>64.037112316635401</v>
@@ -8976,22 +8976,22 @@
         <v>95</v>
       </c>
       <c r="Y53" s="30" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="Z53" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA53" s="30" t="s">
         <v>236</v>
       </c>
       <c r="AB53" s="46" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="AC53" s="30" t="s">
+        <v>535</v>
+      </c>
+      <c r="AD53" s="30" t="s">
         <v>536</v>
-      </c>
-      <c r="AD53" s="30" t="s">
-        <v>537</v>
       </c>
       <c r="AE53" s="67" t="s">
         <v>29</v>
@@ -9002,22 +9002,22 @@
         <v>163</v>
       </c>
       <c r="B54" s="55" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="D54" s="30" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>46</v>
       </c>
       <c r="F54" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="G54" s="30" t="s">
         <v>538</v>
-      </c>
-      <c r="G54" s="30" t="s">
-        <v>539</v>
       </c>
       <c r="H54" s="31">
         <v>0.16981750000000001</v>
@@ -9059,7 +9059,7 @@
         <v>40000000</v>
       </c>
       <c r="U54" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V54" s="24">
         <v>59.127044152710397</v>
@@ -9071,25 +9071,25 @@
         <v>132</v>
       </c>
       <c r="Y54" s="30" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="Z54" s="30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA54" s="30" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="AB54" s="46" t="s">
+        <v>539</v>
+      </c>
+      <c r="AC54" s="30" t="s">
         <v>540</v>
       </c>
-      <c r="AC54" s="30" t="s">
+      <c r="AD54" s="30" t="s">
         <v>541</v>
       </c>
-      <c r="AD54" s="30" t="s">
-        <v>542</v>
-      </c>
       <c r="AE54" s="65" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="55" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -9097,22 +9097,22 @@
         <v>87</v>
       </c>
       <c r="B55" s="55" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="D55" s="30" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>46</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="H55" s="31">
         <v>4.2</v>
@@ -9154,7 +9154,7 @@
         <v>225000000</v>
       </c>
       <c r="U55" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V55" s="23">
         <v>57.788622470324199</v>
@@ -9166,23 +9166,23 @@
         <v>132</v>
       </c>
       <c r="Y55" s="30" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="Z55" s="30" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="AA55" s="30"/>
       <c r="AB55" s="46" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="AC55" s="30" t="s">
+        <v>385</v>
+      </c>
+      <c r="AD55" s="30" t="s">
         <v>386</v>
       </c>
-      <c r="AD55" s="30" t="s">
-        <v>387</v>
-      </c>
       <c r="AE55" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="56" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -9202,10 +9202,10 @@
         <v>42</v>
       </c>
       <c r="F56" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="G56" s="2" t="s">
         <v>546</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>547</v>
       </c>
       <c r="H56" s="31">
         <v>0.17</v>
@@ -9259,25 +9259,25 @@
         <v>95</v>
       </c>
       <c r="Y56" s="30" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="Z56" s="30" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="AA56" s="30" t="s">
         <v>191</v>
       </c>
       <c r="AB56" s="46" t="s">
+        <v>548</v>
+      </c>
+      <c r="AC56" s="30" t="s">
         <v>549</v>
       </c>
-      <c r="AC56" s="30" t="s">
+      <c r="AD56" s="30" t="s">
         <v>550</v>
       </c>
-      <c r="AD56" s="30" t="s">
-        <v>551</v>
-      </c>
       <c r="AE56" s="64" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="57" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -9285,22 +9285,22 @@
         <v>87</v>
       </c>
       <c r="B57" s="55" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="D57" s="30" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>52</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="H57" s="31">
         <v>2</v>
@@ -9342,7 +9342,7 @@
         <v>205061582</v>
       </c>
       <c r="U57" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V57" s="24">
         <v>40.8482802817337</v>
@@ -9354,25 +9354,25 @@
         <v>132</v>
       </c>
       <c r="Y57" s="30" t="s">
+        <v>552</v>
+      </c>
+      <c r="Z57" s="30" t="s">
+        <v>590</v>
+      </c>
+      <c r="AA57" s="30" t="s">
+        <v>300</v>
+      </c>
+      <c r="AB57" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="AC57" s="30" t="s">
         <v>553</v>
       </c>
-      <c r="Z57" s="30" t="s">
-        <v>591</v>
-      </c>
-      <c r="AA57" s="30" t="s">
-        <v>301</v>
-      </c>
-      <c r="AB57" s="25" t="s">
-        <v>302</v>
-      </c>
-      <c r="AC57" s="30" t="s">
+      <c r="AD57" s="30" t="s">
         <v>554</v>
       </c>
-      <c r="AD57" s="30" t="s">
-        <v>555</v>
-      </c>
       <c r="AE57" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="58" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -9386,7 +9386,7 @@
         <v>225</v>
       </c>
       <c r="D58" s="34" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>50</v>
@@ -9449,7 +9449,7 @@
         <v>132</v>
       </c>
       <c r="Y58" s="30" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="Z58" s="30" t="s">
         <v>225</v>
@@ -9458,16 +9458,16 @@
         <v>230</v>
       </c>
       <c r="AB58" s="46" t="s">
+        <v>562</v>
+      </c>
+      <c r="AC58" s="30" t="s">
         <v>563</v>
       </c>
-      <c r="AC58" s="30" t="s">
+      <c r="AD58" s="30" t="s">
         <v>564</v>
       </c>
-      <c r="AD58" s="30" t="s">
-        <v>565</v>
-      </c>
       <c r="AE58" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="59" spans="1:31" ht="68.400000000000006" x14ac:dyDescent="0.3">
@@ -9475,10 +9475,10 @@
         <v>87</v>
       </c>
       <c r="B59" s="54" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D59" s="34" t="s">
         <v>150</v>
@@ -9487,10 +9487,10 @@
         <v>52</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="H59" s="53">
         <v>8.5999999999999993E-2</v>
@@ -9544,25 +9544,25 @@
         <v>244</v>
       </c>
       <c r="Y59" s="34" t="s">
+        <v>555</v>
+      </c>
+      <c r="Z59" s="34" t="s">
+        <v>589</v>
+      </c>
+      <c r="AA59" s="34" t="s">
+        <v>296</v>
+      </c>
+      <c r="AB59" s="27" t="s">
+        <v>297</v>
+      </c>
+      <c r="AC59" s="34" t="s">
         <v>556</v>
       </c>
-      <c r="Z59" s="34" t="s">
-        <v>590</v>
-      </c>
-      <c r="AA59" s="34" t="s">
-        <v>297</v>
-      </c>
-      <c r="AB59" s="27" t="s">
+      <c r="AD59" s="34" t="s">
         <v>298</v>
       </c>
-      <c r="AC59" s="34" t="s">
-        <v>557</v>
-      </c>
-      <c r="AD59" s="34" t="s">
-        <v>299</v>
-      </c>
       <c r="AE59" s="61" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="60" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -9642,22 +9642,22 @@
         <v>187</v>
       </c>
       <c r="Z60" s="34" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA60" s="34" t="s">
         <v>188</v>
       </c>
       <c r="AB60" s="46" t="s">
+        <v>557</v>
+      </c>
+      <c r="AC60" s="34" t="s">
         <v>558</v>
-      </c>
-      <c r="AC60" s="34" t="s">
-        <v>559</v>
       </c>
       <c r="AD60" s="34" t="s">
         <v>189</v>
       </c>
       <c r="AE60" s="60" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="61" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -9665,22 +9665,22 @@
         <v>126</v>
       </c>
       <c r="B61" s="54" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C61" s="2" t="s">
         <v>242</v>
       </c>
       <c r="D61" s="34" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="E61" s="4" t="s">
         <v>46</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="H61" s="35">
         <v>0.1</v>
@@ -9722,7 +9722,7 @@
         <v>26200000</v>
       </c>
       <c r="U61" s="37" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="V61" s="26">
         <v>60.45333865137971</v>
@@ -9734,25 +9734,25 @@
         <v>244</v>
       </c>
       <c r="Y61" s="34" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="Z61" s="34" t="s">
         <v>225</v>
       </c>
       <c r="AA61" s="34" t="s">
+        <v>270</v>
+      </c>
+      <c r="AB61" s="46" t="s">
+        <v>560</v>
+      </c>
+      <c r="AC61" s="34" t="s">
+        <v>561</v>
+      </c>
+      <c r="AD61" s="34" t="s">
         <v>271</v>
       </c>
-      <c r="AB61" s="46" t="s">
-        <v>561</v>
-      </c>
-      <c r="AC61" s="34" t="s">
-        <v>562</v>
-      </c>
-      <c r="AD61" s="34" t="s">
-        <v>272</v>
-      </c>
       <c r="AE61" s="65" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
   </sheetData>
@@ -9840,162 +9840,155 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="87" t="s">
+        <v>314</v>
+      </c>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="73" t="s">
         <v>315</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="78" t="s">
+      <c r="B3" s="74"/>
+      <c r="C3" s="74"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
+    </row>
+    <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="93" t="s">
         <v>316</v>
       </c>
-      <c r="B3" s="76"/>
-      <c r="C3" s="76"/>
-      <c r="D3" s="76"/>
-      <c r="E3" s="76"/>
-    </row>
-    <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="90" t="s">
+      <c r="B4" s="77"/>
+      <c r="C4" s="82" t="s">
         <v>317</v>
       </c>
-      <c r="B4" s="75"/>
-      <c r="C4" s="83" t="s">
+      <c r="D4" s="74"/>
+      <c r="E4" s="74"/>
+    </row>
+    <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="90" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="77"/>
+      <c r="C5" s="82" t="s">
         <v>318</v>
       </c>
-      <c r="D4" s="76"/>
-      <c r="E4" s="76"/>
-    </row>
-    <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="87" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="83" t="s">
+      <c r="D5" s="74"/>
+      <c r="E5" s="74"/>
+    </row>
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="88" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="77"/>
+      <c r="C6" s="82" t="s">
         <v>319</v>
       </c>
-      <c r="D5" s="76"/>
-      <c r="E5" s="76"/>
-    </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="85" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="75"/>
-      <c r="C6" s="83" t="s">
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
+    </row>
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="89" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="77"/>
+      <c r="C7" s="82" t="s">
         <v>320</v>
       </c>
-      <c r="D6" s="76"/>
-      <c r="E6" s="76"/>
-    </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="86" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="75"/>
-      <c r="C7" s="83" t="s">
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
+    </row>
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="92" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="77"/>
+      <c r="C8" s="82" t="s">
         <v>321</v>
       </c>
-      <c r="D7" s="76"/>
-      <c r="E7" s="76"/>
-    </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="89" t="s">
-        <v>35</v>
-      </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="83" t="s">
+      <c r="D8" s="74"/>
+      <c r="E8" s="74"/>
+    </row>
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="85" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="77"/>
+      <c r="C9" s="82" t="s">
         <v>322</v>
       </c>
-      <c r="D8" s="76"/>
-      <c r="E8" s="76"/>
-    </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="93" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" s="75"/>
-      <c r="C9" s="83" t="s">
+      <c r="D9" s="74"/>
+      <c r="E9" s="74"/>
+    </row>
+    <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="83" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="77"/>
+      <c r="C10" s="82" t="s">
         <v>323</v>
       </c>
-      <c r="D9" s="76"/>
-      <c r="E9" s="76"/>
-    </row>
-    <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="91" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="75"/>
-      <c r="C10" s="83" t="s">
+      <c r="D10" s="74"/>
+      <c r="E10" s="74"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="73" t="s">
         <v>324</v>
       </c>
-      <c r="D10" s="76"/>
-      <c r="E10" s="76"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="78" t="s">
+      <c r="B12" s="74"/>
+      <c r="C12" s="74"/>
+      <c r="D12" s="74"/>
+      <c r="E12" s="74"/>
+    </row>
+    <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="84" t="s">
         <v>325</v>
       </c>
-      <c r="B12" s="76"/>
-      <c r="C12" s="76"/>
-      <c r="D12" s="76"/>
-      <c r="E12" s="76"/>
-    </row>
-    <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="92" t="s">
+      <c r="B13" s="77"/>
+      <c r="C13" s="82" t="s">
         <v>326</v>
       </c>
-      <c r="B13" s="75"/>
-      <c r="C13" s="83" t="s">
+      <c r="D13" s="74"/>
+      <c r="E13" s="74"/>
+    </row>
+    <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="91" t="s">
         <v>327</v>
       </c>
-      <c r="D13" s="76"/>
-      <c r="E13" s="76"/>
-    </row>
-    <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="88" t="s">
+      <c r="B14" s="77"/>
+      <c r="C14" s="82" t="s">
         <v>328</v>
       </c>
-      <c r="B14" s="75"/>
-      <c r="C14" s="83" t="s">
+      <c r="D14" s="74"/>
+      <c r="E14" s="74"/>
+    </row>
+    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="86" t="s">
         <v>329</v>
       </c>
-      <c r="D14" s="76"/>
-      <c r="E14" s="76"/>
-    </row>
-    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="82" t="s">
+      <c r="B15" s="77"/>
+      <c r="C15" s="82" t="s">
         <v>330</v>
       </c>
-      <c r="B15" s="75"/>
-      <c r="C15" s="83" t="s">
-        <v>331</v>
-      </c>
-      <c r="D15" s="76"/>
-      <c r="E15" s="76"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="74"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="43" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="42"/>
       <c r="B19" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C10:E10"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="A1:E1"/>
@@ -10012,6 +10005,13 @@
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C6:E6"/>
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C10:E10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -10019,12 +10019,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10269,20 +10271,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CBE187-A7DE-4A9A-99BE-7485C92477B0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10307,18 +10316,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CBE187-A7DE-4A9A-99BE-7485C92477B0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
modified:   excel_data/Innovation_Fund_Projects_data - 130426.xlsx 	modified:   src/App.jsx 	modified:   src/components/FilterPanel.jsx
</commit_message>
<xml_diff>
--- a/excel_data/Innovation_Fund_Projects_data - 130426.xlsx
+++ b/excel_data/Innovation_Fund_Projects_data - 130426.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zeplatform-my.sharepoint.com/personal/salman_muhammad_zeplatform_eu/Documents/Technical/IF mapping tool/if-map/excel_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1790" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A41B1BE-6973-455B-805E-E10DDD73ADBA}"/>
+  <xr:revisionPtr revIDLastSave="1797" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{528203D4-1F04-44F9-875B-BFE978B1697C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -693,7 +693,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1303" uniqueCount="597">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1303" uniqueCount="595">
   <si>
     <t>EU Innovation Fund — CCS/CCU Project Portfolio Summary</t>
   </si>
@@ -2432,9 +2432,6 @@
     <t>Closed-loop biogas system with anaerobic digestion of agricultural and food waste, followed by biomethane upgrading (gas purification) and integrated CO₂ capture and liquefaction; biomethane is injected into the gas grid and partially used on-site for energy, while captured biogenic CO₂ is purified for reuse.</t>
   </si>
   <si>
-    <t>CO₂ transport and export terminal</t>
-  </si>
-  <si>
     <t>Revythoussa/Revithoussa Island, Gulf of Pachi, Megara, Attica, Greece</t>
   </si>
   <si>
@@ -2445,9 +2442,6 @@
   </si>
   <si>
     <t>Onshore CO₂ Storage</t>
-  </si>
-  <si>
-    <t>CO₂ Shipping</t>
   </si>
   <si>
     <t>Carbon Removal (BECCS)</t>
@@ -3082,36 +3076,27 @@
     <xf numFmtId="0" fontId="3" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3133,6 +3118,15 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3454,40 +3448,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="79" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74"/>
-      <c r="D1" s="74"/>
-      <c r="E1" s="74"/>
-      <c r="F1" s="74"/>
-      <c r="G1" s="74"/>
-      <c r="H1" s="74"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="74"/>
-      <c r="D2" s="74"/>
-      <c r="E2" s="74"/>
-      <c r="F2" s="74"/>
-      <c r="G2" s="74"/>
-      <c r="H2" s="74"/>
+      <c r="B2" s="76"/>
+      <c r="C2" s="76"/>
+      <c r="D2" s="76"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="76"/>
+      <c r="G2" s="76"/>
+      <c r="H2" s="76"/>
     </row>
     <row r="4" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="73" t="s">
+      <c r="A4" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="74"/>
-      <c r="C4" s="74"/>
-      <c r="D4" s="74"/>
-      <c r="E4" s="74"/>
-      <c r="F4" s="74"/>
-      <c r="G4" s="74"/>
-      <c r="H4" s="74"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="76"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="76"/>
+      <c r="F4" s="76"/>
+      <c r="G4" s="76"/>
+      <c r="H4" s="76"/>
     </row>
     <row r="5" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3504,12 +3498,12 @@
       <c r="B6" s="3">
         <v>62</v>
       </c>
-      <c r="C6" s="74"/>
-      <c r="D6" s="74"/>
-      <c r="E6" s="74"/>
-      <c r="F6" s="74"/>
-      <c r="G6" s="74"/>
-      <c r="H6" s="74"/>
+      <c r="C6" s="76"/>
+      <c r="D6" s="76"/>
+      <c r="E6" s="76"/>
+      <c r="F6" s="76"/>
+      <c r="G6" s="76"/>
+      <c r="H6" s="76"/>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
@@ -3518,12 +3512,12 @@
       <c r="B7" s="5">
         <v>16</v>
       </c>
-      <c r="C7" s="74"/>
-      <c r="D7" s="74"/>
-      <c r="E7" s="74"/>
-      <c r="F7" s="74"/>
-      <c r="G7" s="74"/>
-      <c r="H7" s="74"/>
+      <c r="C7" s="76"/>
+      <c r="D7" s="76"/>
+      <c r="E7" s="76"/>
+      <c r="F7" s="76"/>
+      <c r="G7" s="76"/>
+      <c r="H7" s="76"/>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -3532,12 +3526,12 @@
       <c r="B8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="74"/>
-      <c r="D8" s="74"/>
-      <c r="E8" s="74"/>
-      <c r="F8" s="74"/>
-      <c r="G8" s="74"/>
-      <c r="H8" s="74"/>
+      <c r="C8" s="76"/>
+      <c r="D8" s="76"/>
+      <c r="E8" s="76"/>
+      <c r="F8" s="76"/>
+      <c r="G8" s="76"/>
+      <c r="H8" s="76"/>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
@@ -3546,12 +3540,12 @@
       <c r="B9" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="74"/>
-      <c r="D9" s="74"/>
-      <c r="E9" s="74"/>
-      <c r="F9" s="74"/>
-      <c r="G9" s="74"/>
-      <c r="H9" s="74"/>
+      <c r="C9" s="76"/>
+      <c r="D9" s="76"/>
+      <c r="E9" s="76"/>
+      <c r="F9" s="76"/>
+      <c r="G9" s="76"/>
+      <c r="H9" s="76"/>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -3560,12 +3554,12 @@
       <c r="B10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="74"/>
-      <c r="D10" s="74"/>
-      <c r="E10" s="74"/>
-      <c r="F10" s="74"/>
-      <c r="G10" s="74"/>
-      <c r="H10" s="74"/>
+      <c r="C10" s="76"/>
+      <c r="D10" s="76"/>
+      <c r="E10" s="76"/>
+      <c r="F10" s="76"/>
+      <c r="G10" s="76"/>
+      <c r="H10" s="76"/>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
@@ -3574,12 +3568,12 @@
       <c r="B11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="74"/>
-      <c r="D11" s="74"/>
-      <c r="E11" s="74"/>
-      <c r="F11" s="74"/>
-      <c r="G11" s="74"/>
-      <c r="H11" s="74"/>
+      <c r="C11" s="76"/>
+      <c r="D11" s="76"/>
+      <c r="E11" s="76"/>
+      <c r="F11" s="76"/>
+      <c r="G11" s="76"/>
+      <c r="H11" s="76"/>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
@@ -3588,24 +3582,24 @@
       <c r="B12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="74"/>
-      <c r="D12" s="74"/>
-      <c r="E12" s="74"/>
-      <c r="F12" s="74"/>
-      <c r="G12" s="74"/>
-      <c r="H12" s="74"/>
+      <c r="C12" s="76"/>
+      <c r="D12" s="76"/>
+      <c r="E12" s="76"/>
+      <c r="F12" s="76"/>
+      <c r="G12" s="76"/>
+      <c r="H12" s="76"/>
     </row>
     <row r="15" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="73" t="s">
+      <c r="A15" s="78" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="74"/>
-      <c r="C15" s="74"/>
-      <c r="D15" s="74"/>
-      <c r="E15" s="74"/>
-      <c r="F15" s="74"/>
-      <c r="G15" s="74"/>
-      <c r="H15" s="74"/>
+      <c r="B15" s="76"/>
+      <c r="C15" s="76"/>
+      <c r="D15" s="76"/>
+      <c r="E15" s="76"/>
+      <c r="F15" s="76"/>
+      <c r="G15" s="76"/>
+      <c r="H15" s="76"/>
     </row>
     <row r="16" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -3617,11 +3611,11 @@
       <c r="C16" s="80" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="76"/>
-      <c r="E16" s="76"/>
-      <c r="F16" s="76"/>
-      <c r="G16" s="76"/>
-      <c r="H16" s="77"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="74"/>
+      <c r="H16" s="75"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
@@ -3630,14 +3624,14 @@
       <c r="B17" s="9">
         <v>21</v>
       </c>
-      <c r="C17" s="75" t="s">
+      <c r="C17" s="73" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="76"/>
-      <c r="E17" s="76"/>
-      <c r="F17" s="76"/>
-      <c r="G17" s="76"/>
-      <c r="H17" s="77"/>
+      <c r="D17" s="74"/>
+      <c r="E17" s="74"/>
+      <c r="F17" s="74"/>
+      <c r="G17" s="74"/>
+      <c r="H17" s="75"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
@@ -3646,14 +3640,14 @@
       <c r="B18" s="11">
         <v>20</v>
       </c>
-      <c r="C18" s="79" t="s">
+      <c r="C18" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="76"/>
-      <c r="E18" s="76"/>
-      <c r="F18" s="76"/>
-      <c r="G18" s="76"/>
-      <c r="H18" s="77"/>
+      <c r="D18" s="74"/>
+      <c r="E18" s="74"/>
+      <c r="F18" s="74"/>
+      <c r="G18" s="74"/>
+      <c r="H18" s="75"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -3662,14 +3656,14 @@
       <c r="B19" s="13">
         <v>10</v>
       </c>
-      <c r="C19" s="75" t="s">
+      <c r="C19" s="73" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="76"/>
-      <c r="E19" s="76"/>
-      <c r="F19" s="76"/>
-      <c r="G19" s="76"/>
-      <c r="H19" s="77"/>
+      <c r="D19" s="74"/>
+      <c r="E19" s="74"/>
+      <c r="F19" s="74"/>
+      <c r="G19" s="74"/>
+      <c r="H19" s="75"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
@@ -3678,14 +3672,14 @@
       <c r="B20" s="15">
         <v>4</v>
       </c>
-      <c r="C20" s="79" t="s">
+      <c r="C20" s="77" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="76"/>
-      <c r="E20" s="76"/>
-      <c r="F20" s="76"/>
-      <c r="G20" s="76"/>
-      <c r="H20" s="77"/>
+      <c r="D20" s="74"/>
+      <c r="E20" s="74"/>
+      <c r="F20" s="74"/>
+      <c r="G20" s="74"/>
+      <c r="H20" s="75"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
@@ -3694,14 +3688,14 @@
       <c r="B21" s="17">
         <v>3</v>
       </c>
-      <c r="C21" s="75" t="s">
+      <c r="C21" s="73" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="76"/>
-      <c r="E21" s="76"/>
-      <c r="F21" s="76"/>
-      <c r="G21" s="76"/>
-      <c r="H21" s="77"/>
+      <c r="D21" s="74"/>
+      <c r="E21" s="74"/>
+      <c r="F21" s="74"/>
+      <c r="G21" s="74"/>
+      <c r="H21" s="75"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="16" t="s">
@@ -3710,14 +3704,14 @@
       <c r="B22" s="17">
         <v>1</v>
       </c>
-      <c r="C22" s="79" t="s">
+      <c r="C22" s="77" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="76"/>
-      <c r="E22" s="76"/>
-      <c r="F22" s="76"/>
-      <c r="G22" s="76"/>
-      <c r="H22" s="77"/>
+      <c r="D22" s="74"/>
+      <c r="E22" s="74"/>
+      <c r="F22" s="74"/>
+      <c r="G22" s="74"/>
+      <c r="H22" s="75"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="16" t="s">
@@ -3726,14 +3720,14 @@
       <c r="B23" s="17">
         <v>1</v>
       </c>
-      <c r="C23" s="75" t="s">
+      <c r="C23" s="73" t="s">
         <v>34</v>
       </c>
-      <c r="D23" s="76"/>
-      <c r="E23" s="76"/>
-      <c r="F23" s="76"/>
-      <c r="G23" s="76"/>
-      <c r="H23" s="77"/>
+      <c r="D23" s="74"/>
+      <c r="E23" s="74"/>
+      <c r="F23" s="74"/>
+      <c r="G23" s="74"/>
+      <c r="H23" s="75"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="s">
@@ -3742,14 +3736,14 @@
       <c r="B24" s="19">
         <v>1</v>
       </c>
-      <c r="C24" s="79" t="s">
+      <c r="C24" s="77" t="s">
         <v>36</v>
       </c>
-      <c r="D24" s="76"/>
-      <c r="E24" s="76"/>
-      <c r="F24" s="76"/>
-      <c r="G24" s="76"/>
-      <c r="H24" s="77"/>
+      <c r="D24" s="74"/>
+      <c r="E24" s="74"/>
+      <c r="F24" s="74"/>
+      <c r="G24" s="74"/>
+      <c r="H24" s="75"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="20" t="s">
@@ -3758,26 +3752,26 @@
       <c r="B25" s="21">
         <v>1</v>
       </c>
-      <c r="C25" s="75" t="s">
+      <c r="C25" s="73" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="76"/>
-      <c r="E25" s="76"/>
-      <c r="F25" s="76"/>
-      <c r="G25" s="76"/>
-      <c r="H25" s="77"/>
+      <c r="D25" s="74"/>
+      <c r="E25" s="74"/>
+      <c r="F25" s="74"/>
+      <c r="G25" s="74"/>
+      <c r="H25" s="75"/>
     </row>
     <row r="28" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="73" t="s">
+      <c r="A28" s="78" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="74"/>
-      <c r="C28" s="74"/>
-      <c r="D28" s="74"/>
-      <c r="E28" s="74"/>
-      <c r="F28" s="74"/>
-      <c r="G28" s="74"/>
-      <c r="H28" s="74"/>
+      <c r="B28" s="76"/>
+      <c r="C28" s="76"/>
+      <c r="D28" s="76"/>
+      <c r="E28" s="76"/>
+      <c r="F28" s="76"/>
+      <c r="G28" s="76"/>
+      <c r="H28" s="76"/>
     </row>
     <row r="29" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -3921,12 +3915,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C23:H23"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="C19:H19"/>
     <mergeCell ref="A1:H1"/>
@@ -3943,6 +3931,12 @@
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="C6:H6"/>
     <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4152,7 +4146,7 @@
         <v>139</v>
       </c>
       <c r="Z2" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA2" s="30" t="s">
         <v>140</v>
@@ -4247,7 +4241,7 @@
         <v>392</v>
       </c>
       <c r="Z3" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA3" s="30" t="s">
         <v>92</v>
@@ -4342,7 +4336,7 @@
         <v>339</v>
       </c>
       <c r="Z4" s="34" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="AA4" s="34" t="s">
         <v>289</v>
@@ -4437,7 +4431,7 @@
         <v>177</v>
       </c>
       <c r="Z5" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA5" s="30" t="s">
         <v>178</v>
@@ -4532,7 +4526,7 @@
         <v>92</v>
       </c>
       <c r="Z6" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA6" s="30" t="s">
         <v>280</v>
@@ -4627,7 +4621,7 @@
         <v>334</v>
       </c>
       <c r="Z7" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA7" s="30" t="s">
         <v>133</v>
@@ -4722,7 +4716,7 @@
         <v>123</v>
       </c>
       <c r="Z8" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA8" s="30" t="s">
         <v>124</v>
@@ -4750,8 +4744,8 @@
       <c r="C9" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="D9" s="34" t="s">
-        <v>574</v>
+      <c r="D9" s="4" t="s">
+        <v>366</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>50</v>
@@ -4814,10 +4808,10 @@
         <v>95</v>
       </c>
       <c r="Y9" s="34" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="Z9" s="34" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="AA9" s="34" t="s">
         <v>226</v>
@@ -4826,7 +4820,7 @@
         <v>367</v>
       </c>
       <c r="AC9" s="34" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="AD9" s="34" t="s">
         <v>227</v>
@@ -4846,7 +4840,7 @@
         <v>357</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>58</v>
@@ -4912,7 +4906,7 @@
         <v>306</v>
       </c>
       <c r="Z10" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA10" s="30" t="s">
         <v>307</v>
@@ -5007,7 +5001,7 @@
         <v>421</v>
       </c>
       <c r="Z11" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA11" s="30" t="s">
         <v>267</v>
@@ -5102,7 +5096,7 @@
         <v>194</v>
       </c>
       <c r="Z12" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA12" s="34" t="s">
         <v>195</v>
@@ -5114,7 +5108,7 @@
         <v>424</v>
       </c>
       <c r="AD12" s="34" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="AE12" s="64" t="s">
         <v>568</v>
@@ -5197,7 +5191,7 @@
         <v>381</v>
       </c>
       <c r="Z13" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA13" s="34" t="s">
         <v>167</v>
@@ -5223,7 +5217,7 @@
         <v>246</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="D14" s="34" t="s">
         <v>109</v>
@@ -5292,7 +5286,7 @@
         <v>248</v>
       </c>
       <c r="Z14" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA14" s="34" t="s">
         <v>413</v>
@@ -5387,7 +5381,7 @@
         <v>176</v>
       </c>
       <c r="Z15" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA15" s="34"/>
       <c r="AB15" s="46" t="s">
@@ -5480,7 +5474,7 @@
         <v>430</v>
       </c>
       <c r="Z16" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA16" s="30" t="s">
         <v>286</v>
@@ -5575,7 +5569,7 @@
         <v>434</v>
       </c>
       <c r="Z17" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA17" s="30" t="s">
         <v>254</v>
@@ -5670,7 +5664,7 @@
         <v>206</v>
       </c>
       <c r="Z18" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA18" s="30" t="s">
         <v>207</v>
@@ -5765,7 +5759,7 @@
         <v>104</v>
       </c>
       <c r="Z19" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA19" s="34" t="s">
         <v>105</v>
@@ -5794,7 +5788,7 @@
         <v>366</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>49</v>
@@ -5860,7 +5854,7 @@
         <v>238</v>
       </c>
       <c r="Z20" s="34" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="AA20" s="34" t="s">
         <v>239</v>
@@ -5888,8 +5882,8 @@
       <c r="C21" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="D21" s="34" t="s">
-        <v>579</v>
+      <c r="D21" s="4" t="s">
+        <v>366</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>52</v>
@@ -5955,7 +5949,7 @@
         <v>438</v>
       </c>
       <c r="Z21" s="34" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="AA21" s="34" t="s">
         <v>303</v>
@@ -6050,7 +6044,7 @@
         <v>444</v>
       </c>
       <c r="Z22" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA22" s="30" t="s">
         <v>245</v>
@@ -6145,7 +6139,7 @@
         <v>449</v>
       </c>
       <c r="Z23" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA23" s="34" t="s">
         <v>233</v>
@@ -6240,7 +6234,7 @@
         <v>459</v>
       </c>
       <c r="Z24" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA24" s="34" t="s">
         <v>181</v>
@@ -6332,13 +6326,13 @@
         <v>244</v>
       </c>
       <c r="Y25" s="34" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="Z25" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA25" s="34" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="AB25" s="46" t="s">
         <v>451</v>
@@ -6361,7 +6355,7 @@
         <v>258</v>
       </c>
       <c r="C26" s="34" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="D26" s="34" t="s">
         <v>150</v>
@@ -6430,7 +6424,7 @@
         <v>454</v>
       </c>
       <c r="Z26" s="34" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="AA26" s="34" t="s">
         <v>260</v>
@@ -6439,10 +6433,10 @@
         <v>261</v>
       </c>
       <c r="AC26" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="AD26" s="34" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="AE26" s="60" t="s">
         <v>565</v>
@@ -6525,7 +6519,7 @@
         <v>464</v>
       </c>
       <c r="Z27" s="30" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="AA27" s="30" t="s">
         <v>171</v>
@@ -6620,7 +6614,7 @@
         <v>465</v>
       </c>
       <c r="Z28" s="30" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="AA28" s="30" t="s">
         <v>148</v>
@@ -6715,7 +6709,7 @@
         <v>469</v>
       </c>
       <c r="Z29" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA29" s="30" t="s">
         <v>198</v>
@@ -6741,7 +6735,7 @@
         <v>496</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="D30" s="34" t="s">
         <v>572</v>
@@ -6810,7 +6804,7 @@
         <v>495</v>
       </c>
       <c r="Z30" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA30" s="34" t="s">
         <v>313</v>
@@ -6905,7 +6899,7 @@
         <v>201</v>
       </c>
       <c r="Z31" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA31" s="34" t="s">
         <v>202</v>
@@ -7000,7 +6994,7 @@
         <v>472</v>
       </c>
       <c r="Z32" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA32" s="34" t="s">
         <v>276</v>
@@ -7095,7 +7089,7 @@
         <v>112</v>
       </c>
       <c r="Z33" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA33" s="30" t="s">
         <v>113</v>
@@ -7188,7 +7182,7 @@
         <v>477</v>
       </c>
       <c r="Z34" s="30" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="AA34" s="30" t="s">
         <v>292</v>
@@ -7283,7 +7277,7 @@
         <v>144</v>
       </c>
       <c r="Z35" s="34" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="AA35" s="34" t="s">
         <v>145</v>
@@ -7309,7 +7303,7 @@
         <v>114</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="D36" s="34" t="s">
         <v>109</v>
@@ -7378,7 +7372,7 @@
         <v>481</v>
       </c>
       <c r="Z36" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA36" s="34" t="s">
         <v>118</v>
@@ -7473,7 +7467,7 @@
         <v>284</v>
       </c>
       <c r="Z37" s="34" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="AA37" s="34" t="s">
         <v>285</v>
@@ -7568,7 +7562,7 @@
         <v>406</v>
       </c>
       <c r="Z38" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA38" s="34" t="s">
         <v>217</v>
@@ -7594,7 +7588,7 @@
         <v>309</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="D39" s="34" t="s">
         <v>109</v>
@@ -7661,7 +7655,7 @@
         <v>395</v>
       </c>
       <c r="Z39" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA39" s="30" t="s">
         <v>311</v>
@@ -7756,7 +7750,7 @@
         <v>221</v>
       </c>
       <c r="Z40" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA40" s="30" t="s">
         <v>222</v>
@@ -7851,7 +7845,7 @@
         <v>96</v>
       </c>
       <c r="Z41" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA41" s="30" t="s">
         <v>97</v>
@@ -7946,7 +7940,7 @@
         <v>136</v>
       </c>
       <c r="Z42" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA42" s="34" t="s">
         <v>134</v>
@@ -7975,7 +7969,7 @@
         <v>377</v>
       </c>
       <c r="D43" s="30" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>43</v>
@@ -8041,7 +8035,7 @@
         <v>257</v>
       </c>
       <c r="Z43" s="34" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="AA43" s="34" t="s">
         <v>92</v>
@@ -8136,7 +8130,7 @@
         <v>500</v>
       </c>
       <c r="Z44" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA44" s="34" t="s">
         <v>129</v>
@@ -8165,7 +8159,7 @@
         <v>357</v>
       </c>
       <c r="D45" s="34" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>46</v>
@@ -8326,7 +8320,7 @@
         <v>214</v>
       </c>
       <c r="Z46" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA46" s="30" t="s">
         <v>215</v>
@@ -8421,7 +8415,7 @@
         <v>154</v>
       </c>
       <c r="Z47" s="30" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="AA47" s="30" t="s">
         <v>155</v>
@@ -8516,7 +8510,7 @@
         <v>350</v>
       </c>
       <c r="Z48" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA48" s="34" t="s">
         <v>308</v>
@@ -8611,7 +8605,7 @@
         <v>151</v>
       </c>
       <c r="Z49" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA49" s="34" t="s">
         <v>152</v>
@@ -8789,7 +8783,7 @@
         <v>528</v>
       </c>
       <c r="Z51" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA51" s="30" t="s">
         <v>184</v>
@@ -8884,7 +8878,7 @@
         <v>158</v>
       </c>
       <c r="Z52" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA52" s="34" t="s">
         <v>159</v>
@@ -8979,7 +8973,7 @@
         <v>531</v>
       </c>
       <c r="Z53" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA53" s="30" t="s">
         <v>236</v>
@@ -9005,7 +8999,7 @@
         <v>272</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="D54" s="30" t="s">
         <v>572</v>
@@ -9074,7 +9068,7 @@
         <v>541</v>
       </c>
       <c r="Z54" s="30" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA54" s="30" t="s">
         <v>273</v>
@@ -9103,7 +9097,7 @@
         <v>377</v>
       </c>
       <c r="D55" s="30" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>46</v>
@@ -9169,7 +9163,7 @@
         <v>543</v>
       </c>
       <c r="Z55" s="30" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="AA55" s="30"/>
       <c r="AB55" s="46" t="s">
@@ -9262,7 +9256,7 @@
         <v>546</v>
       </c>
       <c r="Z56" s="30" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="AA56" s="30" t="s">
         <v>191</v>
@@ -9291,7 +9285,7 @@
         <v>377</v>
       </c>
       <c r="D57" s="30" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>52</v>
@@ -9357,7 +9351,7 @@
         <v>551</v>
       </c>
       <c r="Z57" s="30" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="AA57" s="30" t="s">
         <v>300</v>
@@ -9386,7 +9380,7 @@
         <v>225</v>
       </c>
       <c r="D58" s="34" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>50</v>
@@ -9547,7 +9541,7 @@
         <v>554</v>
       </c>
       <c r="Z59" s="34" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="AA59" s="34" t="s">
         <v>296</v>
@@ -9642,7 +9636,7 @@
         <v>187</v>
       </c>
       <c r="Z60" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA60" s="34" t="s">
         <v>188</v>
@@ -9671,7 +9665,7 @@
         <v>242</v>
       </c>
       <c r="D61" s="34" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="E61" s="4" t="s">
         <v>46</v>
@@ -9840,141 +9834,141 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="84" t="s">
         <v>314</v>
       </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74"/>
-      <c r="D1" s="74"/>
-      <c r="E1" s="74"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="73" t="s">
+      <c r="A3" s="78" t="s">
         <v>315</v>
       </c>
-      <c r="B3" s="74"/>
-      <c r="C3" s="74"/>
-      <c r="D3" s="74"/>
-      <c r="E3" s="74"/>
+      <c r="B3" s="76"/>
+      <c r="C3" s="76"/>
+      <c r="D3" s="76"/>
+      <c r="E3" s="76"/>
     </row>
     <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="93" t="s">
+      <c r="A4" s="90" t="s">
         <v>316</v>
       </c>
-      <c r="B4" s="77"/>
-      <c r="C4" s="82" t="s">
+      <c r="B4" s="75"/>
+      <c r="C4" s="83" t="s">
         <v>317</v>
       </c>
-      <c r="D4" s="74"/>
-      <c r="E4" s="74"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="76"/>
     </row>
     <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="90" t="s">
+      <c r="A5" s="87" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="77"/>
-      <c r="C5" s="82" t="s">
+      <c r="B5" s="75"/>
+      <c r="C5" s="83" t="s">
         <v>318</v>
       </c>
-      <c r="D5" s="74"/>
-      <c r="E5" s="74"/>
+      <c r="D5" s="76"/>
+      <c r="E5" s="76"/>
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="88" t="s">
+      <c r="A6" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="77"/>
-      <c r="C6" s="82" t="s">
+      <c r="B6" s="75"/>
+      <c r="C6" s="83" t="s">
         <v>319</v>
       </c>
-      <c r="D6" s="74"/>
-      <c r="E6" s="74"/>
+      <c r="D6" s="76"/>
+      <c r="E6" s="76"/>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="89" t="s">
+      <c r="A7" s="86" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="77"/>
-      <c r="C7" s="82" t="s">
+      <c r="B7" s="75"/>
+      <c r="C7" s="83" t="s">
         <v>320</v>
       </c>
-      <c r="D7" s="74"/>
-      <c r="E7" s="74"/>
+      <c r="D7" s="76"/>
+      <c r="E7" s="76"/>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="92" t="s">
+      <c r="A8" s="89" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="77"/>
-      <c r="C8" s="82" t="s">
+      <c r="B8" s="75"/>
+      <c r="C8" s="83" t="s">
         <v>321</v>
       </c>
-      <c r="D8" s="74"/>
-      <c r="E8" s="74"/>
+      <c r="D8" s="76"/>
+      <c r="E8" s="76"/>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="85" t="s">
+      <c r="A9" s="93" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="77"/>
-      <c r="C9" s="82" t="s">
+      <c r="B9" s="75"/>
+      <c r="C9" s="83" t="s">
         <v>322</v>
       </c>
-      <c r="D9" s="74"/>
-      <c r="E9" s="74"/>
+      <c r="D9" s="76"/>
+      <c r="E9" s="76"/>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="83" t="s">
+      <c r="A10" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="77"/>
-      <c r="C10" s="82" t="s">
+      <c r="B10" s="75"/>
+      <c r="C10" s="83" t="s">
         <v>323</v>
       </c>
-      <c r="D10" s="74"/>
-      <c r="E10" s="74"/>
+      <c r="D10" s="76"/>
+      <c r="E10" s="76"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="73" t="s">
+      <c r="A12" s="78" t="s">
         <v>324</v>
       </c>
-      <c r="B12" s="74"/>
-      <c r="C12" s="74"/>
-      <c r="D12" s="74"/>
-      <c r="E12" s="74"/>
+      <c r="B12" s="76"/>
+      <c r="C12" s="76"/>
+      <c r="D12" s="76"/>
+      <c r="E12" s="76"/>
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="84" t="s">
+      <c r="A13" s="92" t="s">
         <v>325</v>
       </c>
-      <c r="B13" s="77"/>
-      <c r="C13" s="82" t="s">
+      <c r="B13" s="75"/>
+      <c r="C13" s="83" t="s">
         <v>326</v>
       </c>
-      <c r="D13" s="74"/>
-      <c r="E13" s="74"/>
+      <c r="D13" s="76"/>
+      <c r="E13" s="76"/>
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="91" t="s">
+      <c r="A14" s="88" t="s">
         <v>327</v>
       </c>
-      <c r="B14" s="77"/>
-      <c r="C14" s="82" t="s">
+      <c r="B14" s="75"/>
+      <c r="C14" s="83" t="s">
         <v>328</v>
       </c>
-      <c r="D14" s="74"/>
-      <c r="E14" s="74"/>
+      <c r="D14" s="76"/>
+      <c r="E14" s="76"/>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="86" t="s">
+      <c r="A15" s="82" t="s">
         <v>329</v>
       </c>
-      <c r="B15" s="77"/>
-      <c r="C15" s="82" t="s">
+      <c r="B15" s="75"/>
+      <c r="C15" s="83" t="s">
         <v>330</v>
       </c>
-      <c r="D15" s="74"/>
-      <c r="E15" s="74"/>
+      <c r="D15" s="76"/>
+      <c r="E15" s="76"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="43" t="s">
@@ -9989,6 +9983,13 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C10:E10"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="A1:E1"/>
@@ -10005,13 +10006,6 @@
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C6:E6"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C10:E10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -10019,14 +10013,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10271,27 +10263,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CBE187-A7DE-4A9A-99BE-7485C92477B0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10316,9 +10301,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CBE187-A7DE-4A9A-99BE-7485C92477B0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
modified:   excel_data/innovation_fund_projects_data - 130426.xlsx 	new file:   public/logotype_cme_fullwhite.png 	modified:   public/data/meta.json 	modified:   public/data/projects.json 	modified:   src/app.jsx 	modified:   src/components/disclaimer.jsx 	modified:   src/components/filterpanel.jsx 	modified:   src/components/filterpanel.module.css 	modified:   src/components/mapview.jsx 	modified:   src/components/statsbar.jsx 	modified:   src/components/statsbar.module.css 	modified:   src/constants.js
</commit_message>
<xml_diff>
--- a/excel_data/Innovation_Fund_Projects_data - 130426.xlsx
+++ b/excel_data/Innovation_Fund_Projects_data - 130426.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zeplatform-my.sharepoint.com/personal/salman_muhammad_zeplatform_eu/Documents/Technical/IF mapping tool/if-map/excel_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1797" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{528203D4-1F04-44F9-875B-BFE978B1697C}"/>
+  <xr:revisionPtr revIDLastSave="1813" documentId="11_1EE5EEA0CB77697A79955972BEC118078624C068" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42BF5FE0-E1C9-4F87-B840-6F6B20D24AF8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -693,7 +693,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1303" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1300" uniqueCount="594">
   <si>
     <t>EU Innovation Fund — CCS/CCU Project Portfolio Summary</t>
   </si>
@@ -1798,9 +1798,6 @@
     <t>Hybrid staged CO₂ capture system combining oxyfuel combustion (OxyCal) and post-combustion amine scrubbing. Achieving up to ~99% capture efficiency; CO₂ is processed via a CO₂ Processing Unit (CPU), transported by pipeline, and permanently stored in the depleted Galata gas field under the Black Sea.</t>
   </si>
   <si>
-    <t>Not Acquired</t>
-  </si>
-  <si>
     <t>https://www.anthemis-ccs.com/en/about-the-project</t>
   </si>
   <si>
@@ -1970,9 +1967,6 @@
     <t>Biovind AS</t>
   </si>
   <si>
-    <t>Not Available</t>
-  </si>
-  <si>
     <t>Store Nerheim, 5580 Ølen, Vindafjord, Rogaland, Norway</t>
   </si>
   <si>
@@ -2493,6 +2487,9 @@
   </si>
   <si>
     <t>Oxyfuel combustion + Carbon Processing Unit (CPU) CO₂ capture at Holcim Lägerdorf cement plant; CO₂ utilised in thyssenkrupp/Linde CPU to produce industrial chemicals (methanol, plastics precursors) — CCU/conversion utilisation; ~1.3 Mt/yr</t>
+  </si>
+  <si>
+    <t>CO₂ transport and storage</t>
   </si>
 </sst>
 </file>
@@ -2648,6 +2645,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="25">
@@ -3076,27 +3074,36 @@
     <xf numFmtId="0" fontId="3" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3118,15 +3125,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3448,40 +3446,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="79" t="s">
+      <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
+      <c r="F1" s="74"/>
+      <c r="G1" s="74"/>
+      <c r="H1" s="74"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="76"/>
-      <c r="C2" s="76"/>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="76"/>
+      <c r="B2" s="74"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="74"/>
+      <c r="G2" s="74"/>
+      <c r="H2" s="74"/>
     </row>
     <row r="4" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="78" t="s">
+      <c r="A4" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="76"/>
-      <c r="C4" s="76"/>
-      <c r="D4" s="76"/>
-      <c r="E4" s="76"/>
-      <c r="F4" s="76"/>
-      <c r="G4" s="76"/>
-      <c r="H4" s="76"/>
+      <c r="B4" s="74"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="74"/>
+      <c r="F4" s="74"/>
+      <c r="G4" s="74"/>
+      <c r="H4" s="74"/>
     </row>
     <row r="5" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3498,12 +3496,12 @@
       <c r="B6" s="3">
         <v>62</v>
       </c>
-      <c r="C6" s="76"/>
-      <c r="D6" s="76"/>
-      <c r="E6" s="76"/>
-      <c r="F6" s="76"/>
-      <c r="G6" s="76"/>
-      <c r="H6" s="76"/>
+      <c r="C6" s="74"/>
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="74"/>
+      <c r="G6" s="74"/>
+      <c r="H6" s="74"/>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
@@ -3512,12 +3510,12 @@
       <c r="B7" s="5">
         <v>16</v>
       </c>
-      <c r="C7" s="76"/>
-      <c r="D7" s="76"/>
-      <c r="E7" s="76"/>
-      <c r="F7" s="76"/>
-      <c r="G7" s="76"/>
-      <c r="H7" s="76"/>
+      <c r="C7" s="74"/>
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
+      <c r="F7" s="74"/>
+      <c r="G7" s="74"/>
+      <c r="H7" s="74"/>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -3526,12 +3524,12 @@
       <c r="B8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="76"/>
-      <c r="D8" s="76"/>
-      <c r="E8" s="76"/>
-      <c r="F8" s="76"/>
-      <c r="G8" s="76"/>
-      <c r="H8" s="76"/>
+      <c r="C8" s="74"/>
+      <c r="D8" s="74"/>
+      <c r="E8" s="74"/>
+      <c r="F8" s="74"/>
+      <c r="G8" s="74"/>
+      <c r="H8" s="74"/>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
@@ -3540,12 +3538,12 @@
       <c r="B9" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="76"/>
-      <c r="D9" s="76"/>
-      <c r="E9" s="76"/>
-      <c r="F9" s="76"/>
-      <c r="G9" s="76"/>
-      <c r="H9" s="76"/>
+      <c r="C9" s="74"/>
+      <c r="D9" s="74"/>
+      <c r="E9" s="74"/>
+      <c r="F9" s="74"/>
+      <c r="G9" s="74"/>
+      <c r="H9" s="74"/>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -3554,12 +3552,12 @@
       <c r="B10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="76"/>
-      <c r="D10" s="76"/>
-      <c r="E10" s="76"/>
-      <c r="F10" s="76"/>
-      <c r="G10" s="76"/>
-      <c r="H10" s="76"/>
+      <c r="C10" s="74"/>
+      <c r="D10" s="74"/>
+      <c r="E10" s="74"/>
+      <c r="F10" s="74"/>
+      <c r="G10" s="74"/>
+      <c r="H10" s="74"/>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
@@ -3568,12 +3566,12 @@
       <c r="B11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="76"/>
-      <c r="D11" s="76"/>
-      <c r="E11" s="76"/>
-      <c r="F11" s="76"/>
-      <c r="G11" s="76"/>
-      <c r="H11" s="76"/>
+      <c r="C11" s="74"/>
+      <c r="D11" s="74"/>
+      <c r="E11" s="74"/>
+      <c r="F11" s="74"/>
+      <c r="G11" s="74"/>
+      <c r="H11" s="74"/>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
@@ -3582,24 +3580,24 @@
       <c r="B12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="76"/>
-      <c r="D12" s="76"/>
-      <c r="E12" s="76"/>
-      <c r="F12" s="76"/>
-      <c r="G12" s="76"/>
-      <c r="H12" s="76"/>
+      <c r="C12" s="74"/>
+      <c r="D12" s="74"/>
+      <c r="E12" s="74"/>
+      <c r="F12" s="74"/>
+      <c r="G12" s="74"/>
+      <c r="H12" s="74"/>
     </row>
     <row r="15" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="78" t="s">
+      <c r="A15" s="73" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="76"/>
-      <c r="C15" s="76"/>
-      <c r="D15" s="76"/>
-      <c r="E15" s="76"/>
-      <c r="F15" s="76"/>
-      <c r="G15" s="76"/>
-      <c r="H15" s="76"/>
+      <c r="B15" s="74"/>
+      <c r="C15" s="74"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="74"/>
+      <c r="F15" s="74"/>
+      <c r="G15" s="74"/>
+      <c r="H15" s="74"/>
     </row>
     <row r="16" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -3611,11 +3609,11 @@
       <c r="C16" s="80" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="74"/>
-      <c r="E16" s="74"/>
-      <c r="F16" s="74"/>
-      <c r="G16" s="74"/>
-      <c r="H16" s="75"/>
+      <c r="D16" s="76"/>
+      <c r="E16" s="76"/>
+      <c r="F16" s="76"/>
+      <c r="G16" s="76"/>
+      <c r="H16" s="77"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
@@ -3624,14 +3622,14 @@
       <c r="B17" s="9">
         <v>21</v>
       </c>
-      <c r="C17" s="73" t="s">
+      <c r="C17" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="74"/>
-      <c r="E17" s="74"/>
-      <c r="F17" s="74"/>
-      <c r="G17" s="74"/>
-      <c r="H17" s="75"/>
+      <c r="D17" s="76"/>
+      <c r="E17" s="76"/>
+      <c r="F17" s="76"/>
+      <c r="G17" s="76"/>
+      <c r="H17" s="77"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
@@ -3640,14 +3638,14 @@
       <c r="B18" s="11">
         <v>20</v>
       </c>
-      <c r="C18" s="77" t="s">
+      <c r="C18" s="79" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="74"/>
-      <c r="E18" s="74"/>
-      <c r="F18" s="74"/>
-      <c r="G18" s="74"/>
-      <c r="H18" s="75"/>
+      <c r="D18" s="76"/>
+      <c r="E18" s="76"/>
+      <c r="F18" s="76"/>
+      <c r="G18" s="76"/>
+      <c r="H18" s="77"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -3656,14 +3654,14 @@
       <c r="B19" s="13">
         <v>10</v>
       </c>
-      <c r="C19" s="73" t="s">
+      <c r="C19" s="75" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="74"/>
-      <c r="E19" s="74"/>
-      <c r="F19" s="74"/>
-      <c r="G19" s="74"/>
-      <c r="H19" s="75"/>
+      <c r="D19" s="76"/>
+      <c r="E19" s="76"/>
+      <c r="F19" s="76"/>
+      <c r="G19" s="76"/>
+      <c r="H19" s="77"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
@@ -3672,14 +3670,14 @@
       <c r="B20" s="15">
         <v>4</v>
       </c>
-      <c r="C20" s="77" t="s">
+      <c r="C20" s="79" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="74"/>
-      <c r="E20" s="74"/>
-      <c r="F20" s="74"/>
-      <c r="G20" s="74"/>
-      <c r="H20" s="75"/>
+      <c r="D20" s="76"/>
+      <c r="E20" s="76"/>
+      <c r="F20" s="76"/>
+      <c r="G20" s="76"/>
+      <c r="H20" s="77"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
@@ -3688,14 +3686,14 @@
       <c r="B21" s="17">
         <v>3</v>
       </c>
-      <c r="C21" s="73" t="s">
+      <c r="C21" s="75" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="74"/>
-      <c r="E21" s="74"/>
-      <c r="F21" s="74"/>
-      <c r="G21" s="74"/>
-      <c r="H21" s="75"/>
+      <c r="D21" s="76"/>
+      <c r="E21" s="76"/>
+      <c r="F21" s="76"/>
+      <c r="G21" s="76"/>
+      <c r="H21" s="77"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="16" t="s">
@@ -3704,14 +3702,14 @@
       <c r="B22" s="17">
         <v>1</v>
       </c>
-      <c r="C22" s="77" t="s">
+      <c r="C22" s="79" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="74"/>
-      <c r="E22" s="74"/>
-      <c r="F22" s="74"/>
-      <c r="G22" s="74"/>
-      <c r="H22" s="75"/>
+      <c r="D22" s="76"/>
+      <c r="E22" s="76"/>
+      <c r="F22" s="76"/>
+      <c r="G22" s="76"/>
+      <c r="H22" s="77"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="16" t="s">
@@ -3720,14 +3718,14 @@
       <c r="B23" s="17">
         <v>1</v>
       </c>
-      <c r="C23" s="73" t="s">
+      <c r="C23" s="75" t="s">
         <v>34</v>
       </c>
-      <c r="D23" s="74"/>
-      <c r="E23" s="74"/>
-      <c r="F23" s="74"/>
-      <c r="G23" s="74"/>
-      <c r="H23" s="75"/>
+      <c r="D23" s="76"/>
+      <c r="E23" s="76"/>
+      <c r="F23" s="76"/>
+      <c r="G23" s="76"/>
+      <c r="H23" s="77"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="s">
@@ -3736,14 +3734,14 @@
       <c r="B24" s="19">
         <v>1</v>
       </c>
-      <c r="C24" s="77" t="s">
+      <c r="C24" s="79" t="s">
         <v>36</v>
       </c>
-      <c r="D24" s="74"/>
-      <c r="E24" s="74"/>
-      <c r="F24" s="74"/>
-      <c r="G24" s="74"/>
-      <c r="H24" s="75"/>
+      <c r="D24" s="76"/>
+      <c r="E24" s="76"/>
+      <c r="F24" s="76"/>
+      <c r="G24" s="76"/>
+      <c r="H24" s="77"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="20" t="s">
@@ -3752,26 +3750,26 @@
       <c r="B25" s="21">
         <v>1</v>
       </c>
-      <c r="C25" s="73" t="s">
+      <c r="C25" s="75" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="74"/>
-      <c r="E25" s="74"/>
-      <c r="F25" s="74"/>
-      <c r="G25" s="74"/>
-      <c r="H25" s="75"/>
+      <c r="D25" s="76"/>
+      <c r="E25" s="76"/>
+      <c r="F25" s="76"/>
+      <c r="G25" s="76"/>
+      <c r="H25" s="77"/>
     </row>
     <row r="28" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="78" t="s">
+      <c r="A28" s="73" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="76"/>
-      <c r="C28" s="76"/>
-      <c r="D28" s="76"/>
-      <c r="E28" s="76"/>
-      <c r="F28" s="76"/>
-      <c r="G28" s="76"/>
-      <c r="H28" s="76"/>
+      <c r="B28" s="74"/>
+      <c r="C28" s="74"/>
+      <c r="D28" s="74"/>
+      <c r="E28" s="74"/>
+      <c r="F28" s="74"/>
+      <c r="G28" s="74"/>
+      <c r="H28" s="74"/>
     </row>
     <row r="29" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -3915,6 +3913,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="C19:H19"/>
     <mergeCell ref="A1:H1"/>
@@ -3931,12 +3935,6 @@
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="C6:H6"/>
     <mergeCell ref="C24:H24"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C23:H23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4146,7 +4144,7 @@
         <v>139</v>
       </c>
       <c r="Z2" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA2" s="30" t="s">
         <v>140</v>
@@ -4161,7 +4159,7 @@
         <v>337</v>
       </c>
       <c r="AE2" s="60" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="3" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -4169,7 +4167,7 @@
         <v>141</v>
       </c>
       <c r="B3" s="55" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>242</v>
@@ -4238,10 +4236,10 @@
         <v>95</v>
       </c>
       <c r="Y3" s="30" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="Z3" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA3" s="30" t="s">
         <v>92</v>
@@ -4250,13 +4248,13 @@
         <v>250</v>
       </c>
       <c r="AC3" s="30" t="s">
+        <v>392</v>
+      </c>
+      <c r="AD3" s="30" t="s">
         <v>393</v>
       </c>
-      <c r="AD3" s="30" t="s">
-        <v>394</v>
-      </c>
       <c r="AE3" s="61" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="4" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -4336,7 +4334,7 @@
         <v>339</v>
       </c>
       <c r="Z4" s="34" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="AA4" s="34" t="s">
         <v>289</v>
@@ -4365,7 +4363,7 @@
         <v>108</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>42</v>
@@ -4431,7 +4429,7 @@
         <v>177</v>
       </c>
       <c r="Z5" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA5" s="30" t="s">
         <v>178</v>
@@ -4446,7 +4444,7 @@
         <v>355</v>
       </c>
       <c r="AE5" s="63" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="6" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -4526,7 +4524,7 @@
         <v>92</v>
       </c>
       <c r="Z6" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA6" s="30" t="s">
         <v>280</v>
@@ -4538,10 +4536,10 @@
         <v>358</v>
       </c>
       <c r="AD6" s="30" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="AE6" s="64" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="7" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -4621,7 +4619,7 @@
         <v>334</v>
       </c>
       <c r="Z7" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA7" s="30" t="s">
         <v>133</v>
@@ -4636,7 +4634,7 @@
         <v>362</v>
       </c>
       <c r="AE7" s="63" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="8" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -4697,8 +4695,8 @@
       <c r="S8" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="T8" s="33" t="s">
-        <v>363</v>
+      <c r="T8" s="33">
+        <v>115000000</v>
       </c>
       <c r="U8" s="33" t="s">
         <v>356</v>
@@ -4716,19 +4714,19 @@
         <v>123</v>
       </c>
       <c r="Z8" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA8" s="30" t="s">
         <v>124</v>
       </c>
       <c r="AB8" s="46" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AC8" s="30" t="s">
         <v>125</v>
       </c>
       <c r="AD8" s="30" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AE8" s="63" t="s">
         <v>567</v>
@@ -4742,19 +4740,19 @@
         <v>224</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>366</v>
+        <v>593</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>50</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="H9" s="35">
         <v>2.5819174</v>
@@ -4808,25 +4806,25 @@
         <v>95</v>
       </c>
       <c r="Y9" s="34" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="Z9" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA9" s="34" t="s">
         <v>226</v>
       </c>
       <c r="AB9" s="46" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="AC9" s="34" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="AD9" s="34" t="s">
         <v>227</v>
       </c>
       <c r="AE9" s="61" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="10" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -4834,13 +4832,13 @@
         <v>87</v>
       </c>
       <c r="B10" s="55" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>357</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>58</v>
@@ -4906,19 +4904,19 @@
         <v>306</v>
       </c>
       <c r="Z10" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA10" s="30" t="s">
         <v>307</v>
       </c>
       <c r="AB10" s="46" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="AC10" s="30" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="AD10" s="30" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="AE10" s="62" t="s">
         <v>27</v>
@@ -4941,10 +4939,10 @@
         <v>46</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H11" s="31" t="s">
         <v>92</v>
@@ -4982,8 +4980,8 @@
       <c r="S11" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="T11" s="33" t="s">
-        <v>420</v>
+      <c r="T11" s="33">
+        <v>10206000</v>
       </c>
       <c r="U11" s="33" t="s">
         <v>356</v>
@@ -4998,22 +4996,22 @@
         <v>244</v>
       </c>
       <c r="Y11" s="30" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="Z11" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA11" s="30" t="s">
         <v>267</v>
       </c>
       <c r="AB11" s="46" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="AC11" s="30" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="AD11" s="30" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="AE11" s="63" t="s">
         <v>567</v>
@@ -5096,22 +5094,22 @@
         <v>194</v>
       </c>
       <c r="Z12" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA12" s="34" t="s">
         <v>195</v>
       </c>
       <c r="AB12" s="46" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="AC12" s="34" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="AD12" s="34" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="AE12" s="64" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="13" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5188,10 +5186,10 @@
         <v>95</v>
       </c>
       <c r="Y13" s="34" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="Z13" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA13" s="34" t="s">
         <v>167</v>
@@ -5200,13 +5198,13 @@
         <v>168</v>
       </c>
       <c r="AC13" s="34" t="s">
+        <v>381</v>
+      </c>
+      <c r="AD13" s="34" t="s">
         <v>382</v>
       </c>
-      <c r="AD13" s="34" t="s">
-        <v>383</v>
-      </c>
       <c r="AE13" s="60" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="14" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -5217,7 +5215,7 @@
         <v>246</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="D14" s="34" t="s">
         <v>109</v>
@@ -5286,22 +5284,22 @@
         <v>248</v>
       </c>
       <c r="Z14" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA14" s="34" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="AB14" s="46" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="AC14" s="34" t="s">
+        <v>409</v>
+      </c>
+      <c r="AD14" s="34" t="s">
         <v>410</v>
       </c>
-      <c r="AD14" s="34" t="s">
-        <v>411</v>
-      </c>
       <c r="AE14" s="64" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="15" spans="1:31" ht="148.19999999999999" x14ac:dyDescent="0.3">
@@ -5381,20 +5379,20 @@
         <v>176</v>
       </c>
       <c r="Z15" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA15" s="34"/>
       <c r="AB15" s="46" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="AC15" s="34" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="AD15" s="34" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="AE15" s="64" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="16" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5417,7 +5415,7 @@
         <v>275</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="H16" s="31" t="s">
         <v>92</v>
@@ -5455,8 +5453,8 @@
       <c r="S16" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="T16" s="33" t="s">
-        <v>420</v>
+      <c r="T16" s="33">
+        <v>146415990</v>
       </c>
       <c r="U16" s="33" t="s">
         <v>356</v>
@@ -5471,25 +5469,25 @@
         <v>244</v>
       </c>
       <c r="Y16" s="30" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="Z16" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA16" s="30" t="s">
         <v>286</v>
       </c>
       <c r="AB16" s="46" t="s">
+        <v>424</v>
+      </c>
+      <c r="AC16" s="30" t="s">
         <v>426</v>
       </c>
-      <c r="AC16" s="30" t="s">
-        <v>428</v>
-      </c>
       <c r="AD16" s="30" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="AE16" s="65" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="17" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5512,7 +5510,7 @@
         <v>253</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="H17" s="51">
         <v>4.5999999999999999E-3</v>
@@ -5566,10 +5564,10 @@
         <v>244</v>
       </c>
       <c r="Y17" s="30" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="Z17" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA17" s="30" t="s">
         <v>254</v>
@@ -5578,10 +5576,10 @@
         <v>255</v>
       </c>
       <c r="AC17" s="30" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="AD17" s="30" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="AE17" s="62" t="s">
         <v>27</v>
@@ -5664,7 +5662,7 @@
         <v>206</v>
       </c>
       <c r="Z18" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA18" s="30" t="s">
         <v>207</v>
@@ -5673,13 +5671,13 @@
         <v>208</v>
       </c>
       <c r="AC18" s="30" t="s">
+        <v>386</v>
+      </c>
+      <c r="AD18" s="30" t="s">
         <v>387</v>
       </c>
-      <c r="AD18" s="30" t="s">
-        <v>388</v>
-      </c>
       <c r="AE18" s="65" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="19" spans="1:31" ht="57" x14ac:dyDescent="0.3">
@@ -5759,13 +5757,13 @@
         <v>104</v>
       </c>
       <c r="Z19" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA19" s="34" t="s">
         <v>105</v>
       </c>
       <c r="AB19" s="46" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="AC19" s="34" t="s">
         <v>105</v>
@@ -5785,10 +5783,10 @@
         <v>237</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>49</v>
@@ -5797,7 +5795,7 @@
         <v>235</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="H20" s="35">
         <v>2.11</v>
@@ -5854,7 +5852,7 @@
         <v>238</v>
       </c>
       <c r="Z20" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA20" s="34" t="s">
         <v>239</v>
@@ -5863,13 +5861,13 @@
         <v>240</v>
       </c>
       <c r="AC20" s="34" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="AD20" s="34" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="AE20" s="66" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="21" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -5880,10 +5878,10 @@
         <v>302</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>366</v>
+        <v>593</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>52</v>
@@ -5946,25 +5944,25 @@
         <v>132</v>
       </c>
       <c r="Y21" s="30" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="Z21" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA21" s="34" t="s">
         <v>303</v>
       </c>
       <c r="AB21" s="46" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="AC21" s="34" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="AD21" s="34" t="s">
         <v>304</v>
       </c>
       <c r="AE21" s="65" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="22" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6041,25 +6039,25 @@
         <v>244</v>
       </c>
       <c r="Y22" s="29" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="Z22" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA22" s="30" t="s">
         <v>245</v>
       </c>
       <c r="AB22" s="46" t="s">
+        <v>439</v>
+      </c>
+      <c r="AC22" s="30" t="s">
+        <v>440</v>
+      </c>
+      <c r="AD22" s="30" t="s">
         <v>441</v>
       </c>
-      <c r="AC22" s="30" t="s">
-        <v>442</v>
-      </c>
-      <c r="AD22" s="30" t="s">
-        <v>443</v>
-      </c>
       <c r="AE22" s="64" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="23" spans="1:31" ht="136.80000000000001" x14ac:dyDescent="0.3">
@@ -6079,10 +6077,10 @@
         <v>57</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="H23" s="35">
         <v>0.56499999999999995</v>
@@ -6136,25 +6134,25 @@
         <v>95</v>
       </c>
       <c r="Y23" s="34" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="Z23" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA23" s="34" t="s">
         <v>233</v>
       </c>
       <c r="AB23" s="46" t="s">
+        <v>444</v>
+      </c>
+      <c r="AC23" s="34" t="s">
+        <v>445</v>
+      </c>
+      <c r="AD23" s="34" t="s">
         <v>446</v>
       </c>
-      <c r="AC23" s="34" t="s">
-        <v>447</v>
-      </c>
-      <c r="AD23" s="34" t="s">
-        <v>448</v>
-      </c>
       <c r="AE23" s="65" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="24" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6174,10 +6172,10 @@
         <v>42</v>
       </c>
       <c r="F24" s="71" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="G24" s="72" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="H24" s="35">
         <v>0.2</v>
@@ -6231,25 +6229,25 @@
         <v>180</v>
       </c>
       <c r="Y24" s="34" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="Z24" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA24" s="34" t="s">
         <v>181</v>
       </c>
       <c r="AB24" s="46" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="AC24" s="34" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="AD24" s="34" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="AE24" s="61" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="25" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -6269,10 +6267,10 @@
         <v>56</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="H25" s="35">
         <v>1</v>
@@ -6326,25 +6324,25 @@
         <v>244</v>
       </c>
       <c r="Y25" s="34" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="Z25" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA25" s="34" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="AB25" s="46" t="s">
+        <v>449</v>
+      </c>
+      <c r="AC25" s="34" t="s">
+        <v>450</v>
+      </c>
+      <c r="AD25" s="34" t="s">
         <v>451</v>
       </c>
-      <c r="AC25" s="34" t="s">
-        <v>452</v>
-      </c>
-      <c r="AD25" s="34" t="s">
-        <v>453</v>
-      </c>
       <c r="AE25" s="65" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="26" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6355,7 +6353,7 @@
         <v>258</v>
       </c>
       <c r="C26" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="D26" s="34" t="s">
         <v>150</v>
@@ -6421,10 +6419,10 @@
         <v>244</v>
       </c>
       <c r="Y26" s="34" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="Z26" s="34" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="AA26" s="34" t="s">
         <v>260</v>
@@ -6433,13 +6431,13 @@
         <v>261</v>
       </c>
       <c r="AC26" s="34" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="AD26" s="34" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="AE26" s="60" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="27" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -6462,7 +6460,7 @@
         <v>170</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="H27" s="31">
         <v>0.23252429999999999</v>
@@ -6516,10 +6514,10 @@
         <v>95</v>
       </c>
       <c r="Y27" s="30" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="Z27" s="30" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="AA27" s="30" t="s">
         <v>171</v>
@@ -6528,13 +6526,13 @@
         <v>172</v>
       </c>
       <c r="AC27" s="30" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="AD27" s="30" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="AE27" s="61" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="28" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -6548,7 +6546,7 @@
         <v>225</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>54</v>
@@ -6611,25 +6609,25 @@
         <v>132</v>
       </c>
       <c r="Y28" s="30" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="Z28" s="30" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="AA28" s="30" t="s">
         <v>148</v>
       </c>
       <c r="AB28" s="46" t="s">
+        <v>464</v>
+      </c>
+      <c r="AC28" s="30" t="s">
+        <v>465</v>
+      </c>
+      <c r="AD28" s="30" t="s">
         <v>466</v>
       </c>
-      <c r="AC28" s="30" t="s">
-        <v>467</v>
-      </c>
-      <c r="AD28" s="30" t="s">
-        <v>468</v>
-      </c>
       <c r="AE28" s="60" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="29" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -6706,10 +6704,10 @@
         <v>180</v>
       </c>
       <c r="Y29" s="30" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="Z29" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA29" s="30" t="s">
         <v>198</v>
@@ -6718,13 +6716,13 @@
         <v>199</v>
       </c>
       <c r="AC29" s="30" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="AD29" s="30" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="AE29" s="60" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="30" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6732,19 +6730,19 @@
         <v>163</v>
       </c>
       <c r="B30" s="54" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="D30" s="34" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>58</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="G30" s="4" t="s">
         <v>312</v>
@@ -6801,25 +6799,25 @@
         <v>244</v>
       </c>
       <c r="Y30" s="34" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="Z30" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA30" s="34" t="s">
         <v>313</v>
       </c>
       <c r="AB30" s="47" t="s">
+        <v>495</v>
+      </c>
+      <c r="AC30" s="34" t="s">
+        <v>496</v>
+      </c>
+      <c r="AD30" s="34" t="s">
         <v>497</v>
       </c>
-      <c r="AC30" s="34" t="s">
-        <v>498</v>
-      </c>
-      <c r="AD30" s="34" t="s">
-        <v>499</v>
-      </c>
       <c r="AE30" s="61" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="31" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6899,7 +6897,7 @@
         <v>201</v>
       </c>
       <c r="Z31" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA31" s="34" t="s">
         <v>202</v>
@@ -6908,13 +6906,13 @@
         <v>203</v>
       </c>
       <c r="AC31" s="34" t="s">
+        <v>407</v>
+      </c>
+      <c r="AD31" s="34" t="s">
         <v>408</v>
       </c>
-      <c r="AD31" s="34" t="s">
-        <v>409</v>
-      </c>
       <c r="AE31" s="60" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="32" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -6934,10 +6932,10 @@
         <v>45</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H32" s="35">
         <v>1</v>
@@ -6991,25 +6989,25 @@
         <v>95</v>
       </c>
       <c r="Y32" s="34" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="Z32" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA32" s="34" t="s">
         <v>276</v>
       </c>
       <c r="AB32" s="46" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="AC32" s="34" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="AD32" s="34" t="s">
         <v>277</v>
       </c>
       <c r="AE32" s="60" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="33" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7089,22 +7087,22 @@
         <v>112</v>
       </c>
       <c r="Z33" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA33" s="30" t="s">
         <v>113</v>
       </c>
       <c r="AB33" s="46" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="AC33" s="30" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="AD33" s="30" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="AE33" s="66" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="34" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7118,7 +7116,7 @@
         <v>225</v>
       </c>
       <c r="D34" s="30" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>52</v>
@@ -7179,10 +7177,10 @@
         <v>244</v>
       </c>
       <c r="Y34" s="30" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="Z34" s="30" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="AA34" s="30" t="s">
         <v>292</v>
@@ -7191,13 +7189,13 @@
         <v>293</v>
       </c>
       <c r="AC34" s="30" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="AD34" s="30" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="AE34" s="64" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="35" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7208,10 +7206,10 @@
         <v>142</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>366</v>
+        <v>593</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>54</v>
@@ -7220,7 +7218,7 @@
         <v>143</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="H35" s="35">
         <v>0.28144999999999998</v>
@@ -7277,19 +7275,19 @@
         <v>144</v>
       </c>
       <c r="Z35" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA35" s="34" t="s">
         <v>145</v>
       </c>
       <c r="AB35" s="46" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="AC35" s="34" t="s">
+        <v>372</v>
+      </c>
+      <c r="AD35" s="34" t="s">
         <v>373</v>
-      </c>
-      <c r="AD35" s="34" t="s">
-        <v>374</v>
       </c>
       <c r="AE35" s="62" t="s">
         <v>27</v>
@@ -7303,7 +7301,7 @@
         <v>114</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="D36" s="34" t="s">
         <v>109</v>
@@ -7369,25 +7367,25 @@
         <v>95</v>
       </c>
       <c r="Y36" s="34" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="Z36" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA36" s="34" t="s">
         <v>118</v>
       </c>
       <c r="AB36" s="46" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="AC36" s="34" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="AD36" s="34" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="AE36" s="60" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="37" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7398,10 +7396,10 @@
         <v>281</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>366</v>
+        <v>593</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>45</v>
@@ -7467,22 +7465,22 @@
         <v>284</v>
       </c>
       <c r="Z37" s="34" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="AA37" s="34" t="s">
         <v>285</v>
       </c>
       <c r="AB37" s="46" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="AC37" s="34" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="AD37" s="34" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="AE37" s="60" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="38" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7559,25 +7557,25 @@
         <v>95</v>
       </c>
       <c r="Y38" s="34" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="Z38" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA38" s="34" t="s">
         <v>217</v>
       </c>
       <c r="AB38" s="46" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="AC38" s="34" t="s">
+        <v>403</v>
+      </c>
+      <c r="AD38" s="34" t="s">
         <v>404</v>
       </c>
-      <c r="AD38" s="34" t="s">
-        <v>405</v>
-      </c>
       <c r="AE38" s="61" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="39" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7588,7 +7586,7 @@
         <v>309</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="D39" s="34" t="s">
         <v>109</v>
@@ -7652,25 +7650,25 @@
         <v>180</v>
       </c>
       <c r="Y39" s="30" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="Z39" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA39" s="30" t="s">
         <v>311</v>
       </c>
       <c r="AB39" s="46" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="AC39" s="30" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="AD39" s="30" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="AE39" s="61" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="40" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -7684,7 +7682,7 @@
         <v>219</v>
       </c>
       <c r="D40" s="30" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>50</v>
@@ -7750,7 +7748,7 @@
         <v>221</v>
       </c>
       <c r="Z40" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA40" s="30" t="s">
         <v>222</v>
@@ -7759,13 +7757,13 @@
         <v>223</v>
       </c>
       <c r="AC40" s="30" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="AD40" s="30" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="AE40" s="64" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="41" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -7845,22 +7843,22 @@
         <v>96</v>
       </c>
       <c r="Z41" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA41" s="30" t="s">
         <v>97</v>
       </c>
       <c r="AB41" s="46" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="AC41" s="30" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="AD41" s="30" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="AE41" s="66" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="42" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -7940,22 +7938,22 @@
         <v>136</v>
       </c>
       <c r="Z42" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA42" s="34" t="s">
         <v>134</v>
       </c>
       <c r="AB42" s="46" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="AC42" s="34" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="AD42" s="34" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="AE42" s="60" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="43" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -7963,13 +7961,13 @@
         <v>87</v>
       </c>
       <c r="B43" s="54" t="s">
+        <v>375</v>
+      </c>
+      <c r="C43" s="4" t="s">
         <v>376</v>
       </c>
-      <c r="C43" s="4" t="s">
-        <v>377</v>
-      </c>
       <c r="D43" s="30" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>43</v>
@@ -8035,22 +8033,22 @@
         <v>257</v>
       </c>
       <c r="Z43" s="34" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="AA43" s="34" t="s">
         <v>92</v>
       </c>
       <c r="AB43" s="47" t="s">
+        <v>377</v>
+      </c>
+      <c r="AC43" s="34" t="s">
         <v>378</v>
       </c>
-      <c r="AC43" s="34" t="s">
+      <c r="AD43" s="34" t="s">
         <v>379</v>
       </c>
-      <c r="AD43" s="34" t="s">
-        <v>380</v>
-      </c>
       <c r="AE43" s="60" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="44" spans="1:31" ht="68.400000000000006" x14ac:dyDescent="0.3">
@@ -8127,25 +8125,25 @@
         <v>95</v>
       </c>
       <c r="Y44" s="34" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="Z44" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA44" s="34" t="s">
         <v>129</v>
       </c>
       <c r="AB44" s="46" t="s">
+        <v>499</v>
+      </c>
+      <c r="AC44" s="34" t="s">
+        <v>500</v>
+      </c>
+      <c r="AD44" s="34" t="s">
         <v>501</v>
       </c>
-      <c r="AC44" s="34" t="s">
-        <v>502</v>
-      </c>
-      <c r="AD44" s="34" t="s">
-        <v>503</v>
-      </c>
       <c r="AE44" s="60" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="45" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -8159,13 +8157,13 @@
         <v>357</v>
       </c>
       <c r="D45" s="34" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>46</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="G45" s="4" t="s">
         <v>92</v>
@@ -8222,7 +8220,7 @@
         <v>244</v>
       </c>
       <c r="Y45" s="34" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="Z45" s="34" t="s">
         <v>225</v>
@@ -8231,16 +8229,16 @@
         <v>265</v>
       </c>
       <c r="AB45" s="46" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="AC45" s="34" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="AD45" s="34" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="AE45" s="64" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="46" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8320,22 +8318,22 @@
         <v>214</v>
       </c>
       <c r="Z46" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA46" s="30" t="s">
         <v>215</v>
       </c>
       <c r="AB46" s="46" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="AC46" s="30" t="s">
+        <v>400</v>
+      </c>
+      <c r="AD46" s="30" t="s">
         <v>401</v>
       </c>
-      <c r="AD46" s="30" t="s">
-        <v>402</v>
-      </c>
       <c r="AE46" s="64" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="47" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8355,10 +8353,10 @@
         <v>55</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="H47" s="52">
         <v>1.55E-2</v>
@@ -8415,25 +8413,25 @@
         <v>154</v>
       </c>
       <c r="Z47" s="30" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="AA47" s="30" t="s">
         <v>155</v>
       </c>
       <c r="AB47" s="46" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="AC47" s="30" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="AD47" s="30" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="AE47" s="65" t="s">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="48" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="48" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
         <v>87</v>
       </c>
@@ -8453,7 +8451,7 @@
         <v>344</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="H48" s="35">
         <v>0.40600000000000003</v>
@@ -8510,7 +8508,7 @@
         <v>350</v>
       </c>
       <c r="Z48" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA48" s="34" t="s">
         <v>308</v>
@@ -8519,13 +8517,13 @@
         <v>347</v>
       </c>
       <c r="AC48" s="34" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="AD48" s="34" t="s">
         <v>346</v>
       </c>
       <c r="AE48" s="61" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="49" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -8545,10 +8543,10 @@
         <v>54</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="H49" s="53">
         <v>6.7077999999999999E-2</v>
@@ -8605,22 +8603,22 @@
         <v>151</v>
       </c>
       <c r="Z49" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA49" s="34" t="s">
         <v>152</v>
       </c>
       <c r="AB49" s="46" t="s">
+        <v>515</v>
+      </c>
+      <c r="AC49" s="34" t="s">
+        <v>516</v>
+      </c>
+      <c r="AD49" s="34" t="s">
         <v>517</v>
       </c>
-      <c r="AC49" s="34" t="s">
-        <v>518</v>
-      </c>
-      <c r="AD49" s="34" t="s">
-        <v>519</v>
-      </c>
       <c r="AE49" s="64" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="50" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -8634,7 +8632,7 @@
         <v>225</v>
       </c>
       <c r="D50" s="34" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>48</v>
@@ -8685,7 +8683,7 @@
         <v>132</v>
       </c>
       <c r="Y50" s="34" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="Z50" s="34" t="s">
         <v>225</v>
@@ -8694,16 +8692,16 @@
         <v>211</v>
       </c>
       <c r="AB50" s="46" t="s">
+        <v>519</v>
+      </c>
+      <c r="AC50" s="34" t="s">
+        <v>520</v>
+      </c>
+      <c r="AD50" s="34" t="s">
         <v>521</v>
       </c>
-      <c r="AC50" s="34" t="s">
-        <v>522</v>
-      </c>
-      <c r="AD50" s="34" t="s">
-        <v>523</v>
-      </c>
       <c r="AE50" s="65" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="51" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -8723,10 +8721,10 @@
         <v>42</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="G51" s="30" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="H51" s="31">
         <v>0.27411429999999998</v>
@@ -8780,25 +8778,25 @@
         <v>132</v>
       </c>
       <c r="Y51" s="30" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="Z51" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA51" s="30" t="s">
         <v>184</v>
       </c>
       <c r="AB51" s="46" t="s">
+        <v>523</v>
+      </c>
+      <c r="AC51" s="30" t="s">
+        <v>524</v>
+      </c>
+      <c r="AD51" s="30" t="s">
         <v>525</v>
       </c>
-      <c r="AC51" s="30" t="s">
-        <v>526</v>
-      </c>
-      <c r="AD51" s="30" t="s">
-        <v>527</v>
-      </c>
       <c r="AE51" s="65" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="52" spans="1:31" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -8878,7 +8876,7 @@
         <v>158</v>
       </c>
       <c r="Z52" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA52" s="34" t="s">
         <v>159</v>
@@ -8893,7 +8891,7 @@
         <v>162</v>
       </c>
       <c r="AE52" s="66" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="53" spans="1:31" ht="114" x14ac:dyDescent="0.3">
@@ -8904,7 +8902,7 @@
         <v>234</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="D53" s="30" t="s">
         <v>109</v>
@@ -8916,7 +8914,7 @@
         <v>235</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="H53" s="31">
         <v>1.72E-2</v>
@@ -8970,22 +8968,22 @@
         <v>95</v>
       </c>
       <c r="Y53" s="30" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="Z53" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA53" s="30" t="s">
         <v>236</v>
       </c>
       <c r="AB53" s="46" t="s">
+        <v>530</v>
+      </c>
+      <c r="AC53" s="30" t="s">
         <v>532</v>
       </c>
-      <c r="AC53" s="30" t="s">
-        <v>534</v>
-      </c>
       <c r="AD53" s="30" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="AE53" s="67" t="s">
         <v>29</v>
@@ -8999,19 +8997,19 @@
         <v>272</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="D54" s="30" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>46</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="G54" s="30" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="H54" s="31">
         <v>0.16981750000000001</v>
@@ -9065,25 +9063,25 @@
         <v>132</v>
       </c>
       <c r="Y54" s="30" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="Z54" s="30" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA54" s="30" t="s">
         <v>273</v>
       </c>
       <c r="AB54" s="46" t="s">
+        <v>536</v>
+      </c>
+      <c r="AC54" s="30" t="s">
+        <v>537</v>
+      </c>
+      <c r="AD54" s="30" t="s">
         <v>538</v>
       </c>
-      <c r="AC54" s="30" t="s">
-        <v>539</v>
-      </c>
-      <c r="AD54" s="30" t="s">
-        <v>540</v>
-      </c>
       <c r="AE54" s="65" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="55" spans="1:31" ht="125.4" x14ac:dyDescent="0.3">
@@ -9094,19 +9092,19 @@
         <v>262</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D55" s="30" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>46</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="H55" s="31">
         <v>4.2</v>
@@ -9160,23 +9158,23 @@
         <v>132</v>
       </c>
       <c r="Y55" s="30" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="Z55" s="30" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="AA55" s="30"/>
       <c r="AB55" s="46" t="s">
         <v>263</v>
       </c>
       <c r="AC55" s="30" t="s">
+        <v>384</v>
+      </c>
+      <c r="AD55" s="30" t="s">
         <v>385</v>
       </c>
-      <c r="AD55" s="30" t="s">
-        <v>386</v>
-      </c>
       <c r="AE55" s="60" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="56" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -9196,10 +9194,10 @@
         <v>42</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="H56" s="31">
         <v>0.17</v>
@@ -9253,25 +9251,25 @@
         <v>95</v>
       </c>
       <c r="Y56" s="30" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="Z56" s="30" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="AA56" s="30" t="s">
         <v>191</v>
       </c>
       <c r="AB56" s="46" t="s">
+        <v>545</v>
+      </c>
+      <c r="AC56" s="30" t="s">
+        <v>546</v>
+      </c>
+      <c r="AD56" s="30" t="s">
         <v>547</v>
       </c>
-      <c r="AC56" s="30" t="s">
-        <v>548</v>
-      </c>
-      <c r="AD56" s="30" t="s">
-        <v>549</v>
-      </c>
       <c r="AE56" s="64" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="57" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -9282,19 +9280,19 @@
         <v>299</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D57" s="30" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>52</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="H57" s="31">
         <v>2</v>
@@ -9348,10 +9346,10 @@
         <v>132</v>
       </c>
       <c r="Y57" s="30" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="Z57" s="30" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="AA57" s="30" t="s">
         <v>300</v>
@@ -9360,13 +9358,13 @@
         <v>301</v>
       </c>
       <c r="AC57" s="30" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="AD57" s="30" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="AE57" s="60" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="58" spans="1:31" ht="102.6" x14ac:dyDescent="0.3">
@@ -9380,7 +9378,7 @@
         <v>225</v>
       </c>
       <c r="D58" s="34" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>50</v>
@@ -9443,7 +9441,7 @@
         <v>132</v>
       </c>
       <c r="Y58" s="30" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="Z58" s="30" t="s">
         <v>225</v>
@@ -9452,16 +9450,16 @@
         <v>230</v>
       </c>
       <c r="AB58" s="46" t="s">
+        <v>559</v>
+      </c>
+      <c r="AC58" s="30" t="s">
+        <v>560</v>
+      </c>
+      <c r="AD58" s="30" t="s">
         <v>561</v>
       </c>
-      <c r="AC58" s="30" t="s">
-        <v>562</v>
-      </c>
-      <c r="AD58" s="30" t="s">
+      <c r="AE58" s="60" t="s">
         <v>563</v>
-      </c>
-      <c r="AE58" s="60" t="s">
-        <v>565</v>
       </c>
     </row>
     <row r="59" spans="1:31" ht="68.400000000000006" x14ac:dyDescent="0.3">
@@ -9538,10 +9536,10 @@
         <v>244</v>
       </c>
       <c r="Y59" s="34" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="Z59" s="34" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="AA59" s="34" t="s">
         <v>296</v>
@@ -9550,13 +9548,13 @@
         <v>297</v>
       </c>
       <c r="AC59" s="34" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="AD59" s="34" t="s">
         <v>298</v>
       </c>
       <c r="AE59" s="61" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="60" spans="1:31" ht="79.8" x14ac:dyDescent="0.3">
@@ -9636,22 +9634,22 @@
         <v>187</v>
       </c>
       <c r="Z60" s="34" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="AA60" s="34" t="s">
         <v>188</v>
       </c>
       <c r="AB60" s="46" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="AC60" s="34" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="AD60" s="34" t="s">
         <v>189</v>
       </c>
       <c r="AE60" s="60" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="61" spans="1:31" ht="91.2" x14ac:dyDescent="0.3">
@@ -9665,7 +9663,7 @@
         <v>242</v>
       </c>
       <c r="D61" s="34" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="E61" s="4" t="s">
         <v>46</v>
@@ -9728,7 +9726,7 @@
         <v>244</v>
       </c>
       <c r="Y61" s="34" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="Z61" s="34" t="s">
         <v>225</v>
@@ -9737,16 +9735,16 @@
         <v>270</v>
       </c>
       <c r="AB61" s="46" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="AC61" s="34" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="AD61" s="34" t="s">
         <v>271</v>
       </c>
       <c r="AE61" s="65" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
   </sheetData>
@@ -9834,141 +9832,141 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="87" t="s">
         <v>314</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="78" t="s">
+      <c r="A3" s="73" t="s">
         <v>315</v>
       </c>
-      <c r="B3" s="76"/>
-      <c r="C3" s="76"/>
-      <c r="D3" s="76"/>
-      <c r="E3" s="76"/>
+      <c r="B3" s="74"/>
+      <c r="C3" s="74"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
     </row>
     <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="90" t="s">
+      <c r="A4" s="93" t="s">
         <v>316</v>
       </c>
-      <c r="B4" s="75"/>
-      <c r="C4" s="83" t="s">
+      <c r="B4" s="77"/>
+      <c r="C4" s="82" t="s">
         <v>317</v>
       </c>
-      <c r="D4" s="76"/>
-      <c r="E4" s="76"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="74"/>
     </row>
     <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="87" t="s">
+      <c r="A5" s="90" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="83" t="s">
+      <c r="B5" s="77"/>
+      <c r="C5" s="82" t="s">
         <v>318</v>
       </c>
-      <c r="D5" s="76"/>
-      <c r="E5" s="76"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="74"/>
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="85" t="s">
+      <c r="A6" s="88" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="75"/>
-      <c r="C6" s="83" t="s">
+      <c r="B6" s="77"/>
+      <c r="C6" s="82" t="s">
         <v>319</v>
       </c>
-      <c r="D6" s="76"/>
-      <c r="E6" s="76"/>
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="86" t="s">
+      <c r="A7" s="89" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="75"/>
-      <c r="C7" s="83" t="s">
+      <c r="B7" s="77"/>
+      <c r="C7" s="82" t="s">
         <v>320</v>
       </c>
-      <c r="D7" s="76"/>
-      <c r="E7" s="76"/>
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="89" t="s">
+      <c r="A8" s="92" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="83" t="s">
+      <c r="B8" s="77"/>
+      <c r="C8" s="82" t="s">
         <v>321</v>
       </c>
-      <c r="D8" s="76"/>
-      <c r="E8" s="76"/>
+      <c r="D8" s="74"/>
+      <c r="E8" s="74"/>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="93" t="s">
+      <c r="A9" s="85" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="75"/>
-      <c r="C9" s="83" t="s">
+      <c r="B9" s="77"/>
+      <c r="C9" s="82" t="s">
         <v>322</v>
       </c>
-      <c r="D9" s="76"/>
-      <c r="E9" s="76"/>
+      <c r="D9" s="74"/>
+      <c r="E9" s="74"/>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="91" t="s">
+      <c r="A10" s="83" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="75"/>
-      <c r="C10" s="83" t="s">
+      <c r="B10" s="77"/>
+      <c r="C10" s="82" t="s">
         <v>323</v>
       </c>
-      <c r="D10" s="76"/>
-      <c r="E10" s="76"/>
+      <c r="D10" s="74"/>
+      <c r="E10" s="74"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="78" t="s">
+      <c r="A12" s="73" t="s">
         <v>324</v>
       </c>
-      <c r="B12" s="76"/>
-      <c r="C12" s="76"/>
-      <c r="D12" s="76"/>
-      <c r="E12" s="76"/>
+      <c r="B12" s="74"/>
+      <c r="C12" s="74"/>
+      <c r="D12" s="74"/>
+      <c r="E12" s="74"/>
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="92" t="s">
+      <c r="A13" s="84" t="s">
         <v>325</v>
       </c>
-      <c r="B13" s="75"/>
-      <c r="C13" s="83" t="s">
+      <c r="B13" s="77"/>
+      <c r="C13" s="82" t="s">
         <v>326</v>
       </c>
-      <c r="D13" s="76"/>
-      <c r="E13" s="76"/>
+      <c r="D13" s="74"/>
+      <c r="E13" s="74"/>
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="88" t="s">
+      <c r="A14" s="91" t="s">
         <v>327</v>
       </c>
-      <c r="B14" s="75"/>
-      <c r="C14" s="83" t="s">
+      <c r="B14" s="77"/>
+      <c r="C14" s="82" t="s">
         <v>328</v>
       </c>
-      <c r="D14" s="76"/>
-      <c r="E14" s="76"/>
+      <c r="D14" s="74"/>
+      <c r="E14" s="74"/>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="82" t="s">
+      <c r="A15" s="86" t="s">
         <v>329</v>
       </c>
-      <c r="B15" s="75"/>
-      <c r="C15" s="83" t="s">
+      <c r="B15" s="77"/>
+      <c r="C15" s="82" t="s">
         <v>330</v>
       </c>
-      <c r="D15" s="76"/>
-      <c r="E15" s="76"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="74"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="43" t="s">
@@ -9983,13 +9981,6 @@
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C10:E10"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="A1:E1"/>
@@ -10006,6 +9997,13 @@
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C6:E6"/>
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C10:E10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -10013,12 +10011,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10263,20 +10263,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CBE187-A7DE-4A9A-99BE-7485C92477B0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10301,18 +10308,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CBE187-A7DE-4A9A-99BE-7485C92477B0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>